<commit_message>
Normalize quote template PDF borders
</commit_message>
<xml_diff>
--- a/Codex Plugins/plugins/dhandy-excel-quote-template/skills/artifact-template-dhandy/assets/reference.xlsx
+++ b/Codex Plugins/plugins/dhandy-excel-quote-template/skills/artifact-template-dhandy/assets/reference.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kookie\Documents\견적 업무\tmp\quote_template_line_fix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0A2EE12-CED3-49EC-A967-286CB0ADBC68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74270C47-C043-4004-8539-44C4DB423C82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. 견적서" sheetId="2" r:id="rId1"/>
@@ -506,7 +506,7 @@
     <numFmt numFmtId="179" formatCode="#,##0&quot;원&quot;"/>
     <numFmt numFmtId="180" formatCode="&quot;₩ &quot;#,##0;[Red]\-&quot;₩ &quot;#,##0"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -675,6 +675,14 @@
       <name val="Pretendard"/>
       <charset val="129"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Pretendard"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
   </fonts>
   <fills count="22">
     <fill>
@@ -785,7 +793,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="33">
+  <borders count="35">
     <border>
       <left/>
       <right/>
@@ -1117,13 +1125,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFF04A17"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="204">
+  <cellXfs count="217">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1186,18 +1216,6 @@
     </xf>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="16" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="16" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="16" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
@@ -1266,18 +1284,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="38" fontId="16" fillId="12" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="14" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="14" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="14" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="10" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1382,14 +1388,89 @@
     <xf numFmtId="0" fontId="9" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="21" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="13" fillId="17" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="15" fillId="11" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1409,104 +1490,53 @@
     <xf numFmtId="0" fontId="4" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="15" fillId="11" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="16" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1514,22 +1544,7 @@
     <xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="16" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="16" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="16" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1538,8 +1553,11 @@
     <xf numFmtId="0" fontId="4" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1586,59 +1604,23 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="12" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="4" fillId="16" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="16" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
@@ -1685,55 +1667,142 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="2" fontId="21" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="23" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="4" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="38" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="21" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="38" fontId="20" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="33" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="38" fontId="23" fillId="21" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="38" fontId="23" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="21" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="16" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="38" fontId="16" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="38" fontId="16" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="2" fontId="14" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="13" fillId="17" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="38" fontId="14" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="38" fontId="14" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -14712,528 +14781,6 @@
           <a:endParaRPr/>
         </a:p>
       </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="182" name="COVER_RULE_25">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000B6000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr>
-          <a:spLocks noGrp="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="390525" y="5257800"/>
-          <a:ext cx="8934450" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="line">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="6350">
-          <a:solidFill>
-            <a:srgbClr val="D9D9D9"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="183" name="COVER_RULE_26">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000B7000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr>
-          <a:spLocks noGrp="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="390525" y="5505450"/>
-          <a:ext cx="8934450" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="line">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="6350">
-          <a:solidFill>
-            <a:srgbClr val="D9D9D9"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="184" name="COVER_RULE_27">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000B8000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr>
-          <a:spLocks noGrp="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="390525" y="5753100"/>
-          <a:ext cx="8934450" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="line">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="6350">
-          <a:solidFill>
-            <a:srgbClr val="D9D9D9"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="185" name="COVER_RULE_28">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000B9000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr>
-          <a:spLocks noGrp="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="390525" y="6000750"/>
-          <a:ext cx="8934450" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="line">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="6350">
-          <a:solidFill>
-            <a:srgbClr val="D9D9D9"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="186" name="COVER_RULE_29">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000BA000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr>
-          <a:spLocks noGrp="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="390525" y="6248400"/>
-          <a:ext cx="8934450" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="line">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="6350">
-          <a:solidFill>
-            <a:srgbClr val="D9D9D9"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="187" name="COVER_RULE_30">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000BB000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr>
-          <a:spLocks noGrp="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="390525" y="6496050"/>
-          <a:ext cx="8934450" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="line">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="6350">
-          <a:solidFill>
-            <a:srgbClr val="D9D9D9"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="188" name="COVER_RULE_31">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000BC000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr>
-          <a:spLocks noGrp="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="390525" y="6743700"/>
-          <a:ext cx="8934450" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="line">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="6350">
-          <a:solidFill>
-            <a:srgbClr val="D9D9D9"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="189" name="COVER_RULE_32">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000BD000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr>
-          <a:spLocks noGrp="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="390525" y="6991350"/>
-          <a:ext cx="8934450" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="line">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="6350">
-          <a:solidFill>
-            <a:srgbClr val="D9D9D9"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="190" name="COVER_RULE_33">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000BE000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr>
-          <a:spLocks noGrp="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="390525" y="7239000"/>
-          <a:ext cx="8934450" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="line">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="6350">
-          <a:solidFill>
-            <a:srgbClr val="D9D9D9"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
@@ -28359,19 +27906,19 @@
       <c r="L3" s="3"/>
     </row>
     <row r="4" spans="1:13" ht="8.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="79"/>
-      <c r="B4" s="79"/>
-      <c r="C4" s="79"/>
-      <c r="D4" s="79"/>
-      <c r="E4" s="79"/>
-      <c r="F4" s="79"/>
-      <c r="G4" s="79"/>
-      <c r="H4" s="79"/>
-      <c r="I4" s="79"/>
-      <c r="J4" s="79"/>
-      <c r="K4" s="79"/>
-      <c r="L4" s="79"/>
-      <c r="M4" s="78"/>
+      <c r="A4" s="71"/>
+      <c r="B4" s="71"/>
+      <c r="C4" s="71"/>
+      <c r="D4" s="71"/>
+      <c r="E4" s="71"/>
+      <c r="F4" s="71"/>
+      <c r="G4" s="71"/>
+      <c r="H4" s="71"/>
+      <c r="I4" s="71"/>
+      <c r="J4" s="71"/>
+      <c r="K4" s="71"/>
+      <c r="L4" s="71"/>
+      <c r="M4" s="70"/>
     </row>
     <row r="5" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3"/>
@@ -28381,12 +27928,12 @@
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
-      <c r="H5" s="99" t="s">
+      <c r="H5" s="100" t="s">
         <v>0</v>
       </c>
-      <c r="I5" s="99"/>
-      <c r="J5" s="99"/>
-      <c r="K5" s="99"/>
+      <c r="I5" s="100"/>
+      <c r="J5" s="100"/>
+      <c r="K5" s="100"/>
       <c r="L5" s="3"/>
     </row>
     <row r="6" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.3">
@@ -28397,12 +27944,12 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
-      <c r="H6" s="100" t="s">
+      <c r="H6" s="101" t="s">
         <v>1</v>
       </c>
-      <c r="I6" s="100"/>
-      <c r="J6" s="100"/>
-      <c r="K6" s="100"/>
+      <c r="I6" s="101"/>
+      <c r="J6" s="101"/>
+      <c r="K6" s="101"/>
       <c r="L6" s="3"/>
     </row>
     <row r="7" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.3">
@@ -28413,12 +27960,12 @@
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
-      <c r="H7" s="101" t="s">
+      <c r="H7" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="I7" s="101"/>
-      <c r="J7" s="101"/>
-      <c r="K7" s="101"/>
+      <c r="I7" s="102"/>
+      <c r="J7" s="102"/>
+      <c r="K7" s="102"/>
       <c r="L7" s="3"/>
     </row>
     <row r="8" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -28437,79 +27984,79 @@
     </row>
     <row r="9" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
-      <c r="B9" s="103" t="s">
+      <c r="B9" s="104" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="103"/>
-      <c r="D9" s="103"/>
-      <c r="E9" s="103"/>
-      <c r="F9" s="103"/>
-      <c r="G9" s="103"/>
-      <c r="H9" s="103"/>
-      <c r="I9" s="103"/>
-      <c r="J9" s="103"/>
-      <c r="K9" s="103"/>
-      <c r="L9" s="103"/>
+      <c r="C9" s="104"/>
+      <c r="D9" s="104"/>
+      <c r="E9" s="104"/>
+      <c r="F9" s="104"/>
+      <c r="G9" s="104"/>
+      <c r="H9" s="104"/>
+      <c r="I9" s="104"/>
+      <c r="J9" s="104"/>
+      <c r="K9" s="104"/>
+      <c r="L9" s="104"/>
     </row>
     <row r="10" spans="1:13" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
-      <c r="B10" s="103"/>
-      <c r="C10" s="103"/>
-      <c r="D10" s="103"/>
-      <c r="E10" s="103"/>
-      <c r="F10" s="103"/>
-      <c r="G10" s="103"/>
-      <c r="H10" s="103"/>
-      <c r="I10" s="103"/>
-      <c r="J10" s="103"/>
-      <c r="K10" s="103"/>
-      <c r="L10" s="103"/>
+      <c r="B10" s="104"/>
+      <c r="C10" s="104"/>
+      <c r="D10" s="104"/>
+      <c r="E10" s="104"/>
+      <c r="F10" s="104"/>
+      <c r="G10" s="104"/>
+      <c r="H10" s="104"/>
+      <c r="I10" s="104"/>
+      <c r="J10" s="104"/>
+      <c r="K10" s="104"/>
+      <c r="L10" s="104"/>
     </row>
     <row r="11" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
-      <c r="B11" s="104" t="s">
+      <c r="B11" s="105" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="104"/>
-      <c r="D11" s="104"/>
-      <c r="E11" s="104"/>
-      <c r="F11" s="104"/>
-      <c r="G11" s="104"/>
-      <c r="H11" s="104"/>
-      <c r="I11" s="104"/>
-      <c r="J11" s="104"/>
-      <c r="K11" s="104"/>
-      <c r="L11" s="104"/>
+      <c r="C11" s="105"/>
+      <c r="D11" s="105"/>
+      <c r="E11" s="105"/>
+      <c r="F11" s="105"/>
+      <c r="G11" s="105"/>
+      <c r="H11" s="105"/>
+      <c r="I11" s="105"/>
+      <c r="J11" s="105"/>
+      <c r="K11" s="105"/>
+      <c r="L11" s="105"/>
     </row>
     <row r="12" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3"/>
-      <c r="B12" s="102" t="s">
+      <c r="B12" s="103" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="102"/>
-      <c r="D12" s="102"/>
-      <c r="E12" s="102"/>
-      <c r="F12" s="102"/>
-      <c r="G12" s="102"/>
-      <c r="H12" s="102"/>
-      <c r="I12" s="102"/>
-      <c r="J12" s="102"/>
-      <c r="K12" s="102"/>
-      <c r="L12" s="102"/>
+      <c r="C12" s="103"/>
+      <c r="D12" s="103"/>
+      <c r="E12" s="103"/>
+      <c r="F12" s="103"/>
+      <c r="G12" s="103"/>
+      <c r="H12" s="103"/>
+      <c r="I12" s="103"/>
+      <c r="J12" s="103"/>
+      <c r="K12" s="103"/>
+      <c r="L12" s="103"/>
     </row>
     <row r="13" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3"/>
-      <c r="B13" s="102"/>
-      <c r="C13" s="102"/>
-      <c r="D13" s="102"/>
-      <c r="E13" s="102"/>
-      <c r="F13" s="102"/>
-      <c r="G13" s="102"/>
-      <c r="H13" s="102"/>
-      <c r="I13" s="102"/>
-      <c r="J13" s="102"/>
-      <c r="K13" s="102"/>
-      <c r="L13" s="102"/>
+      <c r="B13" s="103"/>
+      <c r="C13" s="103"/>
+      <c r="D13" s="103"/>
+      <c r="E13" s="103"/>
+      <c r="F13" s="103"/>
+      <c r="G13" s="103"/>
+      <c r="H13" s="103"/>
+      <c r="I13" s="103"/>
+      <c r="J13" s="103"/>
+      <c r="K13" s="103"/>
+      <c r="L13" s="103"/>
     </row>
     <row r="14" spans="1:13" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3"/>
@@ -28526,654 +28073,706 @@
       <c r="L14" s="3"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A15" s="40"/>
-      <c r="B15" s="105" t="s">
+      <c r="A15" s="36"/>
+      <c r="B15" s="95" t="s">
         <v>6</v>
       </c>
-      <c r="C15" s="105"/>
-      <c r="D15" s="105"/>
-      <c r="E15" s="105"/>
-      <c r="F15" s="105"/>
-      <c r="G15" s="105" t="s">
+      <c r="C15" s="95"/>
+      <c r="D15" s="95"/>
+      <c r="E15" s="95"/>
+      <c r="F15" s="95"/>
+      <c r="G15" s="95" t="s">
         <v>7</v>
       </c>
-      <c r="H15" s="105"/>
-      <c r="I15" s="105"/>
-      <c r="J15" s="105"/>
-      <c r="K15" s="105"/>
-      <c r="L15" s="105"/>
+      <c r="H15" s="95"/>
+      <c r="I15" s="95"/>
+      <c r="J15" s="95"/>
+      <c r="K15" s="95"/>
+      <c r="L15" s="95"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A16" s="40"/>
-      <c r="B16" s="108" t="s">
+      <c r="A16" s="36"/>
+      <c r="B16" s="98" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="108"/>
-      <c r="D16" s="108"/>
-      <c r="E16" s="108"/>
-      <c r="F16" s="108"/>
-      <c r="G16" s="108" t="s">
+      <c r="C16" s="98"/>
+      <c r="D16" s="98"/>
+      <c r="E16" s="98"/>
+      <c r="F16" s="98"/>
+      <c r="G16" s="98" t="s">
         <v>9</v>
       </c>
-      <c r="H16" s="108"/>
-      <c r="I16" s="108"/>
-      <c r="J16" s="108"/>
-      <c r="K16" s="108"/>
-      <c r="L16" s="108"/>
+      <c r="H16" s="98"/>
+      <c r="I16" s="98"/>
+      <c r="J16" s="98"/>
+      <c r="K16" s="98"/>
+      <c r="L16" s="98"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A17" s="40"/>
-      <c r="B17" s="109"/>
-      <c r="C17" s="109"/>
-      <c r="D17" s="109"/>
-      <c r="E17" s="109"/>
-      <c r="F17" s="109"/>
-      <c r="G17" s="109"/>
-      <c r="H17" s="109"/>
-      <c r="I17" s="109"/>
-      <c r="J17" s="109"/>
-      <c r="K17" s="109"/>
-      <c r="L17" s="109"/>
+      <c r="A17" s="36"/>
+      <c r="B17" s="99"/>
+      <c r="C17" s="99"/>
+      <c r="D17" s="99"/>
+      <c r="E17" s="99"/>
+      <c r="F17" s="99"/>
+      <c r="G17" s="99"/>
+      <c r="H17" s="99"/>
+      <c r="I17" s="99"/>
+      <c r="J17" s="99"/>
+      <c r="K17" s="99"/>
+      <c r="L17" s="99"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A18" s="40"/>
-      <c r="B18" s="41"/>
-      <c r="C18" s="41"/>
-      <c r="D18" s="41"/>
-      <c r="E18" s="41"/>
-      <c r="F18" s="41"/>
-      <c r="G18" s="41"/>
-      <c r="H18" s="41"/>
-      <c r="I18" s="41"/>
-      <c r="J18" s="41"/>
-      <c r="K18" s="41"/>
-      <c r="L18" s="41"/>
+      <c r="A18" s="36"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="37"/>
+      <c r="G18" s="37"/>
+      <c r="H18" s="37"/>
+      <c r="I18" s="37"/>
+      <c r="J18" s="37"/>
+      <c r="K18" s="37"/>
+      <c r="L18" s="37"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A19" s="40"/>
-      <c r="B19" s="105" t="s">
+      <c r="A19" s="36"/>
+      <c r="B19" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="105"/>
-      <c r="D19" s="105"/>
-      <c r="E19" s="105"/>
-      <c r="F19" s="105"/>
-      <c r="G19" s="105" t="s">
+      <c r="C19" s="95"/>
+      <c r="D19" s="95"/>
+      <c r="E19" s="95"/>
+      <c r="F19" s="95"/>
+      <c r="G19" s="95" t="s">
         <v>11</v>
       </c>
-      <c r="H19" s="105"/>
-      <c r="I19" s="105"/>
-      <c r="J19" s="105"/>
-      <c r="K19" s="105"/>
-      <c r="L19" s="105"/>
+      <c r="H19" s="95"/>
+      <c r="I19" s="95"/>
+      <c r="J19" s="95"/>
+      <c r="K19" s="95"/>
+      <c r="L19" s="95"/>
     </row>
     <row r="20" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="40"/>
-      <c r="B20" s="106" t="s">
+      <c r="A20" s="36"/>
+      <c r="B20" s="96" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="106"/>
-      <c r="D20" s="106"/>
-      <c r="E20" s="106"/>
-      <c r="F20" s="106"/>
-      <c r="G20" s="42" t="s">
+      <c r="C20" s="96"/>
+      <c r="D20" s="96"/>
+      <c r="E20" s="96"/>
+      <c r="F20" s="96"/>
+      <c r="G20" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="H20" s="106" t="s">
+      <c r="H20" s="96" t="s">
         <v>14</v>
       </c>
-      <c r="I20" s="106"/>
-      <c r="J20" s="106"/>
-      <c r="K20" s="106"/>
-      <c r="L20" s="106"/>
+      <c r="I20" s="96"/>
+      <c r="J20" s="96"/>
+      <c r="K20" s="96"/>
+      <c r="L20" s="96"/>
     </row>
     <row r="21" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="40"/>
-      <c r="B21" s="106"/>
-      <c r="C21" s="106"/>
-      <c r="D21" s="106"/>
-      <c r="E21" s="106"/>
-      <c r="F21" s="106"/>
-      <c r="G21" s="42" t="s">
+      <c r="A21" s="36"/>
+      <c r="B21" s="96"/>
+      <c r="C21" s="96"/>
+      <c r="D21" s="96"/>
+      <c r="E21" s="96"/>
+      <c r="F21" s="96"/>
+      <c r="G21" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="H21" s="106" t="s">
+      <c r="H21" s="96" t="s">
         <v>16</v>
       </c>
-      <c r="I21" s="106"/>
-      <c r="J21" s="106"/>
-      <c r="K21" s="106"/>
-      <c r="L21" s="106"/>
+      <c r="I21" s="96"/>
+      <c r="J21" s="96"/>
+      <c r="K21" s="96"/>
+      <c r="L21" s="96"/>
     </row>
     <row r="22" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="40"/>
-      <c r="B22" s="107"/>
-      <c r="C22" s="107"/>
-      <c r="D22" s="107"/>
-      <c r="E22" s="107"/>
-      <c r="F22" s="107"/>
-      <c r="G22" s="43" t="s">
+      <c r="A22" s="36"/>
+      <c r="B22" s="97"/>
+      <c r="C22" s="97"/>
+      <c r="D22" s="97"/>
+      <c r="E22" s="97"/>
+      <c r="F22" s="97"/>
+      <c r="G22" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="H22" s="107" t="s">
+      <c r="H22" s="97" t="s">
         <v>18</v>
       </c>
-      <c r="I22" s="107"/>
-      <c r="J22" s="107"/>
-      <c r="K22" s="107"/>
-      <c r="L22" s="107"/>
+      <c r="I22" s="97"/>
+      <c r="J22" s="97"/>
+      <c r="K22" s="97"/>
+      <c r="L22" s="97"/>
     </row>
     <row r="23" spans="1:12" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="116" t="s">
+      <c r="B23" s="93" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="116"/>
-      <c r="D23" s="116"/>
-      <c r="E23" s="116"/>
-      <c r="F23" s="116"/>
-      <c r="G23" s="116"/>
-      <c r="H23" s="116"/>
-      <c r="I23" s="117" t="s">
+      <c r="C23" s="93"/>
+      <c r="D23" s="93"/>
+      <c r="E23" s="93"/>
+      <c r="F23" s="93"/>
+      <c r="G23" s="93"/>
+      <c r="H23" s="93"/>
+      <c r="I23" s="94" t="s">
         <v>20</v>
       </c>
-      <c r="J23" s="117"/>
-      <c r="K23" s="117"/>
-      <c r="L23" s="117"/>
+      <c r="J23" s="94"/>
+      <c r="K23" s="94"/>
+      <c r="L23" s="94"/>
     </row>
     <row r="24" spans="1:12" ht="23.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="86" t="s">
+      <c r="B24" s="204" t="s">
         <v>21</v>
       </c>
-      <c r="C24" s="86"/>
-      <c r="D24" s="118" t="s">
+      <c r="C24" s="204"/>
+      <c r="D24" s="205" t="s">
         <v>22</v>
       </c>
-      <c r="E24" s="119"/>
-      <c r="F24" s="119"/>
-      <c r="G24" s="118" t="s">
+      <c r="E24" s="206"/>
+      <c r="F24" s="206"/>
+      <c r="G24" s="205" t="s">
         <v>23</v>
       </c>
-      <c r="H24" s="119"/>
-      <c r="I24" s="119"/>
-      <c r="J24" s="118" t="s">
+      <c r="H24" s="206"/>
+      <c r="I24" s="206"/>
+      <c r="J24" s="205" t="s">
         <v>24</v>
       </c>
-      <c r="K24" s="119"/>
-      <c r="L24" s="119"/>
+      <c r="K24" s="206"/>
+      <c r="L24" s="206"/>
     </row>
     <row r="25" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="87">
+      <c r="B25" s="172">
         <v>10</v>
       </c>
-      <c r="C25" s="88"/>
-      <c r="D25" s="110" t="s">
+      <c r="C25" s="173"/>
+      <c r="D25" s="174" t="s">
         <v>25</v>
       </c>
-      <c r="E25" s="111"/>
-      <c r="F25" s="111"/>
-      <c r="G25" s="112" t="s">
+      <c r="E25" s="175"/>
+      <c r="F25" s="175"/>
+      <c r="G25" s="176" t="s">
         <v>26</v>
       </c>
-      <c r="H25" s="113"/>
-      <c r="I25" s="113"/>
-      <c r="J25" s="114">
+      <c r="H25" s="177"/>
+      <c r="I25" s="177"/>
+      <c r="J25" s="178">
         <f>'2. 상세견적'!J11</f>
         <v>40000000</v>
       </c>
-      <c r="K25" s="115"/>
-      <c r="L25" s="115"/>
+      <c r="K25" s="179"/>
+      <c r="L25" s="179"/>
     </row>
     <row r="26" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="87">
+      <c r="B26" s="180">
         <v>20</v>
       </c>
-      <c r="C26" s="88"/>
-      <c r="D26" s="110" t="s">
+      <c r="C26" s="181"/>
+      <c r="D26" s="182" t="s">
         <v>27</v>
       </c>
-      <c r="E26" s="111"/>
-      <c r="F26" s="111"/>
-      <c r="G26" s="112" t="s">
+      <c r="E26" s="183"/>
+      <c r="F26" s="183"/>
+      <c r="G26" s="184" t="s">
         <v>28</v>
       </c>
-      <c r="H26" s="113"/>
-      <c r="I26" s="113"/>
-      <c r="J26" s="114">
+      <c r="H26" s="185"/>
+      <c r="I26" s="185"/>
+      <c r="J26" s="186">
         <f>'2. 상세견적'!J18</f>
         <v>10250000</v>
       </c>
-      <c r="K26" s="115"/>
-      <c r="L26" s="115"/>
+      <c r="K26" s="187"/>
+      <c r="L26" s="187"/>
     </row>
     <row r="27" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="87">
+      <c r="B27" s="180">
         <v>30</v>
       </c>
-      <c r="C27" s="88"/>
-      <c r="D27" s="110" t="s">
+      <c r="C27" s="181"/>
+      <c r="D27" s="182" t="s">
         <v>29</v>
       </c>
-      <c r="E27" s="111"/>
-      <c r="F27" s="111"/>
-      <c r="G27" s="112" t="s">
+      <c r="E27" s="183"/>
+      <c r="F27" s="183"/>
+      <c r="G27" s="184" t="s">
         <v>30</v>
       </c>
-      <c r="H27" s="113"/>
-      <c r="I27" s="113"/>
-      <c r="J27" s="114">
+      <c r="H27" s="185"/>
+      <c r="I27" s="185"/>
+      <c r="J27" s="186">
         <f>'2. 상세견적'!J21</f>
         <v>16500000</v>
       </c>
-      <c r="K27" s="115"/>
-      <c r="L27" s="115"/>
+      <c r="K27" s="187"/>
+      <c r="L27" s="187"/>
     </row>
     <row r="28" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="87">
+      <c r="B28" s="180">
         <v>40</v>
       </c>
-      <c r="C28" s="88"/>
-      <c r="D28" s="110" t="s">
+      <c r="C28" s="181"/>
+      <c r="D28" s="182" t="s">
         <v>31</v>
       </c>
-      <c r="E28" s="111"/>
-      <c r="F28" s="111"/>
-      <c r="G28" s="112" t="s">
+      <c r="E28" s="183"/>
+      <c r="F28" s="183"/>
+      <c r="G28" s="184" t="s">
         <v>32</v>
       </c>
-      <c r="H28" s="113"/>
-      <c r="I28" s="113"/>
-      <c r="J28" s="114">
+      <c r="H28" s="185"/>
+      <c r="I28" s="185"/>
+      <c r="J28" s="186">
         <f>'2. 상세견적'!J24</f>
         <v>16500000</v>
       </c>
-      <c r="K28" s="115"/>
-      <c r="L28" s="115"/>
+      <c r="K28" s="187"/>
+      <c r="L28" s="187"/>
     </row>
     <row r="29" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="87">
+      <c r="B29" s="180">
         <v>50</v>
       </c>
-      <c r="C29" s="88"/>
-      <c r="D29" s="110" t="s">
+      <c r="C29" s="181"/>
+      <c r="D29" s="182" t="s">
         <v>33</v>
       </c>
-      <c r="E29" s="111"/>
-      <c r="F29" s="111"/>
-      <c r="G29" s="112" t="s">
+      <c r="E29" s="183"/>
+      <c r="F29" s="183"/>
+      <c r="G29" s="184" t="s">
         <v>34</v>
       </c>
-      <c r="H29" s="113"/>
-      <c r="I29" s="113"/>
-      <c r="J29" s="114">
+      <c r="H29" s="185"/>
+      <c r="I29" s="185"/>
+      <c r="J29" s="186">
         <f>'2. 상세견적'!J27</f>
         <v>8000000</v>
       </c>
-      <c r="K29" s="115"/>
-      <c r="L29" s="115"/>
+      <c r="K29" s="187"/>
+      <c r="L29" s="187"/>
     </row>
     <row r="30" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="87">
+      <c r="B30" s="180">
         <v>60</v>
       </c>
-      <c r="C30" s="88"/>
-      <c r="D30" s="110" t="s">
+      <c r="C30" s="181"/>
+      <c r="D30" s="182" t="s">
         <v>35</v>
       </c>
-      <c r="E30" s="111"/>
-      <c r="F30" s="111"/>
-      <c r="G30" s="112" t="s">
+      <c r="E30" s="183"/>
+      <c r="F30" s="183"/>
+      <c r="G30" s="184" t="s">
         <v>36</v>
       </c>
-      <c r="H30" s="113"/>
-      <c r="I30" s="113"/>
-      <c r="J30" s="114">
+      <c r="H30" s="185"/>
+      <c r="I30" s="185"/>
+      <c r="J30" s="186">
         <f>'2. 상세견적'!J29</f>
         <v>7000000</v>
       </c>
-      <c r="K30" s="115"/>
-      <c r="L30" s="115"/>
+      <c r="K30" s="187"/>
+      <c r="L30" s="187"/>
     </row>
     <row r="31" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="87">
+      <c r="B31" s="180">
         <v>70</v>
       </c>
-      <c r="C31" s="88"/>
-      <c r="D31" s="110" t="s">
+      <c r="C31" s="181"/>
+      <c r="D31" s="182" t="s">
         <v>37</v>
       </c>
-      <c r="E31" s="111"/>
-      <c r="F31" s="111"/>
-      <c r="G31" s="112" t="s">
+      <c r="E31" s="183"/>
+      <c r="F31" s="183"/>
+      <c r="G31" s="184" t="s">
         <v>38</v>
       </c>
-      <c r="H31" s="113"/>
-      <c r="I31" s="113"/>
-      <c r="J31" s="114">
+      <c r="H31" s="185"/>
+      <c r="I31" s="185"/>
+      <c r="J31" s="186">
         <f>'2. 상세견적'!J34</f>
         <v>12133875</v>
       </c>
-      <c r="K31" s="115"/>
-      <c r="L31" s="115"/>
+      <c r="K31" s="187"/>
+      <c r="L31" s="187"/>
     </row>
     <row r="32" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="187" t="s">
+      <c r="B32" s="200" t="s">
         <v>39</v>
       </c>
-      <c r="C32" s="188"/>
-      <c r="D32" s="189" t="s">
+      <c r="C32" s="201"/>
+      <c r="D32" s="194" t="s">
         <v>40</v>
       </c>
-      <c r="E32" s="190"/>
-      <c r="F32" s="190"/>
-      <c r="G32" s="191" t="s">
+      <c r="E32" s="195"/>
+      <c r="F32" s="195"/>
+      <c r="G32" s="196" t="s">
         <v>41</v>
       </c>
-      <c r="H32" s="192"/>
-      <c r="I32" s="192"/>
-      <c r="J32" s="193">
+      <c r="H32" s="197"/>
+      <c r="I32" s="197"/>
+      <c r="J32" s="198">
         <f>'2. 상세견적'!J38</f>
         <v>-875</v>
       </c>
-      <c r="K32" s="194"/>
-      <c r="L32" s="194"/>
+      <c r="K32" s="199"/>
+      <c r="L32" s="199"/>
     </row>
     <row r="33" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="187" t="s">
+      <c r="B33" s="202" t="s">
         <v>42</v>
       </c>
-      <c r="C33" s="188"/>
-      <c r="D33" s="189" t="s">
+      <c r="C33" s="203"/>
+      <c r="D33" s="188" t="s">
         <v>43</v>
       </c>
-      <c r="E33" s="195"/>
-      <c r="F33" s="195"/>
-      <c r="G33" s="191" t="s">
+      <c r="E33" s="189"/>
+      <c r="F33" s="189"/>
+      <c r="G33" s="190" t="s">
         <v>44</v>
       </c>
-      <c r="H33" s="196"/>
-      <c r="I33" s="196"/>
-      <c r="J33" s="193">
+      <c r="H33" s="191"/>
+      <c r="I33" s="191"/>
+      <c r="J33" s="192">
         <f>'2. 상세견적'!J39</f>
         <v>-10383000</v>
       </c>
-      <c r="K33" s="197"/>
-      <c r="L33" s="197"/>
+      <c r="K33" s="193"/>
+      <c r="L33" s="193"/>
     </row>
     <row r="34" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="198"/>
-      <c r="C34" s="198"/>
-      <c r="D34" s="198"/>
-      <c r="E34" s="198"/>
-      <c r="F34" s="198"/>
-      <c r="G34" s="198"/>
-      <c r="H34" s="198"/>
-      <c r="I34" s="198"/>
-      <c r="J34" s="198"/>
-      <c r="K34" s="198"/>
-      <c r="L34" s="198"/>
+      <c r="B34" s="171"/>
+      <c r="C34" s="171"/>
+      <c r="D34" s="171"/>
+      <c r="E34" s="171"/>
+      <c r="F34" s="171"/>
+      <c r="G34" s="171"/>
+      <c r="H34" s="171"/>
+      <c r="I34" s="171"/>
+      <c r="J34" s="171"/>
+      <c r="K34" s="171"/>
+      <c r="L34" s="171"/>
     </row>
     <row r="35" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="123" t="s">
+      <c r="B35" s="88" t="s">
         <v>45</v>
       </c>
-      <c r="C35" s="123"/>
-      <c r="D35" s="123"/>
-      <c r="E35" s="123"/>
-      <c r="F35" s="123"/>
-      <c r="G35" s="124">
+      <c r="C35" s="88"/>
+      <c r="D35" s="88"/>
+      <c r="E35" s="88"/>
+      <c r="F35" s="88"/>
+      <c r="G35" s="90">
         <f>'2. 상세견적'!J40</f>
         <v>100000000</v>
       </c>
-      <c r="H35" s="125"/>
-      <c r="I35" s="125"/>
-      <c r="J35" s="125"/>
-      <c r="K35" s="125"/>
-      <c r="L35" s="125"/>
+      <c r="H35" s="91"/>
+      <c r="I35" s="91"/>
+      <c r="J35" s="91"/>
+      <c r="K35" s="91"/>
+      <c r="L35" s="91"/>
     </row>
     <row r="36" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="199"/>
-      <c r="C36" s="199"/>
-      <c r="D36" s="199"/>
-      <c r="E36" s="199"/>
-      <c r="F36" s="199"/>
-      <c r="G36" s="200"/>
-      <c r="H36" s="200"/>
-      <c r="I36" s="200"/>
-      <c r="J36" s="200"/>
-      <c r="K36" s="200"/>
-      <c r="L36" s="200"/>
+      <c r="B36" s="89"/>
+      <c r="C36" s="89"/>
+      <c r="D36" s="89"/>
+      <c r="E36" s="89"/>
+      <c r="F36" s="89"/>
+      <c r="G36" s="92"/>
+      <c r="H36" s="92"/>
+      <c r="I36" s="92"/>
+      <c r="J36" s="92"/>
+      <c r="K36" s="92"/>
+      <c r="L36" s="92"/>
     </row>
     <row r="37" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="201" t="s">
+      <c r="B37" s="85" t="s">
         <v>46</v>
       </c>
-      <c r="C37" s="201"/>
-      <c r="D37" s="201"/>
-      <c r="E37" s="201"/>
-      <c r="F37" s="201"/>
-      <c r="G37" s="202" t="s">
+      <c r="C37" s="85"/>
+      <c r="D37" s="85"/>
+      <c r="E37" s="85"/>
+      <c r="F37" s="85"/>
+      <c r="G37" s="86" t="s">
         <v>47</v>
       </c>
-      <c r="H37" s="203"/>
-      <c r="I37" s="203"/>
-      <c r="J37" s="203"/>
-      <c r="K37" s="203"/>
-      <c r="L37" s="203"/>
+      <c r="H37" s="87"/>
+      <c r="I37" s="87"/>
+      <c r="J37" s="87"/>
+      <c r="K37" s="87"/>
+      <c r="L37" s="87"/>
     </row>
     <row r="38" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="3"/>
-      <c r="B38" s="120" t="s">
+      <c r="B38" s="82" t="s">
         <v>48</v>
       </c>
-      <c r="C38" s="120"/>
-      <c r="D38" s="120"/>
-      <c r="E38" s="120"/>
-      <c r="F38" s="120"/>
-      <c r="G38" s="121">
+      <c r="C38" s="82"/>
+      <c r="D38" s="82"/>
+      <c r="E38" s="82"/>
+      <c r="F38" s="82"/>
+      <c r="G38" s="83">
         <f>'2. 상세견적'!J41</f>
         <v>110000000</v>
       </c>
-      <c r="H38" s="122"/>
-      <c r="I38" s="122"/>
-      <c r="J38" s="122"/>
-      <c r="K38" s="122"/>
-      <c r="L38" s="122"/>
+      <c r="H38" s="84"/>
+      <c r="I38" s="84"/>
+      <c r="J38" s="84"/>
+      <c r="K38" s="84"/>
+      <c r="L38" s="84"/>
     </row>
     <row r="39" spans="1:13" ht="267.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="3"/>
-      <c r="B39" s="84"/>
-      <c r="C39" s="84"/>
-      <c r="D39" s="84"/>
-      <c r="E39" s="84"/>
-      <c r="F39" s="84"/>
-      <c r="G39" s="84"/>
-      <c r="H39" s="84"/>
-      <c r="I39" s="84"/>
-      <c r="J39" s="84"/>
-      <c r="K39" s="84"/>
-      <c r="L39" s="84"/>
+      <c r="B39" s="76"/>
+      <c r="C39" s="76"/>
+      <c r="D39" s="76"/>
+      <c r="E39" s="76"/>
+      <c r="F39" s="76"/>
+      <c r="G39" s="76"/>
+      <c r="H39" s="76"/>
+      <c r="I39" s="76"/>
+      <c r="J39" s="76"/>
+      <c r="K39" s="76"/>
+      <c r="L39" s="76"/>
     </row>
     <row r="40" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="3"/>
-      <c r="B40" s="95" t="s">
+      <c r="B40" s="80" t="s">
         <v>49</v>
       </c>
-      <c r="C40" s="96"/>
-      <c r="D40" s="96"/>
-      <c r="E40" s="96"/>
-      <c r="F40" s="96"/>
-      <c r="G40" s="95" t="s">
+      <c r="C40" s="81"/>
+      <c r="D40" s="81"/>
+      <c r="E40" s="81"/>
+      <c r="F40" s="81"/>
+      <c r="G40" s="80" t="s">
         <v>50</v>
       </c>
-      <c r="H40" s="96"/>
-      <c r="I40" s="96"/>
-      <c r="J40" s="96"/>
-      <c r="K40" s="96"/>
-      <c r="L40" s="96"/>
+      <c r="H40" s="81"/>
+      <c r="I40" s="81"/>
+      <c r="J40" s="81"/>
+      <c r="K40" s="81"/>
+      <c r="L40" s="81"/>
     </row>
     <row r="41" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="3"/>
-      <c r="B41" s="97" t="s">
+      <c r="B41" s="78" t="s">
         <v>51</v>
       </c>
-      <c r="C41" s="98"/>
-      <c r="D41" s="98"/>
-      <c r="E41" s="98"/>
-      <c r="F41" s="98"/>
-      <c r="G41" s="97" t="s">
+      <c r="C41" s="79"/>
+      <c r="D41" s="79"/>
+      <c r="E41" s="79"/>
+      <c r="F41" s="79"/>
+      <c r="G41" s="78" t="s">
         <v>52</v>
       </c>
-      <c r="H41" s="98"/>
-      <c r="I41" s="98"/>
-      <c r="J41" s="98"/>
-      <c r="K41" s="98"/>
-      <c r="L41" s="98"/>
+      <c r="H41" s="79"/>
+      <c r="I41" s="79"/>
+      <c r="J41" s="79"/>
+      <c r="K41" s="79"/>
+      <c r="L41" s="79"/>
     </row>
     <row r="42" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="3"/>
-      <c r="B42" s="95" t="s">
+      <c r="B42" s="80" t="s">
         <v>53</v>
       </c>
-      <c r="C42" s="96"/>
-      <c r="D42" s="96"/>
-      <c r="E42" s="96"/>
-      <c r="F42" s="96"/>
-      <c r="G42" s="95" t="s">
+      <c r="C42" s="81"/>
+      <c r="D42" s="81"/>
+      <c r="E42" s="81"/>
+      <c r="F42" s="81"/>
+      <c r="G42" s="80" t="s">
         <v>54</v>
       </c>
-      <c r="H42" s="96"/>
-      <c r="I42" s="96"/>
-      <c r="J42" s="96"/>
-      <c r="K42" s="96"/>
-      <c r="L42" s="96"/>
+      <c r="H42" s="81"/>
+      <c r="I42" s="81"/>
+      <c r="J42" s="81"/>
+      <c r="K42" s="81"/>
+      <c r="L42" s="81"/>
     </row>
     <row r="43" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="3"/>
-      <c r="B43" s="97" t="s">
+      <c r="B43" s="78" t="s">
         <v>55</v>
       </c>
-      <c r="C43" s="98"/>
-      <c r="D43" s="98"/>
-      <c r="E43" s="98"/>
-      <c r="F43" s="98"/>
-      <c r="G43" s="97" t="s">
+      <c r="C43" s="79"/>
+      <c r="D43" s="79"/>
+      <c r="E43" s="79"/>
+      <c r="F43" s="79"/>
+      <c r="G43" s="78" t="s">
         <v>56</v>
       </c>
-      <c r="H43" s="98"/>
-      <c r="I43" s="98"/>
-      <c r="J43" s="98"/>
-      <c r="K43" s="98"/>
-      <c r="L43" s="98"/>
+      <c r="H43" s="79"/>
+      <c r="I43" s="79"/>
+      <c r="J43" s="79"/>
+      <c r="K43" s="79"/>
+      <c r="L43" s="79"/>
     </row>
     <row r="44" spans="1:13" ht="6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="3"/>
-      <c r="B44" s="85"/>
-      <c r="C44" s="85"/>
-      <c r="D44" s="85"/>
-      <c r="E44" s="85"/>
-      <c r="F44" s="85"/>
-      <c r="G44" s="85"/>
-      <c r="H44" s="85"/>
-      <c r="I44" s="85"/>
-      <c r="J44" s="85"/>
-      <c r="K44" s="85"/>
-      <c r="L44" s="85"/>
+      <c r="B44" s="77"/>
+      <c r="C44" s="77"/>
+      <c r="D44" s="77"/>
+      <c r="E44" s="77"/>
+      <c r="F44" s="77"/>
+      <c r="G44" s="77"/>
+      <c r="H44" s="77"/>
+      <c r="I44" s="77"/>
+      <c r="J44" s="77"/>
+      <c r="K44" s="77"/>
+      <c r="L44" s="77"/>
     </row>
     <row r="45" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="3"/>
-      <c r="B45" s="89" t="s">
+      <c r="B45" s="106" t="s">
         <v>57</v>
       </c>
-      <c r="C45" s="90"/>
-      <c r="D45" s="90"/>
-      <c r="E45" s="90"/>
-      <c r="F45" s="90"/>
-      <c r="G45" s="90"/>
-      <c r="H45" s="90"/>
-      <c r="I45" s="90"/>
-      <c r="J45" s="90"/>
-      <c r="K45" s="90"/>
-      <c r="L45" s="90"/>
+      <c r="C45" s="107"/>
+      <c r="D45" s="107"/>
+      <c r="E45" s="107"/>
+      <c r="F45" s="107"/>
+      <c r="G45" s="107"/>
+      <c r="H45" s="107"/>
+      <c r="I45" s="107"/>
+      <c r="J45" s="107"/>
+      <c r="K45" s="107"/>
+      <c r="L45" s="107"/>
     </row>
     <row r="46" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="3"/>
-      <c r="B46" s="90"/>
-      <c r="C46" s="90"/>
-      <c r="D46" s="90"/>
-      <c r="E46" s="90"/>
-      <c r="F46" s="90"/>
-      <c r="G46" s="90"/>
-      <c r="H46" s="90"/>
-      <c r="I46" s="90"/>
-      <c r="J46" s="90"/>
-      <c r="K46" s="90"/>
-      <c r="L46" s="90"/>
+      <c r="B46" s="107"/>
+      <c r="C46" s="107"/>
+      <c r="D46" s="107"/>
+      <c r="E46" s="107"/>
+      <c r="F46" s="107"/>
+      <c r="G46" s="107"/>
+      <c r="H46" s="107"/>
+      <c r="I46" s="107"/>
+      <c r="J46" s="107"/>
+      <c r="K46" s="107"/>
+      <c r="L46" s="107"/>
     </row>
     <row r="47" spans="1:13" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="3"/>
-      <c r="B47" s="79"/>
-      <c r="C47" s="79"/>
-      <c r="D47" s="79"/>
-      <c r="E47" s="79"/>
-      <c r="F47" s="79"/>
-      <c r="G47" s="79"/>
-      <c r="H47" s="79"/>
-      <c r="I47" s="79"/>
-      <c r="J47" s="79"/>
-      <c r="K47" s="79"/>
-      <c r="L47" s="79"/>
+      <c r="B47" s="71"/>
+      <c r="C47" s="71"/>
+      <c r="D47" s="71"/>
+      <c r="E47" s="71"/>
+      <c r="F47" s="71"/>
+      <c r="G47" s="71"/>
+      <c r="H47" s="71"/>
+      <c r="I47" s="71"/>
+      <c r="J47" s="71"/>
+      <c r="K47" s="71"/>
+      <c r="L47" s="71"/>
     </row>
     <row r="48" spans="1:13" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="76"/>
-      <c r="B48" s="91" t="s">
+      <c r="A48" s="68"/>
+      <c r="B48" s="108" t="s">
         <v>58</v>
       </c>
-      <c r="C48" s="91"/>
-      <c r="D48" s="91"/>
-      <c r="E48" s="91"/>
-      <c r="F48" s="91"/>
-      <c r="G48" s="93" t="s">
+      <c r="C48" s="108"/>
+      <c r="D48" s="108"/>
+      <c r="E48" s="108"/>
+      <c r="F48" s="108"/>
+      <c r="G48" s="110" t="s">
         <v>59</v>
       </c>
-      <c r="H48" s="93"/>
-      <c r="I48" s="93"/>
-      <c r="J48" s="93"/>
-      <c r="K48" s="93"/>
-      <c r="L48" s="93"/>
-      <c r="M48" s="77"/>
+      <c r="H48" s="110"/>
+      <c r="I48" s="110"/>
+      <c r="J48" s="110"/>
+      <c r="K48" s="110"/>
+      <c r="L48" s="110"/>
+      <c r="M48" s="69"/>
     </row>
     <row r="49" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="75"/>
-      <c r="B49" s="92"/>
-      <c r="C49" s="92"/>
-      <c r="D49" s="92"/>
-      <c r="E49" s="92"/>
-      <c r="F49" s="92"/>
-      <c r="G49" s="94"/>
-      <c r="H49" s="94"/>
-      <c r="I49" s="94"/>
-      <c r="J49" s="94"/>
-      <c r="K49" s="94"/>
-      <c r="L49" s="94"/>
-      <c r="M49" s="74"/>
+      <c r="A49" s="67"/>
+      <c r="B49" s="109"/>
+      <c r="C49" s="109"/>
+      <c r="D49" s="109"/>
+      <c r="E49" s="109"/>
+      <c r="F49" s="109"/>
+      <c r="G49" s="111"/>
+      <c r="H49" s="111"/>
+      <c r="I49" s="111"/>
+      <c r="J49" s="111"/>
+      <c r="K49" s="111"/>
+      <c r="L49" s="111"/>
+      <c r="M49" s="66"/>
     </row>
     <row r="50" spans="1:13" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="75"/>
-      <c r="B50" s="92"/>
-      <c r="C50" s="92"/>
-      <c r="D50" s="92"/>
-      <c r="E50" s="92"/>
-      <c r="F50" s="92"/>
-      <c r="G50" s="94"/>
-      <c r="H50" s="94"/>
-      <c r="I50" s="94"/>
-      <c r="J50" s="94"/>
-      <c r="K50" s="94"/>
-      <c r="L50" s="94"/>
-      <c r="M50" s="74"/>
+      <c r="A50" s="67"/>
+      <c r="B50" s="109"/>
+      <c r="C50" s="109"/>
+      <c r="D50" s="109"/>
+      <c r="E50" s="109"/>
+      <c r="F50" s="109"/>
+      <c r="G50" s="111"/>
+      <c r="H50" s="111"/>
+      <c r="I50" s="111"/>
+      <c r="J50" s="111"/>
+      <c r="K50" s="111"/>
+      <c r="L50" s="111"/>
+      <c r="M50" s="66"/>
     </row>
   </sheetData>
   <mergeCells count="65">
+    <mergeCell ref="B45:L46"/>
+    <mergeCell ref="B48:F50"/>
+    <mergeCell ref="G48:L50"/>
+    <mergeCell ref="B42:F42"/>
+    <mergeCell ref="G42:L42"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="G43:L43"/>
+    <mergeCell ref="H5:K5"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="B12:L13"/>
+    <mergeCell ref="B9:L10"/>
+    <mergeCell ref="B11:L11"/>
+    <mergeCell ref="G19:L19"/>
+    <mergeCell ref="H20:L20"/>
+    <mergeCell ref="H21:L21"/>
+    <mergeCell ref="H22:L22"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="G15:L15"/>
+    <mergeCell ref="B16:F17"/>
+    <mergeCell ref="G16:L17"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B20:F22"/>
+    <mergeCell ref="D26:F26"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="J26:L26"/>
+    <mergeCell ref="B23:H23"/>
+    <mergeCell ref="I23:L23"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="J24:L24"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="G25:I25"/>
+    <mergeCell ref="J25:L25"/>
+    <mergeCell ref="D27:F27"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="J27:L27"/>
+    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="G28:I28"/>
+    <mergeCell ref="J28:L28"/>
+    <mergeCell ref="D29:F29"/>
+    <mergeCell ref="G29:I29"/>
+    <mergeCell ref="J29:L29"/>
+    <mergeCell ref="D30:F30"/>
+    <mergeCell ref="G30:I30"/>
+    <mergeCell ref="J30:L30"/>
+    <mergeCell ref="D31:F31"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="J31:L31"/>
+    <mergeCell ref="D32:F32"/>
+    <mergeCell ref="G32:I32"/>
+    <mergeCell ref="J32:L32"/>
     <mergeCell ref="B41:F41"/>
     <mergeCell ref="G41:L41"/>
     <mergeCell ref="D33:F33"/>
@@ -29187,62 +28786,10 @@
     <mergeCell ref="G37:L37"/>
     <mergeCell ref="B35:F36"/>
     <mergeCell ref="G35:L36"/>
-    <mergeCell ref="D31:F31"/>
-    <mergeCell ref="G31:I31"/>
-    <mergeCell ref="J31:L31"/>
-    <mergeCell ref="D32:F32"/>
-    <mergeCell ref="G32:I32"/>
-    <mergeCell ref="J32:L32"/>
-    <mergeCell ref="D29:F29"/>
-    <mergeCell ref="G29:I29"/>
-    <mergeCell ref="J29:L29"/>
-    <mergeCell ref="D30:F30"/>
-    <mergeCell ref="G30:I30"/>
-    <mergeCell ref="J30:L30"/>
-    <mergeCell ref="D27:F27"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="J27:L27"/>
-    <mergeCell ref="D28:F28"/>
-    <mergeCell ref="G28:I28"/>
-    <mergeCell ref="J28:L28"/>
-    <mergeCell ref="D26:F26"/>
-    <mergeCell ref="G26:I26"/>
-    <mergeCell ref="J26:L26"/>
-    <mergeCell ref="B23:H23"/>
-    <mergeCell ref="I23:L23"/>
-    <mergeCell ref="D24:F24"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="J24:L24"/>
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="G25:I25"/>
-    <mergeCell ref="J25:L25"/>
-    <mergeCell ref="G19:L19"/>
-    <mergeCell ref="H20:L20"/>
-    <mergeCell ref="H21:L21"/>
-    <mergeCell ref="H22:L22"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="G15:L15"/>
-    <mergeCell ref="B16:F17"/>
-    <mergeCell ref="G16:L17"/>
-    <mergeCell ref="B19:F19"/>
-    <mergeCell ref="B20:F22"/>
-    <mergeCell ref="H5:K5"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="H7:K7"/>
-    <mergeCell ref="B12:L13"/>
-    <mergeCell ref="B9:L10"/>
-    <mergeCell ref="B11:L11"/>
-    <mergeCell ref="B45:L46"/>
-    <mergeCell ref="B48:F50"/>
-    <mergeCell ref="G48:L50"/>
-    <mergeCell ref="B42:F42"/>
-    <mergeCell ref="G42:L42"/>
-    <mergeCell ref="B43:F43"/>
-    <mergeCell ref="G43:L43"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="72" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -29268,40 +28815,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="3.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="73"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
-      <c r="L1" s="73"/>
-      <c r="M1" s="73"/>
-      <c r="N1" s="73"/>
-      <c r="O1" s="73"/>
-      <c r="P1" s="73"/>
-      <c r="Q1" s="73"/>
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="65"/>
+      <c r="H1" s="65"/>
+      <c r="I1" s="65"/>
+      <c r="J1" s="65"/>
+      <c r="K1" s="65"/>
+      <c r="L1" s="65"/>
+      <c r="M1" s="65"/>
+      <c r="N1" s="65"/>
+      <c r="O1" s="65"/>
+      <c r="P1" s="65"/>
+      <c r="Q1" s="65"/>
     </row>
     <row r="2" spans="1:17" ht="2.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="73"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
-      <c r="H2" s="73"/>
-      <c r="I2" s="73"/>
-      <c r="J2" s="73"/>
-      <c r="K2" s="73"/>
-      <c r="L2" s="73"/>
-      <c r="M2" s="73"/>
-      <c r="N2" s="73"/>
-      <c r="O2" s="73"/>
-      <c r="P2" s="73"/>
-      <c r="Q2" s="73"/>
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="65"/>
+      <c r="F2" s="65"/>
+      <c r="G2" s="65"/>
+      <c r="H2" s="65"/>
+      <c r="I2" s="65"/>
+      <c r="J2" s="65"/>
+      <c r="K2" s="65"/>
+      <c r="L2" s="65"/>
+      <c r="M2" s="65"/>
+      <c r="N2" s="65"/>
+      <c r="O2" s="65"/>
+      <c r="P2" s="65"/>
+      <c r="Q2" s="65"/>
     </row>
     <row r="3" spans="1:17" ht="6.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="10"/>
@@ -29322,7 +28869,7 @@
       <c r="Q3" s="10"/>
     </row>
     <row r="4" spans="1:17" ht="12.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="78"/>
+      <c r="A4" s="70"/>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
       <c r="D4" s="10"/>
@@ -29332,7 +28879,7 @@
       <c r="H4" s="10"/>
       <c r="I4" s="10"/>
       <c r="J4" s="10"/>
-      <c r="K4" s="73"/>
+      <c r="K4" s="65"/>
       <c r="L4" s="10"/>
       <c r="M4" s="10"/>
       <c r="N4" s="10"/>
@@ -29341,57 +28888,57 @@
       <c r="Q4" s="10"/>
     </row>
     <row r="5" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="78"/>
-      <c r="B5" s="148" t="s">
+      <c r="A5" s="70"/>
+      <c r="B5" s="144" t="s">
         <v>60</v>
       </c>
-      <c r="C5" s="148"/>
-      <c r="D5" s="148"/>
-      <c r="E5" s="148"/>
-      <c r="F5" s="148"/>
-      <c r="G5" s="150" t="s">
+      <c r="C5" s="144"/>
+      <c r="D5" s="144"/>
+      <c r="E5" s="144"/>
+      <c r="F5" s="144"/>
+      <c r="G5" s="146" t="s">
         <v>1</v>
       </c>
-      <c r="H5" s="150"/>
-      <c r="I5" s="150"/>
-      <c r="J5" s="150"/>
-      <c r="K5" s="73"/>
-      <c r="L5" s="140" t="s">
+      <c r="H5" s="146"/>
+      <c r="I5" s="146"/>
+      <c r="J5" s="146"/>
+      <c r="K5" s="65"/>
+      <c r="L5" s="136" t="s">
         <v>61</v>
       </c>
-      <c r="M5" s="141"/>
-      <c r="N5" s="141"/>
-      <c r="O5" s="141"/>
-      <c r="P5" s="141"/>
-      <c r="Q5" s="141"/>
+      <c r="M5" s="137"/>
+      <c r="N5" s="137"/>
+      <c r="O5" s="137"/>
+      <c r="P5" s="137"/>
+      <c r="Q5" s="137"/>
     </row>
     <row r="6" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="78"/>
-      <c r="B6" s="149" t="s">
+      <c r="A6" s="70"/>
+      <c r="B6" s="145" t="s">
         <v>62</v>
       </c>
-      <c r="C6" s="149"/>
-      <c r="D6" s="149"/>
-      <c r="E6" s="149"/>
-      <c r="F6" s="149"/>
-      <c r="G6" s="151" t="s">
+      <c r="C6" s="145"/>
+      <c r="D6" s="145"/>
+      <c r="E6" s="145"/>
+      <c r="F6" s="145"/>
+      <c r="G6" s="147" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="151"/>
-      <c r="I6" s="151"/>
-      <c r="J6" s="151"/>
-      <c r="K6" s="73"/>
-      <c r="L6" s="142" t="s">
+      <c r="H6" s="147"/>
+      <c r="I6" s="147"/>
+      <c r="J6" s="147"/>
+      <c r="K6" s="65"/>
+      <c r="L6" s="138" t="s">
         <v>63</v>
       </c>
-      <c r="M6" s="143"/>
-      <c r="N6" s="143"/>
-      <c r="O6" s="143"/>
-      <c r="P6" s="143"/>
-      <c r="Q6" s="143"/>
+      <c r="M6" s="139"/>
+      <c r="N6" s="139"/>
+      <c r="O6" s="139"/>
+      <c r="P6" s="139"/>
+      <c r="Q6" s="139"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A7" s="78"/>
+      <c r="A7" s="70"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
@@ -29401,43 +28948,43 @@
       <c r="H7" s="10"/>
       <c r="I7" s="10"/>
       <c r="J7" s="10"/>
-      <c r="K7" s="73"/>
-      <c r="L7" s="142"/>
-      <c r="M7" s="143"/>
-      <c r="N7" s="143"/>
-      <c r="O7" s="143"/>
-      <c r="P7" s="143"/>
-      <c r="Q7" s="143"/>
+      <c r="K7" s="65"/>
+      <c r="L7" s="138"/>
+      <c r="M7" s="139"/>
+      <c r="N7" s="139"/>
+      <c r="O7" s="139"/>
+      <c r="P7" s="139"/>
+      <c r="Q7" s="139"/>
     </row>
     <row r="8" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="78"/>
-      <c r="B8" s="152" t="s">
+      <c r="A8" s="70"/>
+      <c r="B8" s="148" t="s">
         <v>64</v>
       </c>
-      <c r="C8" s="152"/>
-      <c r="D8" s="152"/>
-      <c r="E8" s="152"/>
-      <c r="F8" s="152"/>
-      <c r="G8" s="153" t="s">
+      <c r="C8" s="148"/>
+      <c r="D8" s="148"/>
+      <c r="E8" s="148"/>
+      <c r="F8" s="148"/>
+      <c r="G8" s="149" t="s">
         <v>20</v>
       </c>
-      <c r="H8" s="153"/>
-      <c r="I8" s="153"/>
-      <c r="J8" s="153"/>
-      <c r="K8" s="73"/>
-      <c r="L8" s="144" t="s">
+      <c r="H8" s="149"/>
+      <c r="I8" s="149"/>
+      <c r="J8" s="149"/>
+      <c r="K8" s="65"/>
+      <c r="L8" s="140" t="s">
         <v>65</v>
       </c>
-      <c r="M8" s="145"/>
-      <c r="N8" s="145"/>
-      <c r="O8" s="145" t="s">
+      <c r="M8" s="141"/>
+      <c r="N8" s="141"/>
+      <c r="O8" s="141" t="s">
         <v>66</v>
       </c>
-      <c r="P8" s="145"/>
-      <c r="Q8" s="145"/>
+      <c r="P8" s="141"/>
+      <c r="Q8" s="141"/>
     </row>
     <row r="9" spans="1:17" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="78"/>
+      <c r="A9" s="70"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
@@ -29447,33 +28994,33 @@
       <c r="H9" s="10"/>
       <c r="I9" s="10"/>
       <c r="J9" s="10"/>
-      <c r="K9" s="73"/>
-      <c r="L9" s="146">
+      <c r="K9" s="65"/>
+      <c r="L9" s="142">
         <f>$J$37</f>
         <v>110383875</v>
       </c>
-      <c r="M9" s="147"/>
-      <c r="N9" s="147"/>
-      <c r="O9" s="147">
+      <c r="M9" s="143"/>
+      <c r="N9" s="143"/>
+      <c r="O9" s="143">
         <f>$J$40</f>
         <v>100000000</v>
       </c>
-      <c r="P9" s="147"/>
-      <c r="Q9" s="147"/>
+      <c r="P9" s="143"/>
+      <c r="Q9" s="143"/>
     </row>
     <row r="10" spans="1:17" ht="23.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="78"/>
+      <c r="A10" s="70"/>
       <c r="B10" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="C10" s="139" t="s">
+      <c r="C10" s="135" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="139"/>
-      <c r="E10" s="139" t="s">
+      <c r="D10" s="135"/>
+      <c r="E10" s="135" t="s">
         <v>69</v>
       </c>
-      <c r="F10" s="139"/>
+      <c r="F10" s="135"/>
       <c r="G10" s="5" t="s">
         <v>70</v>
       </c>
@@ -29486,88 +29033,88 @@
       <c r="J10" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="K10" s="73"/>
-      <c r="L10" s="146"/>
-      <c r="M10" s="147"/>
-      <c r="N10" s="147"/>
-      <c r="O10" s="147"/>
-      <c r="P10" s="147"/>
-      <c r="Q10" s="147"/>
+      <c r="K10" s="65"/>
+      <c r="L10" s="142"/>
+      <c r="M10" s="143"/>
+      <c r="N10" s="143"/>
+      <c r="O10" s="143"/>
+      <c r="P10" s="143"/>
+      <c r="Q10" s="143"/>
     </row>
     <row r="11" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="78"/>
-      <c r="B11" s="44">
+      <c r="A11" s="70"/>
+      <c r="B11" s="40">
         <v>10</v>
       </c>
-      <c r="C11" s="154" t="s">
+      <c r="C11" s="121" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="154"/>
-      <c r="E11" s="154" t="s">
+      <c r="D11" s="121"/>
+      <c r="E11" s="121" t="s">
         <v>73</v>
       </c>
-      <c r="F11" s="154"/>
-      <c r="G11" s="45"/>
-      <c r="H11" s="45"/>
-      <c r="I11" s="46"/>
-      <c r="J11" s="47">
+      <c r="F11" s="121"/>
+      <c r="G11" s="41"/>
+      <c r="H11" s="41"/>
+      <c r="I11" s="42"/>
+      <c r="J11" s="43">
         <f>SUM(J12,J15)</f>
         <v>40000000</v>
       </c>
-      <c r="K11" s="73"/>
-      <c r="L11" s="146"/>
-      <c r="M11" s="147"/>
-      <c r="N11" s="147"/>
-      <c r="O11" s="147"/>
-      <c r="P11" s="147"/>
-      <c r="Q11" s="147"/>
+      <c r="K11" s="65"/>
+      <c r="L11" s="142"/>
+      <c r="M11" s="143"/>
+      <c r="N11" s="143"/>
+      <c r="O11" s="143"/>
+      <c r="P11" s="143"/>
+      <c r="Q11" s="143"/>
     </row>
     <row r="12" spans="1:17" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="78"/>
-      <c r="B12" s="52">
+      <c r="A12" s="70"/>
+      <c r="B12" s="44">
         <v>11</v>
       </c>
-      <c r="C12" s="156" t="s">
+      <c r="C12" s="126" t="s">
         <v>74</v>
       </c>
-      <c r="D12" s="156"/>
-      <c r="E12" s="156" t="s">
+      <c r="D12" s="126"/>
+      <c r="E12" s="126" t="s">
         <v>75</v>
       </c>
-      <c r="F12" s="156"/>
-      <c r="G12" s="53"/>
-      <c r="H12" s="53"/>
-      <c r="I12" s="54"/>
-      <c r="J12" s="55">
+      <c r="F12" s="126"/>
+      <c r="G12" s="45"/>
+      <c r="H12" s="45"/>
+      <c r="I12" s="46"/>
+      <c r="J12" s="47">
         <f>SUM(J13:J14)</f>
         <v>30000000</v>
       </c>
-      <c r="K12" s="73"/>
+      <c r="K12" s="65"/>
       <c r="L12" s="128" t="s">
         <v>76</v>
       </c>
       <c r="M12" s="129"/>
       <c r="N12" s="129"/>
       <c r="O12" s="129"/>
-      <c r="P12" s="138">
+      <c r="P12" s="130">
         <f>ABS(($J$38+$J$39)/$J$37)</f>
         <v>9.4070578696390211E-2</v>
       </c>
-      <c r="Q12" s="138"/>
+      <c r="Q12" s="130"/>
     </row>
     <row r="13" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="78"/>
+      <c r="A13" s="70"/>
       <c r="B13" s="18">
         <v>11.01</v>
       </c>
-      <c r="C13" s="157" t="s">
+      <c r="C13" s="125" t="s">
         <v>77</v>
       </c>
-      <c r="D13" s="157"/>
-      <c r="E13" s="158" t="s">
+      <c r="D13" s="125"/>
+      <c r="E13" s="127" t="s">
         <v>78</v>
       </c>
-      <c r="F13" s="158"/>
+      <c r="F13" s="127"/>
       <c r="G13" s="14" t="s">
         <v>79</v>
       </c>
@@ -29581,27 +29128,27 @@
         <f>H13*I13</f>
         <v>20000000</v>
       </c>
-      <c r="K13" s="73"/>
-      <c r="L13" s="70"/>
-      <c r="M13" s="71"/>
-      <c r="N13" s="71"/>
-      <c r="O13" s="71"/>
-      <c r="P13" s="71"/>
-      <c r="Q13" s="71"/>
+      <c r="K13" s="65"/>
+      <c r="L13" s="62"/>
+      <c r="M13" s="63"/>
+      <c r="N13" s="63"/>
+      <c r="O13" s="63"/>
+      <c r="P13" s="63"/>
+      <c r="Q13" s="63"/>
     </row>
     <row r="14" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="78"/>
+      <c r="A14" s="70"/>
       <c r="B14" s="18">
         <v>11.02</v>
       </c>
-      <c r="C14" s="157" t="s">
+      <c r="C14" s="125" t="s">
         <v>80</v>
       </c>
-      <c r="D14" s="157"/>
-      <c r="E14" s="158" t="s">
+      <c r="D14" s="125"/>
+      <c r="E14" s="127" t="s">
         <v>78</v>
       </c>
-      <c r="F14" s="158"/>
+      <c r="F14" s="127"/>
       <c r="G14" s="14" t="s">
         <v>79</v>
       </c>
@@ -29615,57 +29162,57 @@
         <f>H14*I14</f>
         <v>10000000</v>
       </c>
-      <c r="K14" s="73"/>
-      <c r="L14" s="136" t="s">
+      <c r="K14" s="65"/>
+      <c r="L14" s="131" t="s">
         <v>81</v>
       </c>
-      <c r="M14" s="137"/>
-      <c r="N14" s="137"/>
-      <c r="O14" s="137"/>
-      <c r="P14" s="137"/>
-      <c r="Q14" s="137"/>
+      <c r="M14" s="132"/>
+      <c r="N14" s="132"/>
+      <c r="O14" s="132"/>
+      <c r="P14" s="132"/>
+      <c r="Q14" s="132"/>
     </row>
     <row r="15" spans="1:17" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="78"/>
-      <c r="B15" s="52">
+      <c r="A15" s="70"/>
+      <c r="B15" s="44">
         <v>12</v>
       </c>
-      <c r="C15" s="156" t="s">
+      <c r="C15" s="126" t="s">
         <v>82</v>
       </c>
-      <c r="D15" s="156"/>
-      <c r="E15" s="156" t="s">
+      <c r="D15" s="126"/>
+      <c r="E15" s="126" t="s">
         <v>75</v>
       </c>
-      <c r="F15" s="156"/>
-      <c r="G15" s="53"/>
-      <c r="H15" s="53"/>
-      <c r="I15" s="54"/>
-      <c r="J15" s="55">
+      <c r="F15" s="126"/>
+      <c r="G15" s="45"/>
+      <c r="H15" s="45"/>
+      <c r="I15" s="46"/>
+      <c r="J15" s="47">
         <f>SUM(J16:J17)</f>
         <v>10000000</v>
       </c>
-      <c r="K15" s="73"/>
-      <c r="L15" s="70"/>
-      <c r="M15" s="71"/>
-      <c r="N15" s="71"/>
-      <c r="O15" s="71"/>
-      <c r="P15" s="71"/>
-      <c r="Q15" s="71"/>
+      <c r="K15" s="65"/>
+      <c r="L15" s="62"/>
+      <c r="M15" s="63"/>
+      <c r="N15" s="63"/>
+      <c r="O15" s="63"/>
+      <c r="P15" s="63"/>
+      <c r="Q15" s="63"/>
     </row>
     <row r="16" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="78"/>
+      <c r="A16" s="70"/>
       <c r="B16" s="18">
         <v>12.01</v>
       </c>
-      <c r="C16" s="157" t="s">
+      <c r="C16" s="125" t="s">
         <v>83</v>
       </c>
-      <c r="D16" s="157"/>
-      <c r="E16" s="158" t="s">
+      <c r="D16" s="125"/>
+      <c r="E16" s="127" t="s">
         <v>78</v>
       </c>
-      <c r="F16" s="158"/>
+      <c r="F16" s="127"/>
       <c r="G16" s="14" t="s">
         <v>79</v>
       </c>
@@ -29679,32 +29226,32 @@
         <f>H16*I16</f>
         <v>8000000</v>
       </c>
-      <c r="K16" s="73"/>
-      <c r="L16" s="127" t="s">
+      <c r="K16" s="65"/>
+      <c r="L16" s="133" t="s">
         <v>84</v>
       </c>
-      <c r="M16" s="126"/>
-      <c r="N16" s="126"/>
-      <c r="O16" s="126"/>
-      <c r="P16" s="126"/>
-      <c r="Q16" s="72">
+      <c r="M16" s="134"/>
+      <c r="N16" s="134"/>
+      <c r="O16" s="134"/>
+      <c r="P16" s="134"/>
+      <c r="Q16" s="64">
         <f>$J$11/$J$33</f>
         <v>0.40712468193384221</v>
       </c>
     </row>
     <row r="17" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="78"/>
+      <c r="A17" s="70"/>
       <c r="B17" s="18">
         <v>12.02</v>
       </c>
-      <c r="C17" s="157" t="s">
+      <c r="C17" s="125" t="s">
         <v>85</v>
       </c>
-      <c r="D17" s="157"/>
-      <c r="E17" s="158" t="s">
+      <c r="D17" s="125"/>
+      <c r="E17" s="127" t="s">
         <v>78</v>
       </c>
-      <c r="F17" s="158"/>
+      <c r="F17" s="127"/>
       <c r="G17" s="14" t="s">
         <v>79</v>
       </c>
@@ -29718,55 +29265,55 @@
         <f>H17*I17</f>
         <v>2000000</v>
       </c>
-      <c r="K17" s="73"/>
-      <c r="L17" s="70"/>
-      <c r="M17" s="71"/>
-      <c r="N17" s="68"/>
-      <c r="O17" s="68"/>
-      <c r="P17" s="68"/>
-      <c r="Q17" s="69"/>
+      <c r="K17" s="65"/>
+      <c r="L17" s="62"/>
+      <c r="M17" s="63"/>
+      <c r="N17" s="60"/>
+      <c r="O17" s="60"/>
+      <c r="P17" s="60"/>
+      <c r="Q17" s="61"/>
     </row>
     <row r="18" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="78"/>
-      <c r="B18" s="44">
+      <c r="A18" s="70"/>
+      <c r="B18" s="40">
         <v>20</v>
       </c>
-      <c r="C18" s="154" t="s">
+      <c r="C18" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="D18" s="154"/>
-      <c r="E18" s="154" t="s">
+      <c r="D18" s="121"/>
+      <c r="E18" s="121" t="s">
         <v>86</v>
       </c>
-      <c r="F18" s="154"/>
-      <c r="G18" s="45"/>
-      <c r="H18" s="45"/>
-      <c r="I18" s="46"/>
-      <c r="J18" s="47">
+      <c r="F18" s="121"/>
+      <c r="G18" s="41"/>
+      <c r="H18" s="41"/>
+      <c r="I18" s="42"/>
+      <c r="J18" s="43">
         <f>SUM(J19:J20)</f>
         <v>10250000</v>
       </c>
-      <c r="K18" s="73"/>
-      <c r="L18" s="70"/>
-      <c r="M18" s="71"/>
-      <c r="N18" s="68"/>
-      <c r="O18" s="68"/>
-      <c r="P18" s="68"/>
-      <c r="Q18" s="69"/>
+      <c r="K18" s="65"/>
+      <c r="L18" s="62"/>
+      <c r="M18" s="63"/>
+      <c r="N18" s="60"/>
+      <c r="O18" s="60"/>
+      <c r="P18" s="60"/>
+      <c r="Q18" s="61"/>
     </row>
     <row r="19" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="78"/>
+      <c r="A19" s="70"/>
       <c r="B19" s="18">
         <v>20.010000000000002</v>
       </c>
-      <c r="C19" s="155" t="s">
+      <c r="C19" s="122" t="s">
         <v>87</v>
       </c>
-      <c r="D19" s="155"/>
-      <c r="E19" s="155" t="s">
+      <c r="D19" s="122"/>
+      <c r="E19" s="122" t="s">
         <v>88</v>
       </c>
-      <c r="F19" s="155"/>
+      <c r="F19" s="122"/>
       <c r="G19" s="14" t="s">
         <v>89</v>
       </c>
@@ -29781,32 +29328,32 @@
         <f>H19*I19</f>
         <v>8000000</v>
       </c>
-      <c r="K19" s="73"/>
-      <c r="L19" s="127" t="s">
+      <c r="K19" s="65"/>
+      <c r="L19" s="133" t="s">
         <v>90</v>
       </c>
-      <c r="M19" s="126"/>
-      <c r="N19" s="126"/>
-      <c r="O19" s="126"/>
-      <c r="P19" s="126"/>
-      <c r="Q19" s="72">
+      <c r="M19" s="134"/>
+      <c r="N19" s="134"/>
+      <c r="O19" s="134"/>
+      <c r="P19" s="134"/>
+      <c r="Q19" s="64">
         <f>SUM($J$18,$J$21,$J$24,$J$27)/$J$33</f>
         <v>0.52162849872773542</v>
       </c>
     </row>
     <row r="20" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="78"/>
+      <c r="A20" s="70"/>
       <c r="B20" s="18">
         <v>20.02</v>
       </c>
-      <c r="C20" s="155" t="s">
+      <c r="C20" s="122" t="s">
         <v>91</v>
       </c>
-      <c r="D20" s="155"/>
-      <c r="E20" s="155" t="s">
+      <c r="D20" s="122"/>
+      <c r="E20" s="122" t="s">
         <v>92</v>
       </c>
-      <c r="F20" s="155"/>
+      <c r="F20" s="122"/>
       <c r="G20" s="14" t="s">
         <v>89</v>
       </c>
@@ -29821,55 +29368,55 @@
         <f>H20*I20</f>
         <v>2250000</v>
       </c>
-      <c r="K20" s="73"/>
-      <c r="L20" s="70"/>
-      <c r="M20" s="71"/>
-      <c r="N20" s="68"/>
-      <c r="O20" s="68"/>
-      <c r="P20" s="68"/>
-      <c r="Q20" s="69"/>
+      <c r="K20" s="65"/>
+      <c r="L20" s="62"/>
+      <c r="M20" s="63"/>
+      <c r="N20" s="60"/>
+      <c r="O20" s="60"/>
+      <c r="P20" s="60"/>
+      <c r="Q20" s="61"/>
     </row>
     <row r="21" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="78"/>
-      <c r="B21" s="44">
+      <c r="A21" s="70"/>
+      <c r="B21" s="40">
         <v>30</v>
       </c>
-      <c r="C21" s="154" t="s">
+      <c r="C21" s="121" t="s">
         <v>29</v>
       </c>
-      <c r="D21" s="154"/>
-      <c r="E21" s="154" t="s">
+      <c r="D21" s="121"/>
+      <c r="E21" s="121" t="s">
         <v>86</v>
       </c>
-      <c r="F21" s="154"/>
-      <c r="G21" s="45"/>
-      <c r="H21" s="45"/>
-      <c r="I21" s="46"/>
-      <c r="J21" s="47">
+      <c r="F21" s="121"/>
+      <c r="G21" s="41"/>
+      <c r="H21" s="41"/>
+      <c r="I21" s="42"/>
+      <c r="J21" s="43">
         <f>SUM(J22:J23)</f>
         <v>16500000</v>
       </c>
-      <c r="K21" s="73"/>
-      <c r="L21" s="70"/>
-      <c r="M21" s="71"/>
-      <c r="N21" s="68"/>
-      <c r="O21" s="68"/>
-      <c r="P21" s="68"/>
-      <c r="Q21" s="69"/>
+      <c r="K21" s="65"/>
+      <c r="L21" s="62"/>
+      <c r="M21" s="63"/>
+      <c r="N21" s="60"/>
+      <c r="O21" s="60"/>
+      <c r="P21" s="60"/>
+      <c r="Q21" s="61"/>
     </row>
     <row r="22" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="78"/>
+      <c r="A22" s="70"/>
       <c r="B22" s="18">
         <v>30.01</v>
       </c>
-      <c r="C22" s="155" t="s">
+      <c r="C22" s="122" t="s">
         <v>93</v>
       </c>
-      <c r="D22" s="155"/>
-      <c r="E22" s="155" t="s">
+      <c r="D22" s="122"/>
+      <c r="E22" s="122" t="s">
         <v>88</v>
       </c>
-      <c r="F22" s="155"/>
+      <c r="F22" s="122"/>
       <c r="G22" s="14" t="s">
         <v>89</v>
       </c>
@@ -29884,32 +29431,32 @@
         <f>H22*I22</f>
         <v>12000000</v>
       </c>
-      <c r="K22" s="73"/>
-      <c r="L22" s="127" t="s">
+      <c r="K22" s="65"/>
+      <c r="L22" s="133" t="s">
         <v>94</v>
       </c>
-      <c r="M22" s="126"/>
-      <c r="N22" s="126"/>
-      <c r="O22" s="126"/>
-      <c r="P22" s="126"/>
-      <c r="Q22" s="72">
+      <c r="M22" s="134"/>
+      <c r="N22" s="134"/>
+      <c r="O22" s="134"/>
+      <c r="P22" s="134"/>
+      <c r="Q22" s="64">
         <f>$J$29/$J$33</f>
         <v>7.124681933842239E-2</v>
       </c>
     </row>
     <row r="23" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="78"/>
+      <c r="A23" s="70"/>
       <c r="B23" s="18">
         <v>30.02</v>
       </c>
-      <c r="C23" s="155" t="s">
+      <c r="C23" s="122" t="s">
         <v>95</v>
       </c>
-      <c r="D23" s="155"/>
-      <c r="E23" s="155" t="s">
+      <c r="D23" s="122"/>
+      <c r="E23" s="122" t="s">
         <v>92</v>
       </c>
-      <c r="F23" s="155"/>
+      <c r="F23" s="122"/>
       <c r="G23" s="14" t="s">
         <v>89</v>
       </c>
@@ -29924,35 +29471,35 @@
         <f>H23*I23</f>
         <v>4500000</v>
       </c>
-      <c r="K23" s="73"/>
-      <c r="L23" s="70"/>
-      <c r="M23" s="71"/>
-      <c r="N23" s="71"/>
-      <c r="O23" s="71"/>
-      <c r="P23" s="71"/>
-      <c r="Q23" s="71"/>
+      <c r="K23" s="65"/>
+      <c r="L23" s="62"/>
+      <c r="M23" s="63"/>
+      <c r="N23" s="63"/>
+      <c r="O23" s="63"/>
+      <c r="P23" s="63"/>
+      <c r="Q23" s="63"/>
     </row>
     <row r="24" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="78"/>
-      <c r="B24" s="44">
+      <c r="A24" s="70"/>
+      <c r="B24" s="40">
         <v>40</v>
       </c>
-      <c r="C24" s="154" t="s">
+      <c r="C24" s="121" t="s">
         <v>31</v>
       </c>
-      <c r="D24" s="154"/>
-      <c r="E24" s="154" t="s">
+      <c r="D24" s="121"/>
+      <c r="E24" s="121" t="s">
         <v>86</v>
       </c>
-      <c r="F24" s="154"/>
-      <c r="G24" s="45"/>
-      <c r="H24" s="45"/>
-      <c r="I24" s="46"/>
-      <c r="J24" s="47">
+      <c r="F24" s="121"/>
+      <c r="G24" s="41"/>
+      <c r="H24" s="41"/>
+      <c r="I24" s="42"/>
+      <c r="J24" s="43">
         <f>SUM(J25:J26)</f>
         <v>16500000</v>
       </c>
-      <c r="K24" s="73"/>
+      <c r="K24" s="65"/>
       <c r="L24" s="128" t="str">
         <f>"직접비 "&amp;TEXT($J$33,"#,##0")&amp;"원 기준"</f>
         <v>직접비 98,250,000원 기준</v>
@@ -29964,18 +29511,18 @@
       <c r="Q24" s="129"/>
     </row>
     <row r="25" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="78"/>
+      <c r="A25" s="70"/>
       <c r="B25" s="18">
         <v>40.01</v>
       </c>
-      <c r="C25" s="155" t="s">
+      <c r="C25" s="122" t="s">
         <v>96</v>
       </c>
-      <c r="D25" s="155"/>
-      <c r="E25" s="155" t="s">
+      <c r="D25" s="122"/>
+      <c r="E25" s="122" t="s">
         <v>88</v>
       </c>
-      <c r="F25" s="155"/>
+      <c r="F25" s="122"/>
       <c r="G25" s="14" t="s">
         <v>89</v>
       </c>
@@ -29990,27 +29537,27 @@
         <f>H25*I25</f>
         <v>12000000</v>
       </c>
-      <c r="K25" s="73"/>
-      <c r="L25" s="70"/>
-      <c r="M25" s="71"/>
-      <c r="N25" s="71"/>
-      <c r="O25" s="71"/>
-      <c r="P25" s="71"/>
-      <c r="Q25" s="71"/>
+      <c r="K25" s="65"/>
+      <c r="L25" s="62"/>
+      <c r="M25" s="63"/>
+      <c r="N25" s="63"/>
+      <c r="O25" s="63"/>
+      <c r="P25" s="63"/>
+      <c r="Q25" s="63"/>
     </row>
     <row r="26" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="78"/>
+      <c r="A26" s="70"/>
       <c r="B26" s="18">
         <v>40.020000000000003</v>
       </c>
-      <c r="C26" s="155" t="s">
+      <c r="C26" s="122" t="s">
         <v>97</v>
       </c>
-      <c r="D26" s="155"/>
-      <c r="E26" s="155" t="s">
+      <c r="D26" s="122"/>
+      <c r="E26" s="122" t="s">
         <v>92</v>
       </c>
-      <c r="F26" s="155"/>
+      <c r="F26" s="122"/>
       <c r="G26" s="14" t="s">
         <v>89</v>
       </c>
@@ -30025,57 +29572,57 @@
         <f>H26*I26</f>
         <v>4500000</v>
       </c>
-      <c r="K26" s="73"/>
-      <c r="L26" s="70"/>
-      <c r="M26" s="71"/>
-      <c r="N26" s="71"/>
-      <c r="O26" s="71"/>
-      <c r="P26" s="71"/>
-      <c r="Q26" s="71"/>
+      <c r="K26" s="65"/>
+      <c r="L26" s="62"/>
+      <c r="M26" s="63"/>
+      <c r="N26" s="63"/>
+      <c r="O26" s="63"/>
+      <c r="P26" s="63"/>
+      <c r="Q26" s="63"/>
     </row>
     <row r="27" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="78"/>
-      <c r="B27" s="44">
+      <c r="A27" s="70"/>
+      <c r="B27" s="40">
         <v>50</v>
       </c>
-      <c r="C27" s="154" t="s">
+      <c r="C27" s="121" t="s">
         <v>33</v>
       </c>
-      <c r="D27" s="154"/>
-      <c r="E27" s="154" t="s">
+      <c r="D27" s="121"/>
+      <c r="E27" s="121" t="s">
         <v>86</v>
       </c>
-      <c r="F27" s="154"/>
-      <c r="G27" s="45"/>
-      <c r="H27" s="45"/>
-      <c r="I27" s="46"/>
-      <c r="J27" s="47">
+      <c r="F27" s="121"/>
+      <c r="G27" s="41"/>
+      <c r="H27" s="41"/>
+      <c r="I27" s="42"/>
+      <c r="J27" s="43">
         <f>SUM(J28:J28)</f>
         <v>8000000</v>
       </c>
-      <c r="K27" s="73"/>
-      <c r="L27" s="136" t="s">
+      <c r="K27" s="65"/>
+      <c r="L27" s="131" t="s">
         <v>98</v>
       </c>
-      <c r="M27" s="137"/>
-      <c r="N27" s="137"/>
-      <c r="O27" s="137"/>
-      <c r="P27" s="137"/>
-      <c r="Q27" s="137"/>
+      <c r="M27" s="132"/>
+      <c r="N27" s="132"/>
+      <c r="O27" s="132"/>
+      <c r="P27" s="132"/>
+      <c r="Q27" s="132"/>
     </row>
     <row r="28" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="78"/>
+      <c r="A28" s="70"/>
       <c r="B28" s="18">
         <v>50.01</v>
       </c>
-      <c r="C28" s="155" t="s">
+      <c r="C28" s="122" t="s">
         <v>99</v>
       </c>
-      <c r="D28" s="155"/>
-      <c r="E28" s="155" t="s">
+      <c r="D28" s="122"/>
+      <c r="E28" s="122" t="s">
         <v>88</v>
       </c>
-      <c r="F28" s="155"/>
+      <c r="F28" s="122"/>
       <c r="G28" s="14" t="s">
         <v>89</v>
       </c>
@@ -30090,60 +29637,60 @@
         <f>H28*I28</f>
         <v>8000000</v>
       </c>
-      <c r="K28" s="73"/>
-      <c r="L28" s="70"/>
-      <c r="M28" s="71"/>
-      <c r="N28" s="71"/>
-      <c r="O28" s="71"/>
-      <c r="P28" s="71"/>
-      <c r="Q28" s="71"/>
+      <c r="K28" s="65"/>
+      <c r="L28" s="62"/>
+      <c r="M28" s="63"/>
+      <c r="N28" s="63"/>
+      <c r="O28" s="63"/>
+      <c r="P28" s="63"/>
+      <c r="Q28" s="63"/>
     </row>
     <row r="29" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="78"/>
-      <c r="B29" s="44">
+      <c r="A29" s="70"/>
+      <c r="B29" s="40">
         <v>60</v>
       </c>
-      <c r="C29" s="154" t="s">
+      <c r="C29" s="121" t="s">
         <v>35</v>
       </c>
-      <c r="D29" s="154"/>
-      <c r="E29" s="154" t="s">
+      <c r="D29" s="121"/>
+      <c r="E29" s="121" t="s">
         <v>100</v>
       </c>
-      <c r="F29" s="154"/>
-      <c r="G29" s="45"/>
-      <c r="H29" s="45"/>
-      <c r="I29" s="46"/>
-      <c r="J29" s="47">
+      <c r="F29" s="121"/>
+      <c r="G29" s="41"/>
+      <c r="H29" s="41"/>
+      <c r="I29" s="42"/>
+      <c r="J29" s="43">
         <f>SUM(J30:J32)</f>
         <v>7000000</v>
       </c>
-      <c r="K29" s="73"/>
+      <c r="K29" s="65"/>
       <c r="L29" s="128" t="s">
         <v>101</v>
       </c>
       <c r="M29" s="129"/>
       <c r="N29" s="129"/>
       <c r="O29" s="129"/>
-      <c r="P29" s="138">
+      <c r="P29" s="130">
         <f>$J$18/SUM($J$18,$J$21,$J$24,$J$27)</f>
         <v>0.2</v>
       </c>
-      <c r="Q29" s="138"/>
+      <c r="Q29" s="130"/>
     </row>
     <row r="30" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="78"/>
+      <c r="A30" s="70"/>
       <c r="B30" s="19">
         <v>60.01</v>
       </c>
-      <c r="C30" s="159" t="s">
+      <c r="C30" s="124" t="s">
         <v>102</v>
       </c>
-      <c r="D30" s="159"/>
-      <c r="E30" s="159" t="s">
+      <c r="D30" s="124"/>
+      <c r="E30" s="124" t="s">
         <v>103</v>
       </c>
-      <c r="F30" s="159"/>
+      <c r="F30" s="124"/>
       <c r="G30" s="11" t="s">
         <v>79</v>
       </c>
@@ -30157,32 +29704,32 @@
         <f>H30*I30</f>
         <v>3000000</v>
       </c>
-      <c r="K30" s="73"/>
-      <c r="L30" s="130" t="s">
+      <c r="K30" s="65"/>
+      <c r="L30" s="150" t="s">
         <v>104</v>
       </c>
-      <c r="M30" s="131"/>
-      <c r="N30" s="131"/>
-      <c r="O30" s="131"/>
-      <c r="P30" s="132">
+      <c r="M30" s="151"/>
+      <c r="N30" s="151"/>
+      <c r="O30" s="151"/>
+      <c r="P30" s="152">
         <f>$J$21/SUM($J$18,$J$21,$J$24,$J$27)</f>
         <v>0.32195121951219513</v>
       </c>
-      <c r="Q30" s="132"/>
+      <c r="Q30" s="152"/>
     </row>
     <row r="31" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="78"/>
+      <c r="A31" s="70"/>
       <c r="B31" s="18">
         <v>60.02</v>
       </c>
-      <c r="C31" s="157" t="s">
+      <c r="C31" s="125" t="s">
         <v>105</v>
       </c>
-      <c r="D31" s="157"/>
-      <c r="E31" s="157" t="s">
+      <c r="D31" s="125"/>
+      <c r="E31" s="125" t="s">
         <v>103</v>
       </c>
-      <c r="F31" s="157"/>
+      <c r="F31" s="125"/>
       <c r="G31" s="14" t="s">
         <v>79</v>
       </c>
@@ -30196,32 +29743,32 @@
         <f>H31*I31</f>
         <v>2000000</v>
       </c>
-      <c r="K31" s="73"/>
-      <c r="L31" s="130" t="s">
+      <c r="K31" s="65"/>
+      <c r="L31" s="150" t="s">
         <v>106</v>
       </c>
-      <c r="M31" s="131"/>
-      <c r="N31" s="131"/>
-      <c r="O31" s="131"/>
-      <c r="P31" s="132">
+      <c r="M31" s="151"/>
+      <c r="N31" s="151"/>
+      <c r="O31" s="151"/>
+      <c r="P31" s="152">
         <f>$J$24/SUM($J$18,$J$21,$J$24,$J$27)</f>
         <v>0.32195121951219513</v>
       </c>
-      <c r="Q31" s="132"/>
+      <c r="Q31" s="152"/>
     </row>
     <row r="32" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="78"/>
+      <c r="A32" s="70"/>
       <c r="B32" s="18">
         <v>60.03</v>
       </c>
-      <c r="C32" s="157" t="s">
+      <c r="C32" s="125" t="s">
         <v>107</v>
       </c>
-      <c r="D32" s="157"/>
-      <c r="E32" s="157" t="s">
+      <c r="D32" s="125"/>
+      <c r="E32" s="125" t="s">
         <v>103</v>
       </c>
-      <c r="F32" s="157"/>
+      <c r="F32" s="125"/>
       <c r="G32" s="14" t="s">
         <v>79</v>
       </c>
@@ -30235,86 +29782,86 @@
         <f>H32*I32</f>
         <v>2000000</v>
       </c>
-      <c r="K32" s="73"/>
-      <c r="L32" s="133" t="s">
+      <c r="K32" s="65"/>
+      <c r="L32" s="153" t="s">
         <v>108</v>
       </c>
-      <c r="M32" s="134"/>
-      <c r="N32" s="134"/>
-      <c r="O32" s="134"/>
-      <c r="P32" s="135">
+      <c r="M32" s="154"/>
+      <c r="N32" s="154"/>
+      <c r="O32" s="154"/>
+      <c r="P32" s="155">
         <f>$J$27/SUM($J$18,$J$21,$J$24,$J$27)</f>
         <v>0.15609756097560976</v>
       </c>
-      <c r="Q32" s="135"/>
+      <c r="Q32" s="155"/>
     </row>
     <row r="33" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="78"/>
-      <c r="B33" s="56" t="s">
+      <c r="A33" s="70"/>
+      <c r="B33" s="48" t="s">
         <v>109</v>
       </c>
-      <c r="C33" s="162" t="s">
+      <c r="C33" s="120" t="s">
         <v>110</v>
       </c>
-      <c r="D33" s="162"/>
-      <c r="E33" s="162"/>
-      <c r="F33" s="162"/>
-      <c r="G33" s="57"/>
-      <c r="H33" s="57"/>
-      <c r="I33" s="58"/>
-      <c r="J33" s="59">
+      <c r="D33" s="120"/>
+      <c r="E33" s="120"/>
+      <c r="F33" s="120"/>
+      <c r="G33" s="49"/>
+      <c r="H33" s="49"/>
+      <c r="I33" s="50"/>
+      <c r="J33" s="51">
         <f>SUM(J11,J18,J21,J24,J27,J29)</f>
         <v>98250000</v>
       </c>
-      <c r="K33" s="73"/>
-      <c r="L33" s="70"/>
-      <c r="M33" s="71"/>
-      <c r="N33" s="71"/>
-      <c r="O33" s="71"/>
-      <c r="P33" s="71"/>
-      <c r="Q33" s="71"/>
+      <c r="K33" s="65"/>
+      <c r="L33" s="62"/>
+      <c r="M33" s="63"/>
+      <c r="N33" s="63"/>
+      <c r="O33" s="63"/>
+      <c r="P33" s="63"/>
+      <c r="Q33" s="63"/>
     </row>
     <row r="34" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="78"/>
-      <c r="B34" s="44">
+      <c r="A34" s="70"/>
+      <c r="B34" s="40">
         <v>70</v>
       </c>
-      <c r="C34" s="154" t="s">
+      <c r="C34" s="121" t="s">
         <v>37</v>
       </c>
-      <c r="D34" s="154"/>
-      <c r="E34" s="154" t="s">
+      <c r="D34" s="121"/>
+      <c r="E34" s="121" t="s">
         <v>111</v>
       </c>
-      <c r="F34" s="154"/>
-      <c r="G34" s="45"/>
-      <c r="H34" s="45"/>
-      <c r="I34" s="46"/>
-      <c r="J34" s="47">
+      <c r="F34" s="121"/>
+      <c r="G34" s="41"/>
+      <c r="H34" s="41"/>
+      <c r="I34" s="42"/>
+      <c r="J34" s="43">
         <f>SUM(J35:J36)</f>
         <v>12133875</v>
       </c>
-      <c r="K34" s="73"/>
-      <c r="L34" s="70"/>
-      <c r="M34" s="71"/>
-      <c r="N34" s="71"/>
-      <c r="O34" s="71"/>
-      <c r="P34" s="71"/>
-      <c r="Q34" s="71"/>
+      <c r="K34" s="65"/>
+      <c r="L34" s="62"/>
+      <c r="M34" s="63"/>
+      <c r="N34" s="63"/>
+      <c r="O34" s="63"/>
+      <c r="P34" s="63"/>
+      <c r="Q34" s="63"/>
     </row>
     <row r="35" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="78"/>
+      <c r="A35" s="70"/>
       <c r="B35" s="15">
         <v>70.010000000000005</v>
       </c>
-      <c r="C35" s="155" t="s">
+      <c r="C35" s="122" t="s">
         <v>112</v>
       </c>
-      <c r="D35" s="155"/>
-      <c r="E35" s="155" t="s">
+      <c r="D35" s="122"/>
+      <c r="E35" s="122" t="s">
         <v>113</v>
       </c>
-      <c r="F35" s="155"/>
+      <c r="F35" s="122"/>
       <c r="G35" s="14" t="s">
         <v>114</v>
       </c>
@@ -30326,7 +29873,7 @@
         <f>ROUND(J33*H35,0)</f>
         <v>4912500</v>
       </c>
-      <c r="K35" s="73"/>
+      <c r="K35" s="65"/>
       <c r="L35" s="128" t="s">
         <v>115</v>
       </c>
@@ -30337,18 +29884,18 @@
       <c r="Q35" s="129"/>
     </row>
     <row r="36" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="78"/>
+      <c r="A36" s="70"/>
       <c r="B36" s="15">
         <v>70.02</v>
       </c>
-      <c r="C36" s="155" t="s">
+      <c r="C36" s="122" t="s">
         <v>116</v>
       </c>
-      <c r="D36" s="155"/>
-      <c r="E36" s="155" t="s">
+      <c r="D36" s="122"/>
+      <c r="E36" s="122" t="s">
         <v>117</v>
       </c>
-      <c r="F36" s="155"/>
+      <c r="F36" s="122"/>
       <c r="G36" s="14" t="s">
         <v>114</v>
       </c>
@@ -30360,7 +29907,7 @@
         <f>ROUND((J33+J35)*H36,0)</f>
         <v>7221375</v>
       </c>
-      <c r="K36" s="73"/>
+      <c r="K36" s="65"/>
       <c r="L36" s="128" t="str">
         <f>"하드웨어·인건비 비중  "&amp;TEXT(($J$11+SUM($J$18,$J$21,$J$24,$J$27))/$J$33,"0.0%")</f>
         <v>하드웨어·인건비 비중  92.9%</v>
@@ -30372,24 +29919,24 @@
       <c r="Q36" s="129"/>
     </row>
     <row r="37" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="78"/>
-      <c r="B37" s="60" t="s">
+      <c r="A37" s="70"/>
+      <c r="B37" s="52" t="s">
         <v>118</v>
       </c>
-      <c r="C37" s="160" t="s">
+      <c r="C37" s="123" t="s">
         <v>65</v>
       </c>
-      <c r="D37" s="160"/>
-      <c r="E37" s="160"/>
-      <c r="F37" s="160"/>
-      <c r="G37" s="61"/>
-      <c r="H37" s="61"/>
-      <c r="I37" s="62"/>
-      <c r="J37" s="63">
+      <c r="D37" s="123"/>
+      <c r="E37" s="123"/>
+      <c r="F37" s="123"/>
+      <c r="G37" s="53"/>
+      <c r="H37" s="53"/>
+      <c r="I37" s="54"/>
+      <c r="J37" s="55">
         <f>SUM(J33,J34)</f>
         <v>110383875</v>
       </c>
-      <c r="K37" s="73"/>
+      <c r="K37" s="65"/>
       <c r="L37" s="128"/>
       <c r="M37" s="129"/>
       <c r="N37" s="129"/>
@@ -30398,25 +29945,25 @@
       <c r="Q37" s="129"/>
     </row>
     <row r="38" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="78"/>
-      <c r="B38" s="66" t="s">
+      <c r="A38" s="70"/>
+      <c r="B38" s="58" t="s">
         <v>39</v>
       </c>
-      <c r="C38" s="161" t="s">
+      <c r="C38" s="119" t="s">
         <v>40</v>
       </c>
-      <c r="D38" s="161"/>
-      <c r="E38" s="161" t="s">
+      <c r="D38" s="119"/>
+      <c r="E38" s="119" t="s">
         <v>119</v>
       </c>
-      <c r="F38" s="161"/>
-      <c r="G38" s="64"/>
-      <c r="H38" s="64"/>
-      <c r="I38" s="65"/>
-      <c r="J38" s="67">
+      <c r="F38" s="119"/>
+      <c r="G38" s="56"/>
+      <c r="H38" s="56"/>
+      <c r="I38" s="57"/>
+      <c r="J38" s="59">
         <v>-875</v>
       </c>
-      <c r="K38" s="73"/>
+      <c r="K38" s="65"/>
       <c r="L38" s="128" t="str">
         <f>"직접비  "&amp;TEXT($J$33/$J$37,"0.0%")&amp;"  |  관리·이윤  "&amp;TEXT($J$34/$J$37,"0.0%")</f>
         <v>직접비  89.0%  |  관리·이윤  11.0%</v>
@@ -30428,51 +29975,51 @@
       <c r="Q38" s="129"/>
     </row>
     <row r="39" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="78"/>
-      <c r="B39" s="66" t="s">
+      <c r="A39" s="70"/>
+      <c r="B39" s="58" t="s">
         <v>42</v>
       </c>
-      <c r="C39" s="161" t="s">
+      <c r="C39" s="119" t="s">
         <v>43</v>
       </c>
-      <c r="D39" s="161"/>
-      <c r="E39" s="161" t="s">
+      <c r="D39" s="119"/>
+      <c r="E39" s="119" t="s">
         <v>120</v>
       </c>
-      <c r="F39" s="161"/>
-      <c r="G39" s="64"/>
-      <c r="H39" s="64"/>
-      <c r="I39" s="65"/>
-      <c r="J39" s="67">
+      <c r="F39" s="119"/>
+      <c r="G39" s="56"/>
+      <c r="H39" s="56"/>
+      <c r="I39" s="57"/>
+      <c r="J39" s="59">
         <v>-10383000</v>
       </c>
-      <c r="K39" s="73"/>
-      <c r="L39" s="70"/>
-      <c r="M39" s="71"/>
-      <c r="N39" s="71"/>
-      <c r="O39" s="71"/>
-      <c r="P39" s="71"/>
-      <c r="Q39" s="71"/>
+      <c r="K39" s="65"/>
+      <c r="L39" s="62"/>
+      <c r="M39" s="63"/>
+      <c r="N39" s="63"/>
+      <c r="O39" s="63"/>
+      <c r="P39" s="63"/>
+      <c r="Q39" s="63"/>
     </row>
     <row r="40" spans="1:17" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="78"/>
-      <c r="B40" s="48" t="s">
+      <c r="A40" s="70"/>
+      <c r="B40" s="212" t="s">
         <v>121</v>
       </c>
-      <c r="C40" s="170" t="s">
+      <c r="C40" s="213" t="s">
         <v>122</v>
       </c>
-      <c r="D40" s="170"/>
-      <c r="E40" s="170"/>
-      <c r="F40" s="170"/>
-      <c r="G40" s="49"/>
-      <c r="H40" s="49"/>
-      <c r="I40" s="50"/>
-      <c r="J40" s="51">
+      <c r="D40" s="213"/>
+      <c r="E40" s="213"/>
+      <c r="F40" s="213"/>
+      <c r="G40" s="214"/>
+      <c r="H40" s="214"/>
+      <c r="I40" s="215"/>
+      <c r="J40" s="216">
         <f>SUM(J37:J39)</f>
         <v>100000000</v>
       </c>
-      <c r="K40" s="73"/>
+      <c r="K40" s="65"/>
       <c r="L40" s="128" t="s">
         <v>123</v>
       </c>
@@ -30483,24 +30030,24 @@
       <c r="Q40" s="129"/>
     </row>
     <row r="41" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="78"/>
-      <c r="B41" s="21" t="s">
+      <c r="A41" s="70"/>
+      <c r="B41" s="207" t="s">
         <v>124</v>
       </c>
-      <c r="C41" s="171" t="s">
+      <c r="C41" s="208" t="s">
         <v>48</v>
       </c>
-      <c r="D41" s="171"/>
-      <c r="E41" s="171"/>
-      <c r="F41" s="171"/>
-      <c r="G41" s="22"/>
-      <c r="H41" s="22"/>
-      <c r="I41" s="23"/>
-      <c r="J41" s="24">
+      <c r="D41" s="208"/>
+      <c r="E41" s="208"/>
+      <c r="F41" s="208"/>
+      <c r="G41" s="209"/>
+      <c r="H41" s="209"/>
+      <c r="I41" s="210"/>
+      <c r="J41" s="211">
         <f>ROUND(J40*1.1,0)</f>
         <v>110000000</v>
       </c>
-      <c r="K41" s="73"/>
+      <c r="K41" s="65"/>
       <c r="L41" s="9"/>
       <c r="M41" s="9"/>
       <c r="N41" s="9"/>
@@ -30509,7 +30056,7 @@
       <c r="Q41" s="9"/>
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A42" s="78"/>
+      <c r="A42" s="70"/>
       <c r="B42" s="9"/>
       <c r="C42" s="9"/>
       <c r="D42" s="9"/>
@@ -30519,7 +30066,7 @@
       <c r="H42" s="9"/>
       <c r="I42" s="9"/>
       <c r="J42" s="9"/>
-      <c r="K42" s="73"/>
+      <c r="K42" s="65"/>
       <c r="L42" s="9"/>
       <c r="M42" s="9"/>
       <c r="N42" s="9"/>
@@ -30528,19 +30075,19 @@
       <c r="Q42" s="9"/>
     </row>
     <row r="43" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="78"/>
-      <c r="B43" s="169" t="s">
+      <c r="A43" s="70"/>
+      <c r="B43" s="118" t="s">
         <v>57</v>
       </c>
-      <c r="C43" s="169"/>
-      <c r="D43" s="169"/>
-      <c r="E43" s="169"/>
-      <c r="F43" s="169"/>
-      <c r="G43" s="169"/>
-      <c r="H43" s="169"/>
-      <c r="I43" s="169"/>
-      <c r="J43" s="169"/>
-      <c r="K43" s="73"/>
+      <c r="C43" s="118"/>
+      <c r="D43" s="118"/>
+      <c r="E43" s="118"/>
+      <c r="F43" s="118"/>
+      <c r="G43" s="118"/>
+      <c r="H43" s="118"/>
+      <c r="I43" s="118"/>
+      <c r="J43" s="118"/>
+      <c r="K43" s="65"/>
       <c r="L43" s="9"/>
       <c r="M43" s="9"/>
       <c r="N43" s="9"/>
@@ -30549,7 +30096,7 @@
       <c r="Q43" s="9"/>
     </row>
     <row r="44" spans="1:17" ht="266.10000000000002" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="78"/>
+      <c r="A44" s="70"/>
       <c r="B44" s="9"/>
       <c r="C44" s="9"/>
       <c r="D44" s="9"/>
@@ -30559,7 +30106,7 @@
       <c r="H44" s="9"/>
       <c r="I44" s="9"/>
       <c r="J44" s="9"/>
-      <c r="K44" s="73"/>
+      <c r="K44" s="65"/>
       <c r="L44" s="9"/>
       <c r="M44" s="9"/>
       <c r="N44" s="9"/>
@@ -30568,21 +30115,21 @@
       <c r="Q44" s="9"/>
     </row>
     <row r="45" spans="1:17" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="80"/>
-      <c r="B45" s="163" t="s">
+      <c r="A45" s="72"/>
+      <c r="B45" s="112" t="s">
         <v>58</v>
       </c>
-      <c r="C45" s="164"/>
-      <c r="D45" s="164"/>
-      <c r="E45" s="164"/>
-      <c r="F45" s="164"/>
-      <c r="G45" s="166" t="s">
+      <c r="C45" s="113"/>
+      <c r="D45" s="113"/>
+      <c r="E45" s="113"/>
+      <c r="F45" s="113"/>
+      <c r="G45" s="115" t="s">
         <v>59</v>
       </c>
-      <c r="H45" s="167"/>
-      <c r="I45" s="167"/>
-      <c r="J45" s="167"/>
-      <c r="K45" s="81"/>
+      <c r="H45" s="116"/>
+      <c r="I45" s="116"/>
+      <c r="J45" s="116"/>
+      <c r="K45" s="73"/>
       <c r="L45" s="9"/>
       <c r="M45" s="9"/>
       <c r="N45" s="9"/>
@@ -30591,17 +30138,17 @@
       <c r="Q45" s="9"/>
     </row>
     <row r="46" spans="1:17" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="82"/>
-      <c r="B46" s="165"/>
-      <c r="C46" s="165"/>
-      <c r="D46" s="165"/>
-      <c r="E46" s="165"/>
-      <c r="F46" s="165"/>
-      <c r="G46" s="168"/>
-      <c r="H46" s="168"/>
-      <c r="I46" s="168"/>
-      <c r="J46" s="168"/>
-      <c r="K46" s="83"/>
+      <c r="A46" s="74"/>
+      <c r="B46" s="114"/>
+      <c r="C46" s="114"/>
+      <c r="D46" s="114"/>
+      <c r="E46" s="114"/>
+      <c r="F46" s="114"/>
+      <c r="G46" s="117"/>
+      <c r="H46" s="117"/>
+      <c r="I46" s="117"/>
+      <c r="J46" s="117"/>
+      <c r="K46" s="75"/>
       <c r="L46" s="9"/>
       <c r="M46" s="9"/>
       <c r="N46" s="9"/>
@@ -30610,17 +30157,17 @@
       <c r="Q46" s="9"/>
     </row>
     <row r="47" spans="1:17" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="82"/>
-      <c r="B47" s="165"/>
-      <c r="C47" s="165"/>
-      <c r="D47" s="165"/>
-      <c r="E47" s="165"/>
-      <c r="F47" s="165"/>
-      <c r="G47" s="168"/>
-      <c r="H47" s="168"/>
-      <c r="I47" s="168"/>
-      <c r="J47" s="168"/>
-      <c r="K47" s="83"/>
+      <c r="A47" s="74"/>
+      <c r="B47" s="114"/>
+      <c r="C47" s="114"/>
+      <c r="D47" s="114"/>
+      <c r="E47" s="114"/>
+      <c r="F47" s="114"/>
+      <c r="G47" s="117"/>
+      <c r="H47" s="117"/>
+      <c r="I47" s="117"/>
+      <c r="J47" s="117"/>
+      <c r="K47" s="75"/>
       <c r="L47" s="9"/>
       <c r="M47" s="9"/>
       <c r="N47" s="9"/>
@@ -32304,74 +31851,24 @@
     </row>
   </sheetData>
   <mergeCells count="102">
-    <mergeCell ref="B45:F47"/>
-    <mergeCell ref="G45:J47"/>
-    <mergeCell ref="B43:J43"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="E37:F37"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="L12:O12"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="L14:Q14"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="L16:M16"/>
-    <mergeCell ref="N16:P16"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="N19:P19"/>
+    <mergeCell ref="L22:M22"/>
+    <mergeCell ref="N22:P22"/>
+    <mergeCell ref="L24:Q24"/>
+    <mergeCell ref="L38:Q38"/>
+    <mergeCell ref="L27:Q27"/>
+    <mergeCell ref="L29:O29"/>
+    <mergeCell ref="P29:Q29"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="L40:Q40"/>
+    <mergeCell ref="L30:O30"/>
+    <mergeCell ref="P30:Q30"/>
+    <mergeCell ref="L31:O31"/>
+    <mergeCell ref="P31:Q31"/>
+    <mergeCell ref="L32:O32"/>
+    <mergeCell ref="P32:Q32"/>
+    <mergeCell ref="L35:Q35"/>
+    <mergeCell ref="L36:Q37"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="L5:Q5"/>
@@ -32388,28 +31885,78 @@
     <mergeCell ref="G8:J8"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="L40:Q40"/>
-    <mergeCell ref="L30:O30"/>
-    <mergeCell ref="P30:Q30"/>
-    <mergeCell ref="L31:O31"/>
-    <mergeCell ref="P31:Q31"/>
-    <mergeCell ref="L32:O32"/>
-    <mergeCell ref="P32:Q32"/>
-    <mergeCell ref="L35:Q35"/>
-    <mergeCell ref="L36:Q37"/>
-    <mergeCell ref="N19:P19"/>
-    <mergeCell ref="L22:M22"/>
-    <mergeCell ref="N22:P22"/>
-    <mergeCell ref="L24:Q24"/>
-    <mergeCell ref="L38:Q38"/>
-    <mergeCell ref="L27:Q27"/>
-    <mergeCell ref="L29:O29"/>
-    <mergeCell ref="P29:Q29"/>
-    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="L12:O12"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="L14:Q14"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="L16:M16"/>
+    <mergeCell ref="N16:P16"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="B45:F47"/>
+    <mergeCell ref="G45:J47"/>
+    <mergeCell ref="B43:J43"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="E41:F41"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="73" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -32433,14 +31980,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="8.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="25"/>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
+      <c r="A1" s="21"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="8"/>
@@ -32454,36 +32001,36 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="8"/>
-      <c r="B3" s="172" t="s">
+      <c r="B3" s="156" t="s">
         <v>125</v>
       </c>
-      <c r="C3" s="172"/>
-      <c r="D3" s="172"/>
-      <c r="E3" s="172"/>
-      <c r="F3" s="172"/>
-      <c r="G3" s="172"/>
+      <c r="C3" s="156"/>
+      <c r="D3" s="156"/>
+      <c r="E3" s="156"/>
+      <c r="F3" s="156"/>
+      <c r="G3" s="156"/>
       <c r="H3" s="8"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="8"/>
-      <c r="B4" s="172"/>
-      <c r="C4" s="172"/>
-      <c r="D4" s="172"/>
-      <c r="E4" s="172"/>
-      <c r="F4" s="172"/>
-      <c r="G4" s="172"/>
+      <c r="B4" s="156"/>
+      <c r="C4" s="156"/>
+      <c r="D4" s="156"/>
+      <c r="E4" s="156"/>
+      <c r="F4" s="156"/>
+      <c r="G4" s="156"/>
       <c r="H4" s="8"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="8"/>
-      <c r="B5" s="173" t="s">
+      <c r="B5" s="157" t="s">
         <v>126</v>
       </c>
-      <c r="C5" s="173"/>
-      <c r="D5" s="173"/>
-      <c r="E5" s="173"/>
-      <c r="F5" s="173"/>
-      <c r="G5" s="173"/>
+      <c r="C5" s="157"/>
+      <c r="D5" s="157"/>
+      <c r="E5" s="157"/>
+      <c r="F5" s="157"/>
+      <c r="G5" s="157"/>
       <c r="H5" s="8"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -32498,22 +32045,22 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="8"/>
-      <c r="B7" s="26" t="s">
+      <c r="B7" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="C7" s="26" t="s">
+      <c r="C7" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="E7" s="26" t="s">
+      <c r="E7" s="22" t="s">
         <v>128</v>
       </c>
-      <c r="F7" s="26" t="s">
+      <c r="F7" s="22" t="s">
         <v>129</v>
       </c>
-      <c r="G7" s="26" t="s">
+      <c r="G7" s="22" t="s">
         <v>130</v>
       </c>
       <c r="H7" s="8"/>
@@ -32530,88 +32077,88 @@
     </row>
     <row r="9" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="8"/>
-      <c r="B9" s="27" t="s">
+      <c r="B9" s="23" t="s">
         <v>131</v>
       </c>
-      <c r="C9" s="27" t="s">
+      <c r="C9" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="D9" s="27" t="s">
+      <c r="D9" s="23" t="s">
         <v>133</v>
       </c>
-      <c r="E9" s="27" t="s">
+      <c r="E9" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="F9" s="27" t="s">
+      <c r="F9" s="23" t="s">
         <v>135</v>
       </c>
-      <c r="G9" s="27" t="s">
+      <c r="G9" s="23" t="s">
         <v>136</v>
       </c>
       <c r="H9" s="8"/>
     </row>
     <row r="10" spans="1:8" ht="26.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8"/>
-      <c r="B10" s="37" t="s">
+      <c r="B10" s="33" t="s">
         <v>137</v>
       </c>
-      <c r="C10" s="28">
+      <c r="C10" s="24">
         <v>35</v>
       </c>
-      <c r="D10" s="29">
+      <c r="D10" s="25">
         <v>350000</v>
       </c>
-      <c r="E10" s="30" t="s">
+      <c r="E10" s="26" t="s">
         <v>138</v>
       </c>
-      <c r="F10" s="30" t="s">
+      <c r="F10" s="26" t="s">
         <v>139</v>
       </c>
-      <c r="G10" s="30" t="s">
+      <c r="G10" s="26" t="s">
         <v>140</v>
       </c>
       <c r="H10" s="8"/>
     </row>
     <row r="11" spans="1:8" ht="26.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="8"/>
-      <c r="B11" s="38" t="s">
+      <c r="B11" s="34" t="s">
         <v>141</v>
       </c>
-      <c r="C11" s="31">
+      <c r="C11" s="27">
         <v>40</v>
       </c>
-      <c r="D11" s="32">
+      <c r="D11" s="28">
         <v>400000</v>
       </c>
-      <c r="E11" s="33" t="s">
+      <c r="E11" s="29" t="s">
         <v>142</v>
       </c>
-      <c r="F11" s="33" t="s">
+      <c r="F11" s="29" t="s">
         <v>143</v>
       </c>
-      <c r="G11" s="33" t="s">
+      <c r="G11" s="29" t="s">
         <v>140</v>
       </c>
       <c r="H11" s="8"/>
     </row>
     <row r="12" spans="1:8" ht="26.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="8"/>
-      <c r="B12" s="39" t="s">
+      <c r="B12" s="35" t="s">
         <v>144</v>
       </c>
-      <c r="C12" s="34">
+      <c r="C12" s="30">
         <v>45</v>
       </c>
-      <c r="D12" s="35">
+      <c r="D12" s="31">
         <v>450000</v>
       </c>
-      <c r="E12" s="36" t="s">
+      <c r="E12" s="32" t="s">
         <v>145</v>
       </c>
-      <c r="F12" s="36" t="s">
+      <c r="F12" s="32" t="s">
         <v>146</v>
       </c>
-      <c r="G12" s="36" t="s">
+      <c r="G12" s="32" t="s">
         <v>140</v>
       </c>
       <c r="H12" s="8"/>
@@ -32638,34 +32185,34 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="8"/>
-      <c r="B15" s="174" t="s">
+      <c r="B15" s="158" t="s">
         <v>147</v>
       </c>
-      <c r="C15" s="175"/>
-      <c r="D15" s="175"/>
-      <c r="E15" s="175"/>
-      <c r="F15" s="175"/>
-      <c r="G15" s="176"/>
+      <c r="C15" s="159"/>
+      <c r="D15" s="159"/>
+      <c r="E15" s="159"/>
+      <c r="F15" s="159"/>
+      <c r="G15" s="160"/>
       <c r="H15" s="8"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="8"/>
-      <c r="B16" s="177"/>
-      <c r="C16" s="178"/>
-      <c r="D16" s="178"/>
-      <c r="E16" s="178"/>
-      <c r="F16" s="178"/>
-      <c r="G16" s="179"/>
+      <c r="B16" s="161"/>
+      <c r="C16" s="162"/>
+      <c r="D16" s="162"/>
+      <c r="E16" s="162"/>
+      <c r="F16" s="162"/>
+      <c r="G16" s="163"/>
       <c r="H16" s="8"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="8"/>
-      <c r="B17" s="180"/>
-      <c r="C17" s="181"/>
-      <c r="D17" s="181"/>
-      <c r="E17" s="181"/>
-      <c r="F17" s="181"/>
-      <c r="G17" s="182"/>
+      <c r="B17" s="164"/>
+      <c r="C17" s="165"/>
+      <c r="D17" s="165"/>
+      <c r="E17" s="165"/>
+      <c r="F17" s="165"/>
+      <c r="G17" s="166"/>
       <c r="H17" s="8"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
@@ -32720,36 +32267,36 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="8"/>
-      <c r="B23" s="183" t="s">
+      <c r="B23" s="167" t="s">
         <v>148</v>
       </c>
-      <c r="C23" s="183"/>
-      <c r="D23" s="183"/>
-      <c r="E23" s="185" t="s">
+      <c r="C23" s="167"/>
+      <c r="D23" s="167"/>
+      <c r="E23" s="169" t="s">
         <v>149</v>
       </c>
-      <c r="F23" s="185"/>
-      <c r="G23" s="185"/>
+      <c r="F23" s="169"/>
+      <c r="G23" s="169"/>
       <c r="H23" s="8"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="8"/>
-      <c r="B24" s="184"/>
-      <c r="C24" s="184"/>
-      <c r="D24" s="184"/>
-      <c r="E24" s="186"/>
-      <c r="F24" s="186"/>
-      <c r="G24" s="186"/>
+      <c r="B24" s="168"/>
+      <c r="C24" s="168"/>
+      <c r="D24" s="168"/>
+      <c r="E24" s="170"/>
+      <c r="F24" s="170"/>
+      <c r="G24" s="170"/>
       <c r="H24" s="8"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="8"/>
-      <c r="B25" s="184"/>
-      <c r="C25" s="184"/>
-      <c r="D25" s="184"/>
-      <c r="E25" s="186"/>
-      <c r="F25" s="186"/>
-      <c r="G25" s="186"/>
+      <c r="B25" s="168"/>
+      <c r="C25" s="168"/>
+      <c r="D25" s="168"/>
+      <c r="E25" s="170"/>
+      <c r="F25" s="170"/>
+      <c r="G25" s="170"/>
       <c r="H25" s="8"/>
     </row>
   </sheetData>
@@ -32763,6 +32310,6 @@
   <phoneticPr fontId="17" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="85" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix quote code header rendering
</commit_message>
<xml_diff>
--- a/Codex Plugins/plugins/dhandy-excel-quote-template/skills/artifact-template-dhandy/assets/reference.xlsx
+++ b/Codex Plugins/plugins/dhandy-excel-quote-template/skills/artifact-template-dhandy/assets/reference.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kookie\Documents\견적 업무\tmp\quote_template_line_fix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74270C47-C043-4004-8539-44C4DB423C82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA202889-66E9-402E-82C3-A4F8E3D34D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -103,9 +103,6 @@
   </si>
   <si>
     <t>KRW / VAT EXCLUDED</t>
-  </si>
-  <si>
-    <t>코드</t>
   </si>
   <si>
     <t>항목</t>
@@ -493,6 +490,10 @@
   </si>
   <si>
     <t>INTERNAL RATE STANDARD</t>
+  </si>
+  <si>
+    <t>CODE</t>
+    <phoneticPr fontId="17" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1388,17 +1389,170 @@
     <xf numFmtId="0" fontId="9" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="21" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="21" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="16" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="38" fontId="16" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="38" fontId="16" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="38" fontId="14" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="38" fontId="14" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="38" fontId="20" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="38" fontId="23" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="33" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="38" fontId="23" fillId="21" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
@@ -1433,110 +1587,11 @@
     <xf numFmtId="0" fontId="15" fillId="11" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="12" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="16" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1544,20 +1599,32 @@
     <xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="16" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="16" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="16" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1604,23 +1671,59 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="4" fillId="16" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="4" fillId="16" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
@@ -1694,78 +1797,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="21" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="20" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="33" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="23" fillId="21" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="23" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="21" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="26" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
@@ -1774,36 +1805,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="16" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="16" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="16" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="14" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="14" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="14" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -27928,12 +27929,12 @@
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
-      <c r="H5" s="100" t="s">
+      <c r="H5" s="102" t="s">
         <v>0</v>
       </c>
-      <c r="I5" s="100"/>
-      <c r="J5" s="100"/>
-      <c r="K5" s="100"/>
+      <c r="I5" s="102"/>
+      <c r="J5" s="102"/>
+      <c r="K5" s="102"/>
       <c r="L5" s="3"/>
     </row>
     <row r="6" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.3">
@@ -27944,12 +27945,12 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
-      <c r="H6" s="101" t="s">
+      <c r="H6" s="103" t="s">
         <v>1</v>
       </c>
-      <c r="I6" s="101"/>
-      <c r="J6" s="101"/>
-      <c r="K6" s="101"/>
+      <c r="I6" s="103"/>
+      <c r="J6" s="103"/>
+      <c r="K6" s="103"/>
       <c r="L6" s="3"/>
     </row>
     <row r="7" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.3">
@@ -27960,12 +27961,12 @@
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
-      <c r="H7" s="102" t="s">
+      <c r="H7" s="104" t="s">
         <v>2</v>
       </c>
-      <c r="I7" s="102"/>
-      <c r="J7" s="102"/>
-      <c r="K7" s="102"/>
+      <c r="I7" s="104"/>
+      <c r="J7" s="104"/>
+      <c r="K7" s="104"/>
       <c r="L7" s="3"/>
     </row>
     <row r="8" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -27984,79 +27985,79 @@
     </row>
     <row r="9" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
-      <c r="B9" s="104" t="s">
+      <c r="B9" s="106" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="104"/>
-      <c r="D9" s="104"/>
-      <c r="E9" s="104"/>
-      <c r="F9" s="104"/>
-      <c r="G9" s="104"/>
-      <c r="H9" s="104"/>
-      <c r="I9" s="104"/>
-      <c r="J9" s="104"/>
-      <c r="K9" s="104"/>
-      <c r="L9" s="104"/>
+      <c r="C9" s="106"/>
+      <c r="D9" s="106"/>
+      <c r="E9" s="106"/>
+      <c r="F9" s="106"/>
+      <c r="G9" s="106"/>
+      <c r="H9" s="106"/>
+      <c r="I9" s="106"/>
+      <c r="J9" s="106"/>
+      <c r="K9" s="106"/>
+      <c r="L9" s="106"/>
     </row>
     <row r="10" spans="1:13" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
-      <c r="B10" s="104"/>
-      <c r="C10" s="104"/>
-      <c r="D10" s="104"/>
-      <c r="E10" s="104"/>
-      <c r="F10" s="104"/>
-      <c r="G10" s="104"/>
-      <c r="H10" s="104"/>
-      <c r="I10" s="104"/>
-      <c r="J10" s="104"/>
-      <c r="K10" s="104"/>
-      <c r="L10" s="104"/>
+      <c r="B10" s="106"/>
+      <c r="C10" s="106"/>
+      <c r="D10" s="106"/>
+      <c r="E10" s="106"/>
+      <c r="F10" s="106"/>
+      <c r="G10" s="106"/>
+      <c r="H10" s="106"/>
+      <c r="I10" s="106"/>
+      <c r="J10" s="106"/>
+      <c r="K10" s="106"/>
+      <c r="L10" s="106"/>
     </row>
     <row r="11" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
-      <c r="B11" s="105" t="s">
+      <c r="B11" s="107" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="105"/>
-      <c r="D11" s="105"/>
-      <c r="E11" s="105"/>
-      <c r="F11" s="105"/>
-      <c r="G11" s="105"/>
-      <c r="H11" s="105"/>
-      <c r="I11" s="105"/>
-      <c r="J11" s="105"/>
-      <c r="K11" s="105"/>
-      <c r="L11" s="105"/>
+      <c r="C11" s="107"/>
+      <c r="D11" s="107"/>
+      <c r="E11" s="107"/>
+      <c r="F11" s="107"/>
+      <c r="G11" s="107"/>
+      <c r="H11" s="107"/>
+      <c r="I11" s="107"/>
+      <c r="J11" s="107"/>
+      <c r="K11" s="107"/>
+      <c r="L11" s="107"/>
     </row>
     <row r="12" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3"/>
-      <c r="B12" s="103" t="s">
+      <c r="B12" s="105" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="103"/>
-      <c r="D12" s="103"/>
-      <c r="E12" s="103"/>
-      <c r="F12" s="103"/>
-      <c r="G12" s="103"/>
-      <c r="H12" s="103"/>
-      <c r="I12" s="103"/>
-      <c r="J12" s="103"/>
-      <c r="K12" s="103"/>
-      <c r="L12" s="103"/>
+      <c r="C12" s="105"/>
+      <c r="D12" s="105"/>
+      <c r="E12" s="105"/>
+      <c r="F12" s="105"/>
+      <c r="G12" s="105"/>
+      <c r="H12" s="105"/>
+      <c r="I12" s="105"/>
+      <c r="J12" s="105"/>
+      <c r="K12" s="105"/>
+      <c r="L12" s="105"/>
     </row>
     <row r="13" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3"/>
-      <c r="B13" s="103"/>
-      <c r="C13" s="103"/>
-      <c r="D13" s="103"/>
-      <c r="E13" s="103"/>
-      <c r="F13" s="103"/>
-      <c r="G13" s="103"/>
-      <c r="H13" s="103"/>
-      <c r="I13" s="103"/>
-      <c r="J13" s="103"/>
-      <c r="K13" s="103"/>
-      <c r="L13" s="103"/>
+      <c r="B13" s="105"/>
+      <c r="C13" s="105"/>
+      <c r="D13" s="105"/>
+      <c r="E13" s="105"/>
+      <c r="F13" s="105"/>
+      <c r="G13" s="105"/>
+      <c r="H13" s="105"/>
+      <c r="I13" s="105"/>
+      <c r="J13" s="105"/>
+      <c r="K13" s="105"/>
+      <c r="L13" s="105"/>
     </row>
     <row r="14" spans="1:13" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3"/>
@@ -28074,53 +28075,53 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="36"/>
-      <c r="B15" s="95" t="s">
+      <c r="B15" s="108" t="s">
         <v>6</v>
       </c>
-      <c r="C15" s="95"/>
-      <c r="D15" s="95"/>
-      <c r="E15" s="95"/>
-      <c r="F15" s="95"/>
-      <c r="G15" s="95" t="s">
+      <c r="C15" s="108"/>
+      <c r="D15" s="108"/>
+      <c r="E15" s="108"/>
+      <c r="F15" s="108"/>
+      <c r="G15" s="108" t="s">
         <v>7</v>
       </c>
-      <c r="H15" s="95"/>
-      <c r="I15" s="95"/>
-      <c r="J15" s="95"/>
-      <c r="K15" s="95"/>
-      <c r="L15" s="95"/>
+      <c r="H15" s="108"/>
+      <c r="I15" s="108"/>
+      <c r="J15" s="108"/>
+      <c r="K15" s="108"/>
+      <c r="L15" s="108"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="36"/>
-      <c r="B16" s="98" t="s">
+      <c r="B16" s="111" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="98"/>
-      <c r="D16" s="98"/>
-      <c r="E16" s="98"/>
-      <c r="F16" s="98"/>
-      <c r="G16" s="98" t="s">
+      <c r="C16" s="111"/>
+      <c r="D16" s="111"/>
+      <c r="E16" s="111"/>
+      <c r="F16" s="111"/>
+      <c r="G16" s="111" t="s">
         <v>9</v>
       </c>
-      <c r="H16" s="98"/>
-      <c r="I16" s="98"/>
-      <c r="J16" s="98"/>
-      <c r="K16" s="98"/>
-      <c r="L16" s="98"/>
+      <c r="H16" s="111"/>
+      <c r="I16" s="111"/>
+      <c r="J16" s="111"/>
+      <c r="K16" s="111"/>
+      <c r="L16" s="111"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="36"/>
-      <c r="B17" s="99"/>
-      <c r="C17" s="99"/>
-      <c r="D17" s="99"/>
-      <c r="E17" s="99"/>
-      <c r="F17" s="99"/>
-      <c r="G17" s="99"/>
-      <c r="H17" s="99"/>
-      <c r="I17" s="99"/>
-      <c r="J17" s="99"/>
-      <c r="K17" s="99"/>
-      <c r="L17" s="99"/>
+      <c r="B17" s="112"/>
+      <c r="C17" s="112"/>
+      <c r="D17" s="112"/>
+      <c r="E17" s="112"/>
+      <c r="F17" s="112"/>
+      <c r="G17" s="112"/>
+      <c r="H17" s="112"/>
+      <c r="I17" s="112"/>
+      <c r="J17" s="112"/>
+      <c r="K17" s="112"/>
+      <c r="L17" s="112"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="36"/>
@@ -28138,393 +28139,393 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="36"/>
-      <c r="B19" s="95" t="s">
+      <c r="B19" s="108" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="95"/>
-      <c r="D19" s="95"/>
-      <c r="E19" s="95"/>
-      <c r="F19" s="95"/>
-      <c r="G19" s="95" t="s">
+      <c r="C19" s="108"/>
+      <c r="D19" s="108"/>
+      <c r="E19" s="108"/>
+      <c r="F19" s="108"/>
+      <c r="G19" s="108" t="s">
         <v>11</v>
       </c>
-      <c r="H19" s="95"/>
-      <c r="I19" s="95"/>
-      <c r="J19" s="95"/>
-      <c r="K19" s="95"/>
-      <c r="L19" s="95"/>
+      <c r="H19" s="108"/>
+      <c r="I19" s="108"/>
+      <c r="J19" s="108"/>
+      <c r="K19" s="108"/>
+      <c r="L19" s="108"/>
     </row>
     <row r="20" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="36"/>
-      <c r="B20" s="96" t="s">
+      <c r="B20" s="109" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="96"/>
-      <c r="D20" s="96"/>
-      <c r="E20" s="96"/>
-      <c r="F20" s="96"/>
+      <c r="C20" s="109"/>
+      <c r="D20" s="109"/>
+      <c r="E20" s="109"/>
+      <c r="F20" s="109"/>
       <c r="G20" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="H20" s="96" t="s">
+      <c r="H20" s="109" t="s">
         <v>14</v>
       </c>
-      <c r="I20" s="96"/>
-      <c r="J20" s="96"/>
-      <c r="K20" s="96"/>
-      <c r="L20" s="96"/>
+      <c r="I20" s="109"/>
+      <c r="J20" s="109"/>
+      <c r="K20" s="109"/>
+      <c r="L20" s="109"/>
     </row>
     <row r="21" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="36"/>
-      <c r="B21" s="96"/>
-      <c r="C21" s="96"/>
-      <c r="D21" s="96"/>
-      <c r="E21" s="96"/>
-      <c r="F21" s="96"/>
+      <c r="B21" s="109"/>
+      <c r="C21" s="109"/>
+      <c r="D21" s="109"/>
+      <c r="E21" s="109"/>
+      <c r="F21" s="109"/>
       <c r="G21" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="H21" s="96" t="s">
+      <c r="H21" s="109" t="s">
         <v>16</v>
       </c>
-      <c r="I21" s="96"/>
-      <c r="J21" s="96"/>
-      <c r="K21" s="96"/>
-      <c r="L21" s="96"/>
+      <c r="I21" s="109"/>
+      <c r="J21" s="109"/>
+      <c r="K21" s="109"/>
+      <c r="L21" s="109"/>
     </row>
     <row r="22" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="36"/>
-      <c r="B22" s="97"/>
-      <c r="C22" s="97"/>
-      <c r="D22" s="97"/>
-      <c r="E22" s="97"/>
-      <c r="F22" s="97"/>
+      <c r="B22" s="110"/>
+      <c r="C22" s="110"/>
+      <c r="D22" s="110"/>
+      <c r="E22" s="110"/>
+      <c r="F22" s="110"/>
       <c r="G22" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="H22" s="97" t="s">
+      <c r="H22" s="110" t="s">
         <v>18</v>
       </c>
-      <c r="I22" s="97"/>
-      <c r="J22" s="97"/>
-      <c r="K22" s="97"/>
-      <c r="L22" s="97"/>
+      <c r="I22" s="110"/>
+      <c r="J22" s="110"/>
+      <c r="K22" s="110"/>
+      <c r="L22" s="110"/>
     </row>
     <row r="23" spans="1:12" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="93" t="s">
+      <c r="B23" s="119" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="93"/>
-      <c r="D23" s="93"/>
-      <c r="E23" s="93"/>
-      <c r="F23" s="93"/>
-      <c r="G23" s="93"/>
-      <c r="H23" s="93"/>
-      <c r="I23" s="94" t="s">
+      <c r="C23" s="119"/>
+      <c r="D23" s="119"/>
+      <c r="E23" s="119"/>
+      <c r="F23" s="119"/>
+      <c r="G23" s="119"/>
+      <c r="H23" s="119"/>
+      <c r="I23" s="120" t="s">
         <v>20</v>
       </c>
-      <c r="J23" s="94"/>
-      <c r="K23" s="94"/>
-      <c r="L23" s="94"/>
+      <c r="J23" s="120"/>
+      <c r="K23" s="120"/>
+      <c r="L23" s="120"/>
     </row>
     <row r="24" spans="1:12" ht="23.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="204" t="s">
+      <c r="B24" s="214" t="s">
+        <v>149</v>
+      </c>
+      <c r="C24" s="214"/>
+      <c r="D24" s="215" t="s">
         <v>21</v>
       </c>
-      <c r="C24" s="204"/>
-      <c r="D24" s="205" t="s">
+      <c r="E24" s="216"/>
+      <c r="F24" s="216"/>
+      <c r="G24" s="215" t="s">
         <v>22</v>
       </c>
-      <c r="E24" s="206"/>
-      <c r="F24" s="206"/>
-      <c r="G24" s="205" t="s">
+      <c r="H24" s="216"/>
+      <c r="I24" s="216"/>
+      <c r="J24" s="215" t="s">
         <v>23</v>
       </c>
-      <c r="H24" s="206"/>
-      <c r="I24" s="206"/>
-      <c r="J24" s="205" t="s">
+      <c r="K24" s="216"/>
+      <c r="L24" s="216"/>
+    </row>
+    <row r="25" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="206">
+        <v>10</v>
+      </c>
+      <c r="C25" s="207"/>
+      <c r="D25" s="208" t="s">
         <v>24</v>
       </c>
-      <c r="K24" s="206"/>
-      <c r="L24" s="206"/>
-    </row>
-    <row r="25" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="172">
-        <v>10</v>
-      </c>
-      <c r="C25" s="173"/>
-      <c r="D25" s="174" t="s">
+      <c r="E25" s="209"/>
+      <c r="F25" s="209"/>
+      <c r="G25" s="210" t="s">
         <v>25</v>
       </c>
-      <c r="E25" s="175"/>
-      <c r="F25" s="175"/>
-      <c r="G25" s="176" t="s">
-        <v>26</v>
-      </c>
-      <c r="H25" s="177"/>
-      <c r="I25" s="177"/>
-      <c r="J25" s="178">
+      <c r="H25" s="211"/>
+      <c r="I25" s="211"/>
+      <c r="J25" s="212">
         <f>'2. 상세견적'!J11</f>
         <v>40000000</v>
       </c>
-      <c r="K25" s="179"/>
-      <c r="L25" s="179"/>
+      <c r="K25" s="213"/>
+      <c r="L25" s="213"/>
     </row>
     <row r="26" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="180">
+      <c r="B26" s="78">
         <v>20</v>
       </c>
-      <c r="C26" s="181"/>
-      <c r="D26" s="182" t="s">
+      <c r="C26" s="79"/>
+      <c r="D26" s="113" t="s">
+        <v>26</v>
+      </c>
+      <c r="E26" s="114"/>
+      <c r="F26" s="114"/>
+      <c r="G26" s="115" t="s">
         <v>27</v>
       </c>
-      <c r="E26" s="183"/>
-      <c r="F26" s="183"/>
-      <c r="G26" s="184" t="s">
-        <v>28</v>
-      </c>
-      <c r="H26" s="185"/>
-      <c r="I26" s="185"/>
-      <c r="J26" s="186">
+      <c r="H26" s="116"/>
+      <c r="I26" s="116"/>
+      <c r="J26" s="117">
         <f>'2. 상세견적'!J18</f>
         <v>10250000</v>
       </c>
-      <c r="K26" s="187"/>
-      <c r="L26" s="187"/>
+      <c r="K26" s="118"/>
+      <c r="L26" s="118"/>
     </row>
     <row r="27" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="180">
+      <c r="B27" s="78">
         <v>30</v>
       </c>
-      <c r="C27" s="181"/>
-      <c r="D27" s="182" t="s">
+      <c r="C27" s="79"/>
+      <c r="D27" s="113" t="s">
+        <v>28</v>
+      </c>
+      <c r="E27" s="114"/>
+      <c r="F27" s="114"/>
+      <c r="G27" s="115" t="s">
         <v>29</v>
       </c>
-      <c r="E27" s="183"/>
-      <c r="F27" s="183"/>
-      <c r="G27" s="184" t="s">
-        <v>30</v>
-      </c>
-      <c r="H27" s="185"/>
-      <c r="I27" s="185"/>
-      <c r="J27" s="186">
+      <c r="H27" s="116"/>
+      <c r="I27" s="116"/>
+      <c r="J27" s="117">
         <f>'2. 상세견적'!J21</f>
         <v>16500000</v>
       </c>
-      <c r="K27" s="187"/>
-      <c r="L27" s="187"/>
+      <c r="K27" s="118"/>
+      <c r="L27" s="118"/>
     </row>
     <row r="28" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="180">
+      <c r="B28" s="78">
         <v>40</v>
       </c>
-      <c r="C28" s="181"/>
-      <c r="D28" s="182" t="s">
+      <c r="C28" s="79"/>
+      <c r="D28" s="113" t="s">
+        <v>30</v>
+      </c>
+      <c r="E28" s="114"/>
+      <c r="F28" s="114"/>
+      <c r="G28" s="115" t="s">
         <v>31</v>
       </c>
-      <c r="E28" s="183"/>
-      <c r="F28" s="183"/>
-      <c r="G28" s="184" t="s">
-        <v>32</v>
-      </c>
-      <c r="H28" s="185"/>
-      <c r="I28" s="185"/>
-      <c r="J28" s="186">
+      <c r="H28" s="116"/>
+      <c r="I28" s="116"/>
+      <c r="J28" s="117">
         <f>'2. 상세견적'!J24</f>
         <v>16500000</v>
       </c>
-      <c r="K28" s="187"/>
-      <c r="L28" s="187"/>
+      <c r="K28" s="118"/>
+      <c r="L28" s="118"/>
     </row>
     <row r="29" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="180">
+      <c r="B29" s="78">
         <v>50</v>
       </c>
-      <c r="C29" s="181"/>
-      <c r="D29" s="182" t="s">
+      <c r="C29" s="79"/>
+      <c r="D29" s="113" t="s">
+        <v>32</v>
+      </c>
+      <c r="E29" s="114"/>
+      <c r="F29" s="114"/>
+      <c r="G29" s="115" t="s">
         <v>33</v>
       </c>
-      <c r="E29" s="183"/>
-      <c r="F29" s="183"/>
-      <c r="G29" s="184" t="s">
-        <v>34</v>
-      </c>
-      <c r="H29" s="185"/>
-      <c r="I29" s="185"/>
-      <c r="J29" s="186">
+      <c r="H29" s="116"/>
+      <c r="I29" s="116"/>
+      <c r="J29" s="117">
         <f>'2. 상세견적'!J27</f>
         <v>8000000</v>
       </c>
-      <c r="K29" s="187"/>
-      <c r="L29" s="187"/>
+      <c r="K29" s="118"/>
+      <c r="L29" s="118"/>
     </row>
     <row r="30" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="180">
+      <c r="B30" s="78">
         <v>60</v>
       </c>
-      <c r="C30" s="181"/>
-      <c r="D30" s="182" t="s">
+      <c r="C30" s="79"/>
+      <c r="D30" s="113" t="s">
+        <v>34</v>
+      </c>
+      <c r="E30" s="114"/>
+      <c r="F30" s="114"/>
+      <c r="G30" s="115" t="s">
         <v>35</v>
       </c>
-      <c r="E30" s="183"/>
-      <c r="F30" s="183"/>
-      <c r="G30" s="184" t="s">
-        <v>36</v>
-      </c>
-      <c r="H30" s="185"/>
-      <c r="I30" s="185"/>
-      <c r="J30" s="186">
+      <c r="H30" s="116"/>
+      <c r="I30" s="116"/>
+      <c r="J30" s="117">
         <f>'2. 상세견적'!J29</f>
         <v>7000000</v>
       </c>
-      <c r="K30" s="187"/>
-      <c r="L30" s="187"/>
+      <c r="K30" s="118"/>
+      <c r="L30" s="118"/>
     </row>
     <row r="31" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="180">
+      <c r="B31" s="78">
         <v>70</v>
       </c>
-      <c r="C31" s="181"/>
-      <c r="D31" s="182" t="s">
+      <c r="C31" s="79"/>
+      <c r="D31" s="113" t="s">
+        <v>36</v>
+      </c>
+      <c r="E31" s="114"/>
+      <c r="F31" s="114"/>
+      <c r="G31" s="115" t="s">
         <v>37</v>
       </c>
-      <c r="E31" s="183"/>
-      <c r="F31" s="183"/>
-      <c r="G31" s="184" t="s">
-        <v>38</v>
-      </c>
-      <c r="H31" s="185"/>
-      <c r="I31" s="185"/>
-      <c r="J31" s="186">
+      <c r="H31" s="116"/>
+      <c r="I31" s="116"/>
+      <c r="J31" s="117">
         <f>'2. 상세견적'!J34</f>
         <v>12133875</v>
       </c>
-      <c r="K31" s="187"/>
-      <c r="L31" s="187"/>
+      <c r="K31" s="118"/>
+      <c r="L31" s="118"/>
     </row>
     <row r="32" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="200" t="s">
+      <c r="B32" s="80" t="s">
+        <v>38</v>
+      </c>
+      <c r="C32" s="81"/>
+      <c r="D32" s="121" t="s">
         <v>39</v>
       </c>
-      <c r="C32" s="201"/>
-      <c r="D32" s="194" t="s">
+      <c r="E32" s="122"/>
+      <c r="F32" s="122"/>
+      <c r="G32" s="123" t="s">
         <v>40</v>
       </c>
-      <c r="E32" s="195"/>
-      <c r="F32" s="195"/>
-      <c r="G32" s="196" t="s">
-        <v>41</v>
-      </c>
-      <c r="H32" s="197"/>
-      <c r="I32" s="197"/>
-      <c r="J32" s="198">
+      <c r="H32" s="124"/>
+      <c r="I32" s="124"/>
+      <c r="J32" s="125">
         <f>'2. 상세견적'!J38</f>
         <v>-875</v>
       </c>
-      <c r="K32" s="199"/>
-      <c r="L32" s="199"/>
+      <c r="K32" s="126"/>
+      <c r="L32" s="126"/>
     </row>
     <row r="33" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="202" t="s">
+      <c r="B33" s="82" t="s">
+        <v>41</v>
+      </c>
+      <c r="C33" s="83"/>
+      <c r="D33" s="127" t="s">
         <v>42</v>
       </c>
-      <c r="C33" s="203"/>
-      <c r="D33" s="188" t="s">
+      <c r="E33" s="128"/>
+      <c r="F33" s="128"/>
+      <c r="G33" s="129" t="s">
         <v>43</v>
       </c>
-      <c r="E33" s="189"/>
-      <c r="F33" s="189"/>
-      <c r="G33" s="190" t="s">
-        <v>44</v>
-      </c>
-      <c r="H33" s="191"/>
-      <c r="I33" s="191"/>
-      <c r="J33" s="192">
+      <c r="H33" s="130"/>
+      <c r="I33" s="130"/>
+      <c r="J33" s="131">
         <f>'2. 상세견적'!J39</f>
         <v>-10383000</v>
       </c>
-      <c r="K33" s="193"/>
-      <c r="L33" s="193"/>
+      <c r="K33" s="132"/>
+      <c r="L33" s="132"/>
     </row>
     <row r="34" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="171"/>
-      <c r="C34" s="171"/>
-      <c r="D34" s="171"/>
-      <c r="E34" s="171"/>
-      <c r="F34" s="171"/>
-      <c r="G34" s="171"/>
-      <c r="H34" s="171"/>
-      <c r="I34" s="171"/>
-      <c r="J34" s="171"/>
-      <c r="K34" s="171"/>
-      <c r="L34" s="171"/>
+      <c r="B34" s="205"/>
+      <c r="C34" s="205"/>
+      <c r="D34" s="205"/>
+      <c r="E34" s="205"/>
+      <c r="F34" s="205"/>
+      <c r="G34" s="205"/>
+      <c r="H34" s="205"/>
+      <c r="I34" s="205"/>
+      <c r="J34" s="205"/>
+      <c r="K34" s="205"/>
+      <c r="L34" s="205"/>
     </row>
     <row r="35" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="88" t="s">
-        <v>45</v>
+      <c r="B35" s="139" t="s">
+        <v>44</v>
       </c>
-      <c r="C35" s="88"/>
-      <c r="D35" s="88"/>
-      <c r="E35" s="88"/>
-      <c r="F35" s="88"/>
-      <c r="G35" s="90">
+      <c r="C35" s="139"/>
+      <c r="D35" s="139"/>
+      <c r="E35" s="139"/>
+      <c r="F35" s="139"/>
+      <c r="G35" s="141">
         <f>'2. 상세견적'!J40</f>
         <v>100000000</v>
       </c>
-      <c r="H35" s="91"/>
-      <c r="I35" s="91"/>
-      <c r="J35" s="91"/>
-      <c r="K35" s="91"/>
-      <c r="L35" s="91"/>
+      <c r="H35" s="142"/>
+      <c r="I35" s="142"/>
+      <c r="J35" s="142"/>
+      <c r="K35" s="142"/>
+      <c r="L35" s="142"/>
     </row>
     <row r="36" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="89"/>
-      <c r="C36" s="89"/>
-      <c r="D36" s="89"/>
-      <c r="E36" s="89"/>
-      <c r="F36" s="89"/>
-      <c r="G36" s="92"/>
-      <c r="H36" s="92"/>
-      <c r="I36" s="92"/>
-      <c r="J36" s="92"/>
-      <c r="K36" s="92"/>
-      <c r="L36" s="92"/>
+      <c r="B36" s="140"/>
+      <c r="C36" s="140"/>
+      <c r="D36" s="140"/>
+      <c r="E36" s="140"/>
+      <c r="F36" s="140"/>
+      <c r="G36" s="143"/>
+      <c r="H36" s="143"/>
+      <c r="I36" s="143"/>
+      <c r="J36" s="143"/>
+      <c r="K36" s="143"/>
+      <c r="L36" s="143"/>
     </row>
     <row r="37" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="85" t="s">
+      <c r="B37" s="136" t="s">
+        <v>45</v>
+      </c>
+      <c r="C37" s="136"/>
+      <c r="D37" s="136"/>
+      <c r="E37" s="136"/>
+      <c r="F37" s="136"/>
+      <c r="G37" s="137" t="s">
         <v>46</v>
       </c>
-      <c r="C37" s="85"/>
-      <c r="D37" s="85"/>
-      <c r="E37" s="85"/>
-      <c r="F37" s="85"/>
-      <c r="G37" s="86" t="s">
-        <v>47</v>
-      </c>
-      <c r="H37" s="87"/>
-      <c r="I37" s="87"/>
-      <c r="J37" s="87"/>
-      <c r="K37" s="87"/>
-      <c r="L37" s="87"/>
+      <c r="H37" s="138"/>
+      <c r="I37" s="138"/>
+      <c r="J37" s="138"/>
+      <c r="K37" s="138"/>
+      <c r="L37" s="138"/>
     </row>
     <row r="38" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="3"/>
-      <c r="B38" s="82" t="s">
-        <v>48</v>
+      <c r="B38" s="133" t="s">
+        <v>47</v>
       </c>
-      <c r="C38" s="82"/>
-      <c r="D38" s="82"/>
-      <c r="E38" s="82"/>
-      <c r="F38" s="82"/>
-      <c r="G38" s="83">
+      <c r="C38" s="133"/>
+      <c r="D38" s="133"/>
+      <c r="E38" s="133"/>
+      <c r="F38" s="133"/>
+      <c r="G38" s="134">
         <f>'2. 상세견적'!J41</f>
         <v>110000000</v>
       </c>
-      <c r="H38" s="84"/>
-      <c r="I38" s="84"/>
-      <c r="J38" s="84"/>
-      <c r="K38" s="84"/>
-      <c r="L38" s="84"/>
+      <c r="H38" s="135"/>
+      <c r="I38" s="135"/>
+      <c r="J38" s="135"/>
+      <c r="K38" s="135"/>
+      <c r="L38" s="135"/>
     </row>
     <row r="39" spans="1:13" ht="267.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="3"/>
@@ -28542,75 +28543,75 @@
     </row>
     <row r="40" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="3"/>
-      <c r="B40" s="80" t="s">
+      <c r="B40" s="98" t="s">
+        <v>48</v>
+      </c>
+      <c r="C40" s="99"/>
+      <c r="D40" s="99"/>
+      <c r="E40" s="99"/>
+      <c r="F40" s="99"/>
+      <c r="G40" s="98" t="s">
         <v>49</v>
       </c>
-      <c r="C40" s="81"/>
-      <c r="D40" s="81"/>
-      <c r="E40" s="81"/>
-      <c r="F40" s="81"/>
-      <c r="G40" s="80" t="s">
-        <v>50</v>
-      </c>
-      <c r="H40" s="81"/>
-      <c r="I40" s="81"/>
-      <c r="J40" s="81"/>
-      <c r="K40" s="81"/>
-      <c r="L40" s="81"/>
+      <c r="H40" s="99"/>
+      <c r="I40" s="99"/>
+      <c r="J40" s="99"/>
+      <c r="K40" s="99"/>
+      <c r="L40" s="99"/>
     </row>
     <row r="41" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="3"/>
-      <c r="B41" s="78" t="s">
+      <c r="B41" s="100" t="s">
+        <v>50</v>
+      </c>
+      <c r="C41" s="101"/>
+      <c r="D41" s="101"/>
+      <c r="E41" s="101"/>
+      <c r="F41" s="101"/>
+      <c r="G41" s="100" t="s">
         <v>51</v>
       </c>
-      <c r="C41" s="79"/>
-      <c r="D41" s="79"/>
-      <c r="E41" s="79"/>
-      <c r="F41" s="79"/>
-      <c r="G41" s="78" t="s">
-        <v>52</v>
-      </c>
-      <c r="H41" s="79"/>
-      <c r="I41" s="79"/>
-      <c r="J41" s="79"/>
-      <c r="K41" s="79"/>
-      <c r="L41" s="79"/>
+      <c r="H41" s="101"/>
+      <c r="I41" s="101"/>
+      <c r="J41" s="101"/>
+      <c r="K41" s="101"/>
+      <c r="L41" s="101"/>
     </row>
     <row r="42" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="3"/>
-      <c r="B42" s="80" t="s">
+      <c r="B42" s="98" t="s">
+        <v>52</v>
+      </c>
+      <c r="C42" s="99"/>
+      <c r="D42" s="99"/>
+      <c r="E42" s="99"/>
+      <c r="F42" s="99"/>
+      <c r="G42" s="98" t="s">
         <v>53</v>
       </c>
-      <c r="C42" s="81"/>
-      <c r="D42" s="81"/>
-      <c r="E42" s="81"/>
-      <c r="F42" s="81"/>
-      <c r="G42" s="80" t="s">
-        <v>54</v>
-      </c>
-      <c r="H42" s="81"/>
-      <c r="I42" s="81"/>
-      <c r="J42" s="81"/>
-      <c r="K42" s="81"/>
-      <c r="L42" s="81"/>
+      <c r="H42" s="99"/>
+      <c r="I42" s="99"/>
+      <c r="J42" s="99"/>
+      <c r="K42" s="99"/>
+      <c r="L42" s="99"/>
     </row>
     <row r="43" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="3"/>
-      <c r="B43" s="78" t="s">
+      <c r="B43" s="100" t="s">
+        <v>54</v>
+      </c>
+      <c r="C43" s="101"/>
+      <c r="D43" s="101"/>
+      <c r="E43" s="101"/>
+      <c r="F43" s="101"/>
+      <c r="G43" s="100" t="s">
         <v>55</v>
       </c>
-      <c r="C43" s="79"/>
-      <c r="D43" s="79"/>
-      <c r="E43" s="79"/>
-      <c r="F43" s="79"/>
-      <c r="G43" s="78" t="s">
-        <v>56</v>
-      </c>
-      <c r="H43" s="79"/>
-      <c r="I43" s="79"/>
-      <c r="J43" s="79"/>
-      <c r="K43" s="79"/>
-      <c r="L43" s="79"/>
+      <c r="H43" s="101"/>
+      <c r="I43" s="101"/>
+      <c r="J43" s="101"/>
+      <c r="K43" s="101"/>
+      <c r="L43" s="101"/>
     </row>
     <row r="44" spans="1:13" ht="6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="3"/>
@@ -28628,33 +28629,33 @@
     </row>
     <row r="45" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="3"/>
-      <c r="B45" s="106" t="s">
-        <v>57</v>
+      <c r="B45" s="92" t="s">
+        <v>56</v>
       </c>
-      <c r="C45" s="107"/>
-      <c r="D45" s="107"/>
-      <c r="E45" s="107"/>
-      <c r="F45" s="107"/>
-      <c r="G45" s="107"/>
-      <c r="H45" s="107"/>
-      <c r="I45" s="107"/>
-      <c r="J45" s="107"/>
-      <c r="K45" s="107"/>
-      <c r="L45" s="107"/>
+      <c r="C45" s="93"/>
+      <c r="D45" s="93"/>
+      <c r="E45" s="93"/>
+      <c r="F45" s="93"/>
+      <c r="G45" s="93"/>
+      <c r="H45" s="93"/>
+      <c r="I45" s="93"/>
+      <c r="J45" s="93"/>
+      <c r="K45" s="93"/>
+      <c r="L45" s="93"/>
     </row>
     <row r="46" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="3"/>
-      <c r="B46" s="107"/>
-      <c r="C46" s="107"/>
-      <c r="D46" s="107"/>
-      <c r="E46" s="107"/>
-      <c r="F46" s="107"/>
-      <c r="G46" s="107"/>
-      <c r="H46" s="107"/>
-      <c r="I46" s="107"/>
-      <c r="J46" s="107"/>
-      <c r="K46" s="107"/>
-      <c r="L46" s="107"/>
+      <c r="B46" s="93"/>
+      <c r="C46" s="93"/>
+      <c r="D46" s="93"/>
+      <c r="E46" s="93"/>
+      <c r="F46" s="93"/>
+      <c r="G46" s="93"/>
+      <c r="H46" s="93"/>
+      <c r="I46" s="93"/>
+      <c r="J46" s="93"/>
+      <c r="K46" s="93"/>
+      <c r="L46" s="93"/>
     </row>
     <row r="47" spans="1:13" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="3"/>
@@ -28672,107 +28673,55 @@
     </row>
     <row r="48" spans="1:13" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="68"/>
-      <c r="B48" s="108" t="s">
+      <c r="B48" s="94" t="s">
+        <v>57</v>
+      </c>
+      <c r="C48" s="94"/>
+      <c r="D48" s="94"/>
+      <c r="E48" s="94"/>
+      <c r="F48" s="94"/>
+      <c r="G48" s="96" t="s">
         <v>58</v>
       </c>
-      <c r="C48" s="108"/>
-      <c r="D48" s="108"/>
-      <c r="E48" s="108"/>
-      <c r="F48" s="108"/>
-      <c r="G48" s="110" t="s">
-        <v>59</v>
-      </c>
-      <c r="H48" s="110"/>
-      <c r="I48" s="110"/>
-      <c r="J48" s="110"/>
-      <c r="K48" s="110"/>
-      <c r="L48" s="110"/>
+      <c r="H48" s="96"/>
+      <c r="I48" s="96"/>
+      <c r="J48" s="96"/>
+      <c r="K48" s="96"/>
+      <c r="L48" s="96"/>
       <c r="M48" s="69"/>
     </row>
     <row r="49" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="67"/>
-      <c r="B49" s="109"/>
-      <c r="C49" s="109"/>
-      <c r="D49" s="109"/>
-      <c r="E49" s="109"/>
-      <c r="F49" s="109"/>
-      <c r="G49" s="111"/>
-      <c r="H49" s="111"/>
-      <c r="I49" s="111"/>
-      <c r="J49" s="111"/>
-      <c r="K49" s="111"/>
-      <c r="L49" s="111"/>
+      <c r="B49" s="95"/>
+      <c r="C49" s="95"/>
+      <c r="D49" s="95"/>
+      <c r="E49" s="95"/>
+      <c r="F49" s="95"/>
+      <c r="G49" s="97"/>
+      <c r="H49" s="97"/>
+      <c r="I49" s="97"/>
+      <c r="J49" s="97"/>
+      <c r="K49" s="97"/>
+      <c r="L49" s="97"/>
       <c r="M49" s="66"/>
     </row>
     <row r="50" spans="1:13" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="67"/>
-      <c r="B50" s="109"/>
-      <c r="C50" s="109"/>
-      <c r="D50" s="109"/>
-      <c r="E50" s="109"/>
-      <c r="F50" s="109"/>
-      <c r="G50" s="111"/>
-      <c r="H50" s="111"/>
-      <c r="I50" s="111"/>
-      <c r="J50" s="111"/>
-      <c r="K50" s="111"/>
-      <c r="L50" s="111"/>
+      <c r="B50" s="95"/>
+      <c r="C50" s="95"/>
+      <c r="D50" s="95"/>
+      <c r="E50" s="95"/>
+      <c r="F50" s="95"/>
+      <c r="G50" s="97"/>
+      <c r="H50" s="97"/>
+      <c r="I50" s="97"/>
+      <c r="J50" s="97"/>
+      <c r="K50" s="97"/>
+      <c r="L50" s="97"/>
       <c r="M50" s="66"/>
     </row>
   </sheetData>
   <mergeCells count="65">
-    <mergeCell ref="B45:L46"/>
-    <mergeCell ref="B48:F50"/>
-    <mergeCell ref="G48:L50"/>
-    <mergeCell ref="B42:F42"/>
-    <mergeCell ref="G42:L42"/>
-    <mergeCell ref="B43:F43"/>
-    <mergeCell ref="G43:L43"/>
-    <mergeCell ref="H5:K5"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="H7:K7"/>
-    <mergeCell ref="B12:L13"/>
-    <mergeCell ref="B9:L10"/>
-    <mergeCell ref="B11:L11"/>
-    <mergeCell ref="G19:L19"/>
-    <mergeCell ref="H20:L20"/>
-    <mergeCell ref="H21:L21"/>
-    <mergeCell ref="H22:L22"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="G15:L15"/>
-    <mergeCell ref="B16:F17"/>
-    <mergeCell ref="G16:L17"/>
-    <mergeCell ref="B19:F19"/>
-    <mergeCell ref="B20:F22"/>
-    <mergeCell ref="D26:F26"/>
-    <mergeCell ref="G26:I26"/>
-    <mergeCell ref="J26:L26"/>
-    <mergeCell ref="B23:H23"/>
-    <mergeCell ref="I23:L23"/>
-    <mergeCell ref="D24:F24"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="J24:L24"/>
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="G25:I25"/>
-    <mergeCell ref="J25:L25"/>
-    <mergeCell ref="D27:F27"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="J27:L27"/>
-    <mergeCell ref="D28:F28"/>
-    <mergeCell ref="G28:I28"/>
-    <mergeCell ref="J28:L28"/>
-    <mergeCell ref="D29:F29"/>
-    <mergeCell ref="G29:I29"/>
-    <mergeCell ref="J29:L29"/>
-    <mergeCell ref="D30:F30"/>
-    <mergeCell ref="G30:I30"/>
-    <mergeCell ref="J30:L30"/>
-    <mergeCell ref="D31:F31"/>
-    <mergeCell ref="G31:I31"/>
-    <mergeCell ref="J31:L31"/>
-    <mergeCell ref="D32:F32"/>
-    <mergeCell ref="G32:I32"/>
-    <mergeCell ref="J32:L32"/>
     <mergeCell ref="B41:F41"/>
     <mergeCell ref="G41:L41"/>
     <mergeCell ref="D33:F33"/>
@@ -28786,6 +28735,58 @@
     <mergeCell ref="G37:L37"/>
     <mergeCell ref="B35:F36"/>
     <mergeCell ref="G35:L36"/>
+    <mergeCell ref="D31:F31"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="J31:L31"/>
+    <mergeCell ref="D32:F32"/>
+    <mergeCell ref="G32:I32"/>
+    <mergeCell ref="J32:L32"/>
+    <mergeCell ref="D29:F29"/>
+    <mergeCell ref="G29:I29"/>
+    <mergeCell ref="J29:L29"/>
+    <mergeCell ref="D30:F30"/>
+    <mergeCell ref="G30:I30"/>
+    <mergeCell ref="J30:L30"/>
+    <mergeCell ref="D27:F27"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="J27:L27"/>
+    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="G28:I28"/>
+    <mergeCell ref="J28:L28"/>
+    <mergeCell ref="D26:F26"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="J26:L26"/>
+    <mergeCell ref="B23:H23"/>
+    <mergeCell ref="I23:L23"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="J24:L24"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="G25:I25"/>
+    <mergeCell ref="J25:L25"/>
+    <mergeCell ref="G19:L19"/>
+    <mergeCell ref="H20:L20"/>
+    <mergeCell ref="H21:L21"/>
+    <mergeCell ref="H22:L22"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="G15:L15"/>
+    <mergeCell ref="B16:F17"/>
+    <mergeCell ref="G16:L17"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B20:F22"/>
+    <mergeCell ref="H5:K5"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="B12:L13"/>
+    <mergeCell ref="B9:L10"/>
+    <mergeCell ref="B11:L11"/>
+    <mergeCell ref="B45:L46"/>
+    <mergeCell ref="B48:F50"/>
+    <mergeCell ref="G48:L50"/>
+    <mergeCell ref="B42:F42"/>
+    <mergeCell ref="G42:L42"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="G43:L43"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
@@ -28889,53 +28890,53 @@
     </row>
     <row r="5" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="70"/>
-      <c r="B5" s="144" t="s">
+      <c r="B5" s="166" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" s="166"/>
+      <c r="D5" s="166"/>
+      <c r="E5" s="166"/>
+      <c r="F5" s="166"/>
+      <c r="G5" s="168" t="s">
+        <v>1</v>
+      </c>
+      <c r="H5" s="168"/>
+      <c r="I5" s="168"/>
+      <c r="J5" s="168"/>
+      <c r="K5" s="65"/>
+      <c r="L5" s="158" t="s">
         <v>60</v>
       </c>
-      <c r="C5" s="144"/>
-      <c r="D5" s="144"/>
-      <c r="E5" s="144"/>
-      <c r="F5" s="144"/>
-      <c r="G5" s="146" t="s">
-        <v>1</v>
-      </c>
-      <c r="H5" s="146"/>
-      <c r="I5" s="146"/>
-      <c r="J5" s="146"/>
-      <c r="K5" s="65"/>
-      <c r="L5" s="136" t="s">
-        <v>61</v>
-      </c>
-      <c r="M5" s="137"/>
-      <c r="N5" s="137"/>
-      <c r="O5" s="137"/>
-      <c r="P5" s="137"/>
-      <c r="Q5" s="137"/>
+      <c r="M5" s="159"/>
+      <c r="N5" s="159"/>
+      <c r="O5" s="159"/>
+      <c r="P5" s="159"/>
+      <c r="Q5" s="159"/>
     </row>
     <row r="6" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="70"/>
-      <c r="B6" s="145" t="s">
+      <c r="B6" s="167" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="167"/>
+      <c r="D6" s="167"/>
+      <c r="E6" s="167"/>
+      <c r="F6" s="167"/>
+      <c r="G6" s="169" t="s">
+        <v>5</v>
+      </c>
+      <c r="H6" s="169"/>
+      <c r="I6" s="169"/>
+      <c r="J6" s="169"/>
+      <c r="K6" s="65"/>
+      <c r="L6" s="160" t="s">
         <v>62</v>
       </c>
-      <c r="C6" s="145"/>
-      <c r="D6" s="145"/>
-      <c r="E6" s="145"/>
-      <c r="F6" s="145"/>
-      <c r="G6" s="147" t="s">
-        <v>5</v>
-      </c>
-      <c r="H6" s="147"/>
-      <c r="I6" s="147"/>
-      <c r="J6" s="147"/>
-      <c r="K6" s="65"/>
-      <c r="L6" s="138" t="s">
-        <v>63</v>
-      </c>
-      <c r="M6" s="139"/>
-      <c r="N6" s="139"/>
-      <c r="O6" s="139"/>
-      <c r="P6" s="139"/>
-      <c r="Q6" s="139"/>
+      <c r="M6" s="161"/>
+      <c r="N6" s="161"/>
+      <c r="O6" s="161"/>
+      <c r="P6" s="161"/>
+      <c r="Q6" s="161"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" s="70"/>
@@ -28949,39 +28950,39 @@
       <c r="I7" s="10"/>
       <c r="J7" s="10"/>
       <c r="K7" s="65"/>
-      <c r="L7" s="138"/>
-      <c r="M7" s="139"/>
-      <c r="N7" s="139"/>
-      <c r="O7" s="139"/>
-      <c r="P7" s="139"/>
-      <c r="Q7" s="139"/>
+      <c r="L7" s="160"/>
+      <c r="M7" s="161"/>
+      <c r="N7" s="161"/>
+      <c r="O7" s="161"/>
+      <c r="P7" s="161"/>
+      <c r="Q7" s="161"/>
     </row>
     <row r="8" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="70"/>
-      <c r="B8" s="148" t="s">
+      <c r="B8" s="170" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="170"/>
+      <c r="D8" s="170"/>
+      <c r="E8" s="170"/>
+      <c r="F8" s="170"/>
+      <c r="G8" s="171" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" s="171"/>
+      <c r="I8" s="171"/>
+      <c r="J8" s="171"/>
+      <c r="K8" s="65"/>
+      <c r="L8" s="162" t="s">
         <v>64</v>
       </c>
-      <c r="C8" s="148"/>
-      <c r="D8" s="148"/>
-      <c r="E8" s="148"/>
-      <c r="F8" s="148"/>
-      <c r="G8" s="149" t="s">
-        <v>20</v>
-      </c>
-      <c r="H8" s="149"/>
-      <c r="I8" s="149"/>
-      <c r="J8" s="149"/>
-      <c r="K8" s="65"/>
-      <c r="L8" s="140" t="s">
+      <c r="M8" s="163"/>
+      <c r="N8" s="163"/>
+      <c r="O8" s="163" t="s">
         <v>65</v>
       </c>
-      <c r="M8" s="141"/>
-      <c r="N8" s="141"/>
-      <c r="O8" s="141" t="s">
-        <v>66</v>
-      </c>
-      <c r="P8" s="141"/>
-      <c r="Q8" s="141"/>
+      <c r="P8" s="163"/>
+      <c r="Q8" s="163"/>
     </row>
     <row r="9" spans="1:17" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="70"/>
@@ -28995,65 +28996,65 @@
       <c r="I9" s="10"/>
       <c r="J9" s="10"/>
       <c r="K9" s="65"/>
-      <c r="L9" s="142">
+      <c r="L9" s="164">
         <f>$J$37</f>
         <v>110383875</v>
       </c>
-      <c r="M9" s="143"/>
-      <c r="N9" s="143"/>
-      <c r="O9" s="143">
+      <c r="M9" s="165"/>
+      <c r="N9" s="165"/>
+      <c r="O9" s="165">
         <f>$J$40</f>
         <v>100000000</v>
       </c>
-      <c r="P9" s="143"/>
-      <c r="Q9" s="143"/>
+      <c r="P9" s="165"/>
+      <c r="Q9" s="165"/>
     </row>
     <row r="10" spans="1:17" ht="23.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="70"/>
       <c r="B10" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" s="157" t="s">
         <v>67</v>
       </c>
-      <c r="C10" s="135" t="s">
+      <c r="D10" s="157"/>
+      <c r="E10" s="157" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="135"/>
-      <c r="E10" s="135" t="s">
+      <c r="F10" s="157"/>
+      <c r="G10" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="F10" s="135"/>
-      <c r="G10" s="5" t="s">
+      <c r="H10" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="H10" s="6" t="s">
+      <c r="I10" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="I10" s="6" t="s">
-        <v>72</v>
-      </c>
       <c r="J10" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K10" s="65"/>
-      <c r="L10" s="142"/>
-      <c r="M10" s="143"/>
-      <c r="N10" s="143"/>
-      <c r="O10" s="143"/>
-      <c r="P10" s="143"/>
-      <c r="Q10" s="143"/>
+      <c r="L10" s="164"/>
+      <c r="M10" s="165"/>
+      <c r="N10" s="165"/>
+      <c r="O10" s="165"/>
+      <c r="P10" s="165"/>
+      <c r="Q10" s="165"/>
     </row>
     <row r="11" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="70"/>
       <c r="B11" s="40">
         <v>10</v>
       </c>
-      <c r="C11" s="121" t="s">
-        <v>25</v>
+      <c r="C11" s="172" t="s">
+        <v>24</v>
       </c>
-      <c r="D11" s="121"/>
-      <c r="E11" s="121" t="s">
-        <v>73</v>
+      <c r="D11" s="172"/>
+      <c r="E11" s="172" t="s">
+        <v>72</v>
       </c>
-      <c r="F11" s="121"/>
+      <c r="F11" s="172"/>
       <c r="G11" s="41"/>
       <c r="H11" s="41"/>
       <c r="I11" s="42"/>
@@ -29062,26 +29063,26 @@
         <v>40000000</v>
       </c>
       <c r="K11" s="65"/>
-      <c r="L11" s="142"/>
-      <c r="M11" s="143"/>
-      <c r="N11" s="143"/>
-      <c r="O11" s="143"/>
-      <c r="P11" s="143"/>
-      <c r="Q11" s="143"/>
+      <c r="L11" s="164"/>
+      <c r="M11" s="165"/>
+      <c r="N11" s="165"/>
+      <c r="O11" s="165"/>
+      <c r="P11" s="165"/>
+      <c r="Q11" s="165"/>
     </row>
     <row r="12" spans="1:17" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="70"/>
       <c r="B12" s="44">
         <v>11</v>
       </c>
-      <c r="C12" s="126" t="s">
+      <c r="C12" s="173" t="s">
+        <v>73</v>
+      </c>
+      <c r="D12" s="173"/>
+      <c r="E12" s="173" t="s">
         <v>74</v>
       </c>
-      <c r="D12" s="126"/>
-      <c r="E12" s="126" t="s">
-        <v>75</v>
-      </c>
-      <c r="F12" s="126"/>
+      <c r="F12" s="173"/>
       <c r="G12" s="45"/>
       <c r="H12" s="45"/>
       <c r="I12" s="46"/>
@@ -29090,33 +29091,33 @@
         <v>30000000</v>
       </c>
       <c r="K12" s="65"/>
-      <c r="L12" s="128" t="s">
-        <v>76</v>
+      <c r="L12" s="146" t="s">
+        <v>75</v>
       </c>
-      <c r="M12" s="129"/>
-      <c r="N12" s="129"/>
-      <c r="O12" s="129"/>
-      <c r="P12" s="130">
+      <c r="M12" s="147"/>
+      <c r="N12" s="147"/>
+      <c r="O12" s="147"/>
+      <c r="P12" s="150">
         <f>ABS(($J$38+$J$39)/$J$37)</f>
         <v>9.4070578696390211E-2</v>
       </c>
-      <c r="Q12" s="130"/>
+      <c r="Q12" s="150"/>
     </row>
     <row r="13" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="70"/>
       <c r="B13" s="18">
         <v>11.01</v>
       </c>
-      <c r="C13" s="125" t="s">
+      <c r="C13" s="174" t="s">
+        <v>76</v>
+      </c>
+      <c r="D13" s="174"/>
+      <c r="E13" s="175" t="s">
         <v>77</v>
       </c>
-      <c r="D13" s="125"/>
-      <c r="E13" s="127" t="s">
+      <c r="F13" s="175"/>
+      <c r="G13" s="14" t="s">
         <v>78</v>
-      </c>
-      <c r="F13" s="127"/>
-      <c r="G13" s="14" t="s">
-        <v>79</v>
       </c>
       <c r="H13" s="14">
         <v>1</v>
@@ -29141,16 +29142,16 @@
       <c r="B14" s="18">
         <v>11.02</v>
       </c>
-      <c r="C14" s="125" t="s">
-        <v>80</v>
+      <c r="C14" s="174" t="s">
+        <v>79</v>
       </c>
-      <c r="D14" s="125"/>
-      <c r="E14" s="127" t="s">
+      <c r="D14" s="174"/>
+      <c r="E14" s="175" t="s">
+        <v>77</v>
+      </c>
+      <c r="F14" s="175"/>
+      <c r="G14" s="14" t="s">
         <v>78</v>
-      </c>
-      <c r="F14" s="127"/>
-      <c r="G14" s="14" t="s">
-        <v>79</v>
       </c>
       <c r="H14" s="14">
         <v>1</v>
@@ -29163,28 +29164,28 @@
         <v>10000000</v>
       </c>
       <c r="K14" s="65"/>
-      <c r="L14" s="131" t="s">
-        <v>81</v>
+      <c r="L14" s="148" t="s">
+        <v>80</v>
       </c>
-      <c r="M14" s="132"/>
-      <c r="N14" s="132"/>
-      <c r="O14" s="132"/>
-      <c r="P14" s="132"/>
-      <c r="Q14" s="132"/>
+      <c r="M14" s="149"/>
+      <c r="N14" s="149"/>
+      <c r="O14" s="149"/>
+      <c r="P14" s="149"/>
+      <c r="Q14" s="149"/>
     </row>
     <row r="15" spans="1:17" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="70"/>
       <c r="B15" s="44">
         <v>12</v>
       </c>
-      <c r="C15" s="126" t="s">
-        <v>82</v>
+      <c r="C15" s="173" t="s">
+        <v>81</v>
       </c>
-      <c r="D15" s="126"/>
-      <c r="E15" s="126" t="s">
-        <v>75</v>
+      <c r="D15" s="173"/>
+      <c r="E15" s="173" t="s">
+        <v>74</v>
       </c>
-      <c r="F15" s="126"/>
+      <c r="F15" s="173"/>
       <c r="G15" s="45"/>
       <c r="H15" s="45"/>
       <c r="I15" s="46"/>
@@ -29205,16 +29206,16 @@
       <c r="B16" s="18">
         <v>12.01</v>
       </c>
-      <c r="C16" s="125" t="s">
-        <v>83</v>
+      <c r="C16" s="174" t="s">
+        <v>82</v>
       </c>
-      <c r="D16" s="125"/>
-      <c r="E16" s="127" t="s">
+      <c r="D16" s="174"/>
+      <c r="E16" s="175" t="s">
+        <v>77</v>
+      </c>
+      <c r="F16" s="175"/>
+      <c r="G16" s="14" t="s">
         <v>78</v>
-      </c>
-      <c r="F16" s="127"/>
-      <c r="G16" s="14" t="s">
-        <v>79</v>
       </c>
       <c r="H16" s="14">
         <v>1</v>
@@ -29227,13 +29228,13 @@
         <v>8000000</v>
       </c>
       <c r="K16" s="65"/>
-      <c r="L16" s="133" t="s">
-        <v>84</v>
+      <c r="L16" s="145" t="s">
+        <v>83</v>
       </c>
-      <c r="M16" s="134"/>
-      <c r="N16" s="134"/>
-      <c r="O16" s="134"/>
-      <c r="P16" s="134"/>
+      <c r="M16" s="144"/>
+      <c r="N16" s="144"/>
+      <c r="O16" s="144"/>
+      <c r="P16" s="144"/>
       <c r="Q16" s="64">
         <f>$J$11/$J$33</f>
         <v>0.40712468193384221</v>
@@ -29244,16 +29245,16 @@
       <c r="B17" s="18">
         <v>12.02</v>
       </c>
-      <c r="C17" s="125" t="s">
-        <v>85</v>
+      <c r="C17" s="174" t="s">
+        <v>84</v>
       </c>
-      <c r="D17" s="125"/>
-      <c r="E17" s="127" t="s">
+      <c r="D17" s="174"/>
+      <c r="E17" s="175" t="s">
+        <v>77</v>
+      </c>
+      <c r="F17" s="175"/>
+      <c r="G17" s="14" t="s">
         <v>78</v>
-      </c>
-      <c r="F17" s="127"/>
-      <c r="G17" s="14" t="s">
-        <v>79</v>
       </c>
       <c r="H17" s="14">
         <v>1</v>
@@ -29278,14 +29279,14 @@
       <c r="B18" s="40">
         <v>20</v>
       </c>
-      <c r="C18" s="121" t="s">
-        <v>27</v>
+      <c r="C18" s="172" t="s">
+        <v>26</v>
       </c>
-      <c r="D18" s="121"/>
-      <c r="E18" s="121" t="s">
-        <v>86</v>
+      <c r="D18" s="172"/>
+      <c r="E18" s="172" t="s">
+        <v>85</v>
       </c>
-      <c r="F18" s="121"/>
+      <c r="F18" s="172"/>
       <c r="G18" s="41"/>
       <c r="H18" s="41"/>
       <c r="I18" s="42"/>
@@ -29306,16 +29307,16 @@
       <c r="B19" s="18">
         <v>20.010000000000002</v>
       </c>
-      <c r="C19" s="122" t="s">
+      <c r="C19" s="176" t="s">
+        <v>86</v>
+      </c>
+      <c r="D19" s="176"/>
+      <c r="E19" s="176" t="s">
         <v>87</v>
       </c>
-      <c r="D19" s="122"/>
-      <c r="E19" s="122" t="s">
+      <c r="F19" s="176"/>
+      <c r="G19" s="14" t="s">
         <v>88</v>
-      </c>
-      <c r="F19" s="122"/>
-      <c r="G19" s="14" t="s">
-        <v>89</v>
       </c>
       <c r="H19" s="14">
         <v>20</v>
@@ -29329,13 +29330,13 @@
         <v>8000000</v>
       </c>
       <c r="K19" s="65"/>
-      <c r="L19" s="133" t="s">
-        <v>90</v>
+      <c r="L19" s="145" t="s">
+        <v>89</v>
       </c>
-      <c r="M19" s="134"/>
-      <c r="N19" s="134"/>
-      <c r="O19" s="134"/>
-      <c r="P19" s="134"/>
+      <c r="M19" s="144"/>
+      <c r="N19" s="144"/>
+      <c r="O19" s="144"/>
+      <c r="P19" s="144"/>
       <c r="Q19" s="64">
         <f>SUM($J$18,$J$21,$J$24,$J$27)/$J$33</f>
         <v>0.52162849872773542</v>
@@ -29346,16 +29347,16 @@
       <c r="B20" s="18">
         <v>20.02</v>
       </c>
-      <c r="C20" s="122" t="s">
+      <c r="C20" s="176" t="s">
+        <v>90</v>
+      </c>
+      <c r="D20" s="176"/>
+      <c r="E20" s="176" t="s">
         <v>91</v>
       </c>
-      <c r="D20" s="122"/>
-      <c r="E20" s="122" t="s">
-        <v>92</v>
-      </c>
-      <c r="F20" s="122"/>
+      <c r="F20" s="176"/>
       <c r="G20" s="14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H20" s="14">
         <v>5</v>
@@ -29381,14 +29382,14 @@
       <c r="B21" s="40">
         <v>30</v>
       </c>
-      <c r="C21" s="121" t="s">
-        <v>29</v>
+      <c r="C21" s="172" t="s">
+        <v>28</v>
       </c>
-      <c r="D21" s="121"/>
-      <c r="E21" s="121" t="s">
-        <v>86</v>
+      <c r="D21" s="172"/>
+      <c r="E21" s="172" t="s">
+        <v>85</v>
       </c>
-      <c r="F21" s="121"/>
+      <c r="F21" s="172"/>
       <c r="G21" s="41"/>
       <c r="H21" s="41"/>
       <c r="I21" s="42"/>
@@ -29409,16 +29410,16 @@
       <c r="B22" s="18">
         <v>30.01</v>
       </c>
-      <c r="C22" s="122" t="s">
-        <v>93</v>
+      <c r="C22" s="176" t="s">
+        <v>92</v>
       </c>
-      <c r="D22" s="122"/>
-      <c r="E22" s="122" t="s">
+      <c r="D22" s="176"/>
+      <c r="E22" s="176" t="s">
+        <v>87</v>
+      </c>
+      <c r="F22" s="176"/>
+      <c r="G22" s="14" t="s">
         <v>88</v>
-      </c>
-      <c r="F22" s="122"/>
-      <c r="G22" s="14" t="s">
-        <v>89</v>
       </c>
       <c r="H22" s="14">
         <v>30</v>
@@ -29432,13 +29433,13 @@
         <v>12000000</v>
       </c>
       <c r="K22" s="65"/>
-      <c r="L22" s="133" t="s">
-        <v>94</v>
+      <c r="L22" s="145" t="s">
+        <v>93</v>
       </c>
-      <c r="M22" s="134"/>
-      <c r="N22" s="134"/>
-      <c r="O22" s="134"/>
-      <c r="P22" s="134"/>
+      <c r="M22" s="144"/>
+      <c r="N22" s="144"/>
+      <c r="O22" s="144"/>
+      <c r="P22" s="144"/>
       <c r="Q22" s="64">
         <f>$J$29/$J$33</f>
         <v>7.124681933842239E-2</v>
@@ -29449,16 +29450,16 @@
       <c r="B23" s="18">
         <v>30.02</v>
       </c>
-      <c r="C23" s="122" t="s">
-        <v>95</v>
+      <c r="C23" s="176" t="s">
+        <v>94</v>
       </c>
-      <c r="D23" s="122"/>
-      <c r="E23" s="122" t="s">
-        <v>92</v>
+      <c r="D23" s="176"/>
+      <c r="E23" s="176" t="s">
+        <v>91</v>
       </c>
-      <c r="F23" s="122"/>
+      <c r="F23" s="176"/>
       <c r="G23" s="14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H23" s="14">
         <v>10</v>
@@ -29484,14 +29485,14 @@
       <c r="B24" s="40">
         <v>40</v>
       </c>
-      <c r="C24" s="121" t="s">
-        <v>31</v>
+      <c r="C24" s="172" t="s">
+        <v>30</v>
       </c>
-      <c r="D24" s="121"/>
-      <c r="E24" s="121" t="s">
-        <v>86</v>
+      <c r="D24" s="172"/>
+      <c r="E24" s="172" t="s">
+        <v>85</v>
       </c>
-      <c r="F24" s="121"/>
+      <c r="F24" s="172"/>
       <c r="G24" s="41"/>
       <c r="H24" s="41"/>
       <c r="I24" s="42"/>
@@ -29500,31 +29501,31 @@
         <v>16500000</v>
       </c>
       <c r="K24" s="65"/>
-      <c r="L24" s="128" t="str">
+      <c r="L24" s="146" t="str">
         <f>"직접비 "&amp;TEXT($J$33,"#,##0")&amp;"원 기준"</f>
         <v>직접비 98,250,000원 기준</v>
       </c>
-      <c r="M24" s="129"/>
-      <c r="N24" s="129"/>
-      <c r="O24" s="129"/>
-      <c r="P24" s="129"/>
-      <c r="Q24" s="129"/>
+      <c r="M24" s="147"/>
+      <c r="N24" s="147"/>
+      <c r="O24" s="147"/>
+      <c r="P24" s="147"/>
+      <c r="Q24" s="147"/>
     </row>
     <row r="25" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="70"/>
       <c r="B25" s="18">
         <v>40.01</v>
       </c>
-      <c r="C25" s="122" t="s">
-        <v>96</v>
+      <c r="C25" s="176" t="s">
+        <v>95</v>
       </c>
-      <c r="D25" s="122"/>
-      <c r="E25" s="122" t="s">
+      <c r="D25" s="176"/>
+      <c r="E25" s="176" t="s">
+        <v>87</v>
+      </c>
+      <c r="F25" s="176"/>
+      <c r="G25" s="14" t="s">
         <v>88</v>
-      </c>
-      <c r="F25" s="122"/>
-      <c r="G25" s="14" t="s">
-        <v>89</v>
       </c>
       <c r="H25" s="14">
         <v>30</v>
@@ -29550,16 +29551,16 @@
       <c r="B26" s="18">
         <v>40.020000000000003</v>
       </c>
-      <c r="C26" s="122" t="s">
-        <v>97</v>
+      <c r="C26" s="176" t="s">
+        <v>96</v>
       </c>
-      <c r="D26" s="122"/>
-      <c r="E26" s="122" t="s">
-        <v>92</v>
+      <c r="D26" s="176"/>
+      <c r="E26" s="176" t="s">
+        <v>91</v>
       </c>
-      <c r="F26" s="122"/>
+      <c r="F26" s="176"/>
       <c r="G26" s="14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H26" s="14">
         <v>10</v>
@@ -29585,14 +29586,14 @@
       <c r="B27" s="40">
         <v>50</v>
       </c>
-      <c r="C27" s="121" t="s">
-        <v>33</v>
+      <c r="C27" s="172" t="s">
+        <v>32</v>
       </c>
-      <c r="D27" s="121"/>
-      <c r="E27" s="121" t="s">
-        <v>86</v>
+      <c r="D27" s="172"/>
+      <c r="E27" s="172" t="s">
+        <v>85</v>
       </c>
-      <c r="F27" s="121"/>
+      <c r="F27" s="172"/>
       <c r="G27" s="41"/>
       <c r="H27" s="41"/>
       <c r="I27" s="42"/>
@@ -29601,30 +29602,30 @@
         <v>8000000</v>
       </c>
       <c r="K27" s="65"/>
-      <c r="L27" s="131" t="s">
-        <v>98</v>
+      <c r="L27" s="148" t="s">
+        <v>97</v>
       </c>
-      <c r="M27" s="132"/>
-      <c r="N27" s="132"/>
-      <c r="O27" s="132"/>
-      <c r="P27" s="132"/>
-      <c r="Q27" s="132"/>
+      <c r="M27" s="149"/>
+      <c r="N27" s="149"/>
+      <c r="O27" s="149"/>
+      <c r="P27" s="149"/>
+      <c r="Q27" s="149"/>
     </row>
     <row r="28" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="70"/>
       <c r="B28" s="18">
         <v>50.01</v>
       </c>
-      <c r="C28" s="122" t="s">
-        <v>99</v>
+      <c r="C28" s="176" t="s">
+        <v>98</v>
       </c>
-      <c r="D28" s="122"/>
-      <c r="E28" s="122" t="s">
+      <c r="D28" s="176"/>
+      <c r="E28" s="176" t="s">
+        <v>87</v>
+      </c>
+      <c r="F28" s="176"/>
+      <c r="G28" s="14" t="s">
         <v>88</v>
-      </c>
-      <c r="F28" s="122"/>
-      <c r="G28" s="14" t="s">
-        <v>89</v>
       </c>
       <c r="H28" s="14">
         <v>20</v>
@@ -29650,14 +29651,14 @@
       <c r="B29" s="40">
         <v>60</v>
       </c>
-      <c r="C29" s="121" t="s">
-        <v>35</v>
+      <c r="C29" s="172" t="s">
+        <v>34</v>
       </c>
-      <c r="D29" s="121"/>
-      <c r="E29" s="121" t="s">
-        <v>100</v>
+      <c r="D29" s="172"/>
+      <c r="E29" s="172" t="s">
+        <v>99</v>
       </c>
-      <c r="F29" s="121"/>
+      <c r="F29" s="172"/>
       <c r="G29" s="41"/>
       <c r="H29" s="41"/>
       <c r="I29" s="42"/>
@@ -29666,33 +29667,33 @@
         <v>7000000</v>
       </c>
       <c r="K29" s="65"/>
-      <c r="L29" s="128" t="s">
-        <v>101</v>
+      <c r="L29" s="146" t="s">
+        <v>100</v>
       </c>
-      <c r="M29" s="129"/>
-      <c r="N29" s="129"/>
-      <c r="O29" s="129"/>
-      <c r="P29" s="130">
+      <c r="M29" s="147"/>
+      <c r="N29" s="147"/>
+      <c r="O29" s="147"/>
+      <c r="P29" s="150">
         <f>$J$18/SUM($J$18,$J$21,$J$24,$J$27)</f>
         <v>0.2</v>
       </c>
-      <c r="Q29" s="130"/>
+      <c r="Q29" s="150"/>
     </row>
     <row r="30" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="70"/>
       <c r="B30" s="19">
         <v>60.01</v>
       </c>
-      <c r="C30" s="124" t="s">
+      <c r="C30" s="178" t="s">
+        <v>101</v>
+      </c>
+      <c r="D30" s="178"/>
+      <c r="E30" s="178" t="s">
         <v>102</v>
       </c>
-      <c r="D30" s="124"/>
-      <c r="E30" s="124" t="s">
-        <v>103</v>
-      </c>
-      <c r="F30" s="124"/>
+      <c r="F30" s="178"/>
       <c r="G30" s="11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H30" s="11">
         <v>1</v>
@@ -29705,33 +29706,33 @@
         <v>3000000</v>
       </c>
       <c r="K30" s="65"/>
-      <c r="L30" s="150" t="s">
-        <v>104</v>
+      <c r="L30" s="151" t="s">
+        <v>103</v>
       </c>
-      <c r="M30" s="151"/>
-      <c r="N30" s="151"/>
-      <c r="O30" s="151"/>
-      <c r="P30" s="152">
+      <c r="M30" s="152"/>
+      <c r="N30" s="152"/>
+      <c r="O30" s="152"/>
+      <c r="P30" s="153">
         <f>$J$21/SUM($J$18,$J$21,$J$24,$J$27)</f>
         <v>0.32195121951219513</v>
       </c>
-      <c r="Q30" s="152"/>
+      <c r="Q30" s="153"/>
     </row>
     <row r="31" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="70"/>
       <c r="B31" s="18">
         <v>60.02</v>
       </c>
-      <c r="C31" s="125" t="s">
-        <v>105</v>
+      <c r="C31" s="174" t="s">
+        <v>104</v>
       </c>
-      <c r="D31" s="125"/>
-      <c r="E31" s="125" t="s">
-        <v>103</v>
+      <c r="D31" s="174"/>
+      <c r="E31" s="174" t="s">
+        <v>102</v>
       </c>
-      <c r="F31" s="125"/>
+      <c r="F31" s="174"/>
       <c r="G31" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H31" s="14">
         <v>1</v>
@@ -29744,33 +29745,33 @@
         <v>2000000</v>
       </c>
       <c r="K31" s="65"/>
-      <c r="L31" s="150" t="s">
-        <v>106</v>
+      <c r="L31" s="151" t="s">
+        <v>105</v>
       </c>
-      <c r="M31" s="151"/>
-      <c r="N31" s="151"/>
-      <c r="O31" s="151"/>
-      <c r="P31" s="152">
+      <c r="M31" s="152"/>
+      <c r="N31" s="152"/>
+      <c r="O31" s="152"/>
+      <c r="P31" s="153">
         <f>$J$24/SUM($J$18,$J$21,$J$24,$J$27)</f>
         <v>0.32195121951219513</v>
       </c>
-      <c r="Q31" s="152"/>
+      <c r="Q31" s="153"/>
     </row>
     <row r="32" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="70"/>
       <c r="B32" s="18">
         <v>60.03</v>
       </c>
-      <c r="C32" s="125" t="s">
-        <v>107</v>
+      <c r="C32" s="174" t="s">
+        <v>106</v>
       </c>
-      <c r="D32" s="125"/>
-      <c r="E32" s="125" t="s">
-        <v>103</v>
+      <c r="D32" s="174"/>
+      <c r="E32" s="174" t="s">
+        <v>102</v>
       </c>
-      <c r="F32" s="125"/>
+      <c r="F32" s="174"/>
       <c r="G32" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H32" s="14">
         <v>1</v>
@@ -29783,29 +29784,29 @@
         <v>2000000</v>
       </c>
       <c r="K32" s="65"/>
-      <c r="L32" s="153" t="s">
-        <v>108</v>
+      <c r="L32" s="154" t="s">
+        <v>107</v>
       </c>
-      <c r="M32" s="154"/>
-      <c r="N32" s="154"/>
-      <c r="O32" s="154"/>
-      <c r="P32" s="155">
+      <c r="M32" s="155"/>
+      <c r="N32" s="155"/>
+      <c r="O32" s="155"/>
+      <c r="P32" s="156">
         <f>$J$27/SUM($J$18,$J$21,$J$24,$J$27)</f>
         <v>0.15609756097560976</v>
       </c>
-      <c r="Q32" s="155"/>
+      <c r="Q32" s="156"/>
     </row>
     <row r="33" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="70"/>
       <c r="B33" s="48" t="s">
+        <v>108</v>
+      </c>
+      <c r="C33" s="179" t="s">
         <v>109</v>
       </c>
-      <c r="C33" s="120" t="s">
-        <v>110</v>
-      </c>
-      <c r="D33" s="120"/>
-      <c r="E33" s="120"/>
-      <c r="F33" s="120"/>
+      <c r="D33" s="179"/>
+      <c r="E33" s="179"/>
+      <c r="F33" s="179"/>
       <c r="G33" s="49"/>
       <c r="H33" s="49"/>
       <c r="I33" s="50"/>
@@ -29826,14 +29827,14 @@
       <c r="B34" s="40">
         <v>70</v>
       </c>
-      <c r="C34" s="121" t="s">
-        <v>37</v>
+      <c r="C34" s="172" t="s">
+        <v>36</v>
       </c>
-      <c r="D34" s="121"/>
-      <c r="E34" s="121" t="s">
-        <v>111</v>
+      <c r="D34" s="172"/>
+      <c r="E34" s="172" t="s">
+        <v>110</v>
       </c>
-      <c r="F34" s="121"/>
+      <c r="F34" s="172"/>
       <c r="G34" s="41"/>
       <c r="H34" s="41"/>
       <c r="I34" s="42"/>
@@ -29854,16 +29855,16 @@
       <c r="B35" s="15">
         <v>70.010000000000005</v>
       </c>
-      <c r="C35" s="122" t="s">
+      <c r="C35" s="176" t="s">
+        <v>111</v>
+      </c>
+      <c r="D35" s="176"/>
+      <c r="E35" s="176" t="s">
         <v>112</v>
       </c>
-      <c r="D35" s="122"/>
-      <c r="E35" s="122" t="s">
+      <c r="F35" s="176"/>
+      <c r="G35" s="14" t="s">
         <v>113</v>
-      </c>
-      <c r="F35" s="122"/>
-      <c r="G35" s="14" t="s">
-        <v>114</v>
       </c>
       <c r="H35" s="20">
         <v>0.05</v>
@@ -29874,30 +29875,30 @@
         <v>4912500</v>
       </c>
       <c r="K35" s="65"/>
-      <c r="L35" s="128" t="s">
-        <v>115</v>
+      <c r="L35" s="146" t="s">
+        <v>114</v>
       </c>
-      <c r="M35" s="129"/>
-      <c r="N35" s="129"/>
-      <c r="O35" s="129"/>
-      <c r="P35" s="129"/>
-      <c r="Q35" s="129"/>
+      <c r="M35" s="147"/>
+      <c r="N35" s="147"/>
+      <c r="O35" s="147"/>
+      <c r="P35" s="147"/>
+      <c r="Q35" s="147"/>
     </row>
     <row r="36" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="70"/>
       <c r="B36" s="15">
         <v>70.02</v>
       </c>
-      <c r="C36" s="122" t="s">
+      <c r="C36" s="176" t="s">
+        <v>115</v>
+      </c>
+      <c r="D36" s="176"/>
+      <c r="E36" s="176" t="s">
         <v>116</v>
       </c>
-      <c r="D36" s="122"/>
-      <c r="E36" s="122" t="s">
-        <v>117</v>
-      </c>
-      <c r="F36" s="122"/>
+      <c r="F36" s="176"/>
       <c r="G36" s="14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H36" s="20">
         <v>7.0000000000000007E-2</v>
@@ -29908,27 +29909,27 @@
         <v>7221375</v>
       </c>
       <c r="K36" s="65"/>
-      <c r="L36" s="128" t="str">
+      <c r="L36" s="146" t="str">
         <f>"하드웨어·인건비 비중  "&amp;TEXT(($J$11+SUM($J$18,$J$21,$J$24,$J$27))/$J$33,"0.0%")</f>
         <v>하드웨어·인건비 비중  92.9%</v>
       </c>
-      <c r="M36" s="129"/>
-      <c r="N36" s="129"/>
-      <c r="O36" s="129"/>
-      <c r="P36" s="129"/>
-      <c r="Q36" s="129"/>
+      <c r="M36" s="147"/>
+      <c r="N36" s="147"/>
+      <c r="O36" s="147"/>
+      <c r="P36" s="147"/>
+      <c r="Q36" s="147"/>
     </row>
     <row r="37" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="70"/>
       <c r="B37" s="52" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
-      <c r="C37" s="123" t="s">
-        <v>65</v>
+      <c r="C37" s="180" t="s">
+        <v>64</v>
       </c>
-      <c r="D37" s="123"/>
-      <c r="E37" s="123"/>
-      <c r="F37" s="123"/>
+      <c r="D37" s="180"/>
+      <c r="E37" s="180"/>
+      <c r="F37" s="180"/>
       <c r="G37" s="53"/>
       <c r="H37" s="53"/>
       <c r="I37" s="54"/>
@@ -29937,26 +29938,26 @@
         <v>110383875</v>
       </c>
       <c r="K37" s="65"/>
-      <c r="L37" s="128"/>
-      <c r="M37" s="129"/>
-      <c r="N37" s="129"/>
-      <c r="O37" s="129"/>
-      <c r="P37" s="129"/>
-      <c r="Q37" s="129"/>
+      <c r="L37" s="146"/>
+      <c r="M37" s="147"/>
+      <c r="N37" s="147"/>
+      <c r="O37" s="147"/>
+      <c r="P37" s="147"/>
+      <c r="Q37" s="147"/>
     </row>
     <row r="38" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="70"/>
       <c r="B38" s="58" t="s">
+        <v>38</v>
+      </c>
+      <c r="C38" s="177" t="s">
         <v>39</v>
       </c>
-      <c r="C38" s="119" t="s">
-        <v>40</v>
+      <c r="D38" s="177"/>
+      <c r="E38" s="177" t="s">
+        <v>118</v>
       </c>
-      <c r="D38" s="119"/>
-      <c r="E38" s="119" t="s">
-        <v>119</v>
-      </c>
-      <c r="F38" s="119"/>
+      <c r="F38" s="177"/>
       <c r="G38" s="56"/>
       <c r="H38" s="56"/>
       <c r="I38" s="57"/>
@@ -29964,29 +29965,29 @@
         <v>-875</v>
       </c>
       <c r="K38" s="65"/>
-      <c r="L38" s="128" t="str">
+      <c r="L38" s="146" t="str">
         <f>"직접비  "&amp;TEXT($J$33/$J$37,"0.0%")&amp;"  |  관리·이윤  "&amp;TEXT($J$34/$J$37,"0.0%")</f>
         <v>직접비  89.0%  |  관리·이윤  11.0%</v>
       </c>
-      <c r="M38" s="129"/>
-      <c r="N38" s="129"/>
-      <c r="O38" s="129"/>
-      <c r="P38" s="129"/>
-      <c r="Q38" s="129"/>
+      <c r="M38" s="147"/>
+      <c r="N38" s="147"/>
+      <c r="O38" s="147"/>
+      <c r="P38" s="147"/>
+      <c r="Q38" s="147"/>
     </row>
     <row r="39" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="70"/>
       <c r="B39" s="58" t="s">
+        <v>41</v>
+      </c>
+      <c r="C39" s="177" t="s">
         <v>42</v>
       </c>
-      <c r="C39" s="119" t="s">
-        <v>43</v>
+      <c r="D39" s="177"/>
+      <c r="E39" s="177" t="s">
+        <v>119</v>
       </c>
-      <c r="D39" s="119"/>
-      <c r="E39" s="119" t="s">
-        <v>120</v>
-      </c>
-      <c r="F39" s="119"/>
+      <c r="F39" s="177"/>
       <c r="G39" s="56"/>
       <c r="H39" s="56"/>
       <c r="I39" s="57"/>
@@ -30003,47 +30004,47 @@
     </row>
     <row r="40" spans="1:17" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="70"/>
-      <c r="B40" s="212" t="s">
+      <c r="B40" s="88" t="s">
+        <v>120</v>
+      </c>
+      <c r="C40" s="188" t="s">
         <v>121</v>
       </c>
-      <c r="C40" s="213" t="s">
-        <v>122</v>
-      </c>
-      <c r="D40" s="213"/>
-      <c r="E40" s="213"/>
-      <c r="F40" s="213"/>
-      <c r="G40" s="214"/>
-      <c r="H40" s="214"/>
-      <c r="I40" s="215"/>
-      <c r="J40" s="216">
+      <c r="D40" s="188"/>
+      <c r="E40" s="188"/>
+      <c r="F40" s="188"/>
+      <c r="G40" s="89"/>
+      <c r="H40" s="89"/>
+      <c r="I40" s="90"/>
+      <c r="J40" s="91">
         <f>SUM(J37:J39)</f>
         <v>100000000</v>
       </c>
       <c r="K40" s="65"/>
-      <c r="L40" s="128" t="s">
-        <v>123</v>
+      <c r="L40" s="146" t="s">
+        <v>122</v>
       </c>
-      <c r="M40" s="129"/>
-      <c r="N40" s="129"/>
-      <c r="O40" s="129"/>
-      <c r="P40" s="129"/>
-      <c r="Q40" s="129"/>
+      <c r="M40" s="147"/>
+      <c r="N40" s="147"/>
+      <c r="O40" s="147"/>
+      <c r="P40" s="147"/>
+      <c r="Q40" s="147"/>
     </row>
     <row r="41" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="70"/>
-      <c r="B41" s="207" t="s">
-        <v>124</v>
+      <c r="B41" s="84" t="s">
+        <v>123</v>
       </c>
-      <c r="C41" s="208" t="s">
-        <v>48</v>
+      <c r="C41" s="189" t="s">
+        <v>47</v>
       </c>
-      <c r="D41" s="208"/>
-      <c r="E41" s="208"/>
-      <c r="F41" s="208"/>
-      <c r="G41" s="209"/>
-      <c r="H41" s="209"/>
-      <c r="I41" s="210"/>
-      <c r="J41" s="211">
+      <c r="D41" s="189"/>
+      <c r="E41" s="189"/>
+      <c r="F41" s="189"/>
+      <c r="G41" s="85"/>
+      <c r="H41" s="85"/>
+      <c r="I41" s="86"/>
+      <c r="J41" s="87">
         <f>ROUND(J40*1.1,0)</f>
         <v>110000000</v>
       </c>
@@ -30076,17 +30077,17 @@
     </row>
     <row r="43" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="70"/>
-      <c r="B43" s="118" t="s">
-        <v>57</v>
+      <c r="B43" s="187" t="s">
+        <v>56</v>
       </c>
-      <c r="C43" s="118"/>
-      <c r="D43" s="118"/>
-      <c r="E43" s="118"/>
-      <c r="F43" s="118"/>
-      <c r="G43" s="118"/>
-      <c r="H43" s="118"/>
-      <c r="I43" s="118"/>
-      <c r="J43" s="118"/>
+      <c r="C43" s="187"/>
+      <c r="D43" s="187"/>
+      <c r="E43" s="187"/>
+      <c r="F43" s="187"/>
+      <c r="G43" s="187"/>
+      <c r="H43" s="187"/>
+      <c r="I43" s="187"/>
+      <c r="J43" s="187"/>
       <c r="K43" s="65"/>
       <c r="L43" s="9"/>
       <c r="M43" s="9"/>
@@ -30116,19 +30117,19 @@
     </row>
     <row r="45" spans="1:17" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="72"/>
-      <c r="B45" s="112" t="s">
+      <c r="B45" s="181" t="s">
+        <v>57</v>
+      </c>
+      <c r="C45" s="182"/>
+      <c r="D45" s="182"/>
+      <c r="E45" s="182"/>
+      <c r="F45" s="182"/>
+      <c r="G45" s="184" t="s">
         <v>58</v>
       </c>
-      <c r="C45" s="113"/>
-      <c r="D45" s="113"/>
-      <c r="E45" s="113"/>
-      <c r="F45" s="113"/>
-      <c r="G45" s="115" t="s">
-        <v>59</v>
-      </c>
-      <c r="H45" s="116"/>
-      <c r="I45" s="116"/>
-      <c r="J45" s="116"/>
+      <c r="H45" s="185"/>
+      <c r="I45" s="185"/>
+      <c r="J45" s="185"/>
       <c r="K45" s="73"/>
       <c r="L45" s="9"/>
       <c r="M45" s="9"/>
@@ -30139,15 +30140,15 @@
     </row>
     <row r="46" spans="1:17" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="74"/>
-      <c r="B46" s="114"/>
-      <c r="C46" s="114"/>
-      <c r="D46" s="114"/>
-      <c r="E46" s="114"/>
-      <c r="F46" s="114"/>
-      <c r="G46" s="117"/>
-      <c r="H46" s="117"/>
-      <c r="I46" s="117"/>
-      <c r="J46" s="117"/>
+      <c r="B46" s="183"/>
+      <c r="C46" s="183"/>
+      <c r="D46" s="183"/>
+      <c r="E46" s="183"/>
+      <c r="F46" s="183"/>
+      <c r="G46" s="186"/>
+      <c r="H46" s="186"/>
+      <c r="I46" s="186"/>
+      <c r="J46" s="186"/>
       <c r="K46" s="75"/>
       <c r="L46" s="9"/>
       <c r="M46" s="9"/>
@@ -30158,15 +30159,15 @@
     </row>
     <row r="47" spans="1:17" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="74"/>
-      <c r="B47" s="114"/>
-      <c r="C47" s="114"/>
-      <c r="D47" s="114"/>
-      <c r="E47" s="114"/>
-      <c r="F47" s="114"/>
-      <c r="G47" s="117"/>
-      <c r="H47" s="117"/>
-      <c r="I47" s="117"/>
-      <c r="J47" s="117"/>
+      <c r="B47" s="183"/>
+      <c r="C47" s="183"/>
+      <c r="D47" s="183"/>
+      <c r="E47" s="183"/>
+      <c r="F47" s="183"/>
+      <c r="G47" s="186"/>
+      <c r="H47" s="186"/>
+      <c r="I47" s="186"/>
+      <c r="J47" s="186"/>
       <c r="K47" s="75"/>
       <c r="L47" s="9"/>
       <c r="M47" s="9"/>
@@ -31851,75 +31852,15 @@
     </row>
   </sheetData>
   <mergeCells count="102">
-    <mergeCell ref="N19:P19"/>
-    <mergeCell ref="L22:M22"/>
-    <mergeCell ref="N22:P22"/>
-    <mergeCell ref="L24:Q24"/>
-    <mergeCell ref="L38:Q38"/>
-    <mergeCell ref="L27:Q27"/>
-    <mergeCell ref="L29:O29"/>
-    <mergeCell ref="P29:Q29"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="L40:Q40"/>
-    <mergeCell ref="L30:O30"/>
-    <mergeCell ref="P30:Q30"/>
-    <mergeCell ref="L31:O31"/>
-    <mergeCell ref="P31:Q31"/>
-    <mergeCell ref="L32:O32"/>
-    <mergeCell ref="P32:Q32"/>
-    <mergeCell ref="L35:Q35"/>
-    <mergeCell ref="L36:Q37"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="L5:Q5"/>
-    <mergeCell ref="L6:Q7"/>
-    <mergeCell ref="L8:N8"/>
-    <mergeCell ref="O8:Q8"/>
-    <mergeCell ref="L9:N11"/>
-    <mergeCell ref="O9:Q11"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="G5:J5"/>
-    <mergeCell ref="G6:J6"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="G8:J8"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="L12:O12"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="L14:Q14"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="L16:M16"/>
-    <mergeCell ref="N16:P16"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="B45:F47"/>
+    <mergeCell ref="G45:J47"/>
+    <mergeCell ref="B43:J43"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="E41:F41"/>
     <mergeCell ref="C38:D38"/>
     <mergeCell ref="E38:F38"/>
     <mergeCell ref="C27:D27"/>
@@ -31944,15 +31885,75 @@
     <mergeCell ref="E36:F36"/>
     <mergeCell ref="C37:D37"/>
     <mergeCell ref="E37:F37"/>
-    <mergeCell ref="B45:F47"/>
-    <mergeCell ref="G45:J47"/>
-    <mergeCell ref="B43:J43"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="L12:O12"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="L14:Q14"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="L16:M16"/>
+    <mergeCell ref="N16:P16"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="L5:Q5"/>
+    <mergeCell ref="L6:Q7"/>
+    <mergeCell ref="L8:N8"/>
+    <mergeCell ref="O8:Q8"/>
+    <mergeCell ref="L9:N11"/>
+    <mergeCell ref="O9:Q11"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="G5:J5"/>
+    <mergeCell ref="G6:J6"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="G8:J8"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="L40:Q40"/>
+    <mergeCell ref="L30:O30"/>
+    <mergeCell ref="P30:Q30"/>
+    <mergeCell ref="L31:O31"/>
+    <mergeCell ref="P31:Q31"/>
+    <mergeCell ref="L32:O32"/>
+    <mergeCell ref="P32:Q32"/>
+    <mergeCell ref="L35:Q35"/>
+    <mergeCell ref="L36:Q37"/>
+    <mergeCell ref="N19:P19"/>
+    <mergeCell ref="L22:M22"/>
+    <mergeCell ref="N22:P22"/>
+    <mergeCell ref="L24:Q24"/>
+    <mergeCell ref="L38:Q38"/>
+    <mergeCell ref="L27:Q27"/>
+    <mergeCell ref="L29:O29"/>
+    <mergeCell ref="P29:Q29"/>
+    <mergeCell ref="L19:M19"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
@@ -32001,36 +32002,36 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="8"/>
-      <c r="B3" s="156" t="s">
-        <v>125</v>
+      <c r="B3" s="190" t="s">
+        <v>124</v>
       </c>
-      <c r="C3" s="156"/>
-      <c r="D3" s="156"/>
-      <c r="E3" s="156"/>
-      <c r="F3" s="156"/>
-      <c r="G3" s="156"/>
+      <c r="C3" s="190"/>
+      <c r="D3" s="190"/>
+      <c r="E3" s="190"/>
+      <c r="F3" s="190"/>
+      <c r="G3" s="190"/>
       <c r="H3" s="8"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="8"/>
-      <c r="B4" s="156"/>
-      <c r="C4" s="156"/>
-      <c r="D4" s="156"/>
-      <c r="E4" s="156"/>
-      <c r="F4" s="156"/>
-      <c r="G4" s="156"/>
+      <c r="B4" s="190"/>
+      <c r="C4" s="190"/>
+      <c r="D4" s="190"/>
+      <c r="E4" s="190"/>
+      <c r="F4" s="190"/>
+      <c r="G4" s="190"/>
       <c r="H4" s="8"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="8"/>
-      <c r="B5" s="157" t="s">
-        <v>126</v>
+      <c r="B5" s="191" t="s">
+        <v>125</v>
       </c>
-      <c r="C5" s="157"/>
-      <c r="D5" s="157"/>
-      <c r="E5" s="157"/>
-      <c r="F5" s="157"/>
-      <c r="G5" s="157"/>
+      <c r="C5" s="191"/>
+      <c r="D5" s="191"/>
+      <c r="E5" s="191"/>
+      <c r="F5" s="191"/>
+      <c r="G5" s="191"/>
       <c r="H5" s="8"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -32046,22 +32047,22 @@
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="8"/>
       <c r="B7" s="22" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C7" s="22" t="s">
         <v>2</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E7" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="F7" s="22" t="s">
         <v>128</v>
       </c>
-      <c r="F7" s="22" t="s">
+      <c r="G7" s="22" t="s">
         <v>129</v>
-      </c>
-      <c r="G7" s="22" t="s">
-        <v>130</v>
       </c>
       <c r="H7" s="8"/>
     </row>
@@ -32078,29 +32079,29 @@
     <row r="9" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="8"/>
       <c r="B9" s="23" t="s">
+        <v>130</v>
+      </c>
+      <c r="C9" s="23" t="s">
         <v>131</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="D9" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="D9" s="23" t="s">
+      <c r="E9" s="23" t="s">
         <v>133</v>
       </c>
-      <c r="E9" s="23" t="s">
+      <c r="F9" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="F9" s="23" t="s">
+      <c r="G9" s="23" t="s">
         <v>135</v>
-      </c>
-      <c r="G9" s="23" t="s">
-        <v>136</v>
       </c>
       <c r="H9" s="8"/>
     </row>
     <row r="10" spans="1:8" ht="26.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8"/>
       <c r="B10" s="33" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C10" s="24">
         <v>35</v>
@@ -32109,20 +32110,20 @@
         <v>350000</v>
       </c>
       <c r="E10" s="26" t="s">
+        <v>137</v>
+      </c>
+      <c r="F10" s="26" t="s">
         <v>138</v>
       </c>
-      <c r="F10" s="26" t="s">
+      <c r="G10" s="26" t="s">
         <v>139</v>
-      </c>
-      <c r="G10" s="26" t="s">
-        <v>140</v>
       </c>
       <c r="H10" s="8"/>
     </row>
     <row r="11" spans="1:8" ht="26.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="8"/>
       <c r="B11" s="34" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C11" s="27">
         <v>40</v>
@@ -32131,20 +32132,20 @@
         <v>400000</v>
       </c>
       <c r="E11" s="29" t="s">
+        <v>141</v>
+      </c>
+      <c r="F11" s="29" t="s">
         <v>142</v>
       </c>
-      <c r="F11" s="29" t="s">
-        <v>143</v>
-      </c>
       <c r="G11" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H11" s="8"/>
     </row>
     <row r="12" spans="1:8" ht="26.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="8"/>
       <c r="B12" s="35" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C12" s="30">
         <v>45</v>
@@ -32153,13 +32154,13 @@
         <v>450000</v>
       </c>
       <c r="E12" s="32" t="s">
+        <v>144</v>
+      </c>
+      <c r="F12" s="32" t="s">
         <v>145</v>
       </c>
-      <c r="F12" s="32" t="s">
-        <v>146</v>
-      </c>
       <c r="G12" s="32" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H12" s="8"/>
     </row>
@@ -32185,34 +32186,34 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="8"/>
-      <c r="B15" s="158" t="s">
-        <v>147</v>
+      <c r="B15" s="192" t="s">
+        <v>146</v>
       </c>
-      <c r="C15" s="159"/>
-      <c r="D15" s="159"/>
-      <c r="E15" s="159"/>
-      <c r="F15" s="159"/>
-      <c r="G15" s="160"/>
+      <c r="C15" s="193"/>
+      <c r="D15" s="193"/>
+      <c r="E15" s="193"/>
+      <c r="F15" s="193"/>
+      <c r="G15" s="194"/>
       <c r="H15" s="8"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="8"/>
-      <c r="B16" s="161"/>
-      <c r="C16" s="162"/>
-      <c r="D16" s="162"/>
-      <c r="E16" s="162"/>
-      <c r="F16" s="162"/>
-      <c r="G16" s="163"/>
+      <c r="B16" s="195"/>
+      <c r="C16" s="196"/>
+      <c r="D16" s="196"/>
+      <c r="E16" s="196"/>
+      <c r="F16" s="196"/>
+      <c r="G16" s="197"/>
       <c r="H16" s="8"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="8"/>
-      <c r="B17" s="164"/>
-      <c r="C17" s="165"/>
-      <c r="D17" s="165"/>
-      <c r="E17" s="165"/>
-      <c r="F17" s="165"/>
-      <c r="G17" s="166"/>
+      <c r="B17" s="198"/>
+      <c r="C17" s="199"/>
+      <c r="D17" s="199"/>
+      <c r="E17" s="199"/>
+      <c r="F17" s="199"/>
+      <c r="G17" s="200"/>
       <c r="H17" s="8"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
@@ -32267,36 +32268,36 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="8"/>
-      <c r="B23" s="167" t="s">
+      <c r="B23" s="201" t="s">
+        <v>147</v>
+      </c>
+      <c r="C23" s="201"/>
+      <c r="D23" s="201"/>
+      <c r="E23" s="203" t="s">
         <v>148</v>
       </c>
-      <c r="C23" s="167"/>
-      <c r="D23" s="167"/>
-      <c r="E23" s="169" t="s">
-        <v>149</v>
-      </c>
-      <c r="F23" s="169"/>
-      <c r="G23" s="169"/>
+      <c r="F23" s="203"/>
+      <c r="G23" s="203"/>
       <c r="H23" s="8"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="8"/>
-      <c r="B24" s="168"/>
-      <c r="C24" s="168"/>
-      <c r="D24" s="168"/>
-      <c r="E24" s="170"/>
-      <c r="F24" s="170"/>
-      <c r="G24" s="170"/>
+      <c r="B24" s="202"/>
+      <c r="C24" s="202"/>
+      <c r="D24" s="202"/>
+      <c r="E24" s="204"/>
+      <c r="F24" s="204"/>
+      <c r="G24" s="204"/>
       <c r="H24" s="8"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="8"/>
-      <c r="B25" s="168"/>
-      <c r="C25" s="168"/>
-      <c r="D25" s="168"/>
-      <c r="E25" s="170"/>
-      <c r="F25" s="170"/>
-      <c r="G25" s="170"/>
+      <c r="B25" s="202"/>
+      <c r="C25" s="202"/>
+      <c r="D25" s="202"/>
+      <c r="E25" s="204"/>
+      <c r="F25" s="204"/>
+      <c r="G25" s="204"/>
       <c r="H25" s="8"/>
     </row>
   </sheetData>

</xml_diff>